<commit_message>
RM/SRD UC 식별자 변경, RTM SRD 기준 완성
</commit_message>
<xml_diff>
--- a/Document/요구사항추적표(RTM).xlsx
+++ b/Document/요구사항추적표(RTM).xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\82102\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rlaal\Documents\FalshTalk\Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCD68975-2266-413D-8713-3FBFC1B7F269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11FF53AE-17AF-4490-A9E5-05FE6193FB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2768" yWindow="420" windowWidth="17745" windowHeight="12727" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="원본" sheetId="4" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="204">
   <si>
     <t>번호</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -692,30 +692,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>사용자 조회 및 검색</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>1:1 채팅</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>그룹 채팅</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>지도 검색</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>파일 전송</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>AI 챗봇</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>BW-02</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -770,13 +746,84 @@
   <si>
     <t>BW-01, BW-09, BW-10</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AD-01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AD-02</t>
+  </si>
+  <si>
+    <t>AD-03</t>
+  </si>
+  <si>
+    <t>AD-04</t>
+  </si>
+  <si>
+    <t>AD-05</t>
+  </si>
+  <si>
+    <t>AD-06</t>
+  </si>
+  <si>
+    <t>AD-07</t>
+  </si>
+  <si>
+    <t>AD-08</t>
+  </si>
+  <si>
+    <t>AD-09</t>
+  </si>
+  <si>
+    <t>FR-01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FR-02</t>
+  </si>
+  <si>
+    <t>FR-03</t>
+  </si>
+  <si>
+    <t>FR-04</t>
+  </si>
+  <si>
+    <t>FR-05</t>
+  </si>
+  <si>
+    <t>FR-06</t>
+  </si>
+  <si>
+    <t>FR-07</t>
+  </si>
+  <si>
+    <t>FR-08</t>
+  </si>
+  <si>
+    <t>FR-09</t>
+  </si>
+  <si>
+    <t>FR-10</t>
+  </si>
+  <si>
+    <t>친구 찾기</t>
+  </si>
+  <si>
+    <t>플래시 채팅</t>
+  </si>
+  <si>
+    <t>대화방 생성</t>
+  </si>
+  <si>
+    <t xml:space="preserve">대화방 초대 </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -885,6 +932,14 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -918,7 +973,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="47">
     <border>
       <left/>
       <right/>
@@ -1381,36 +1436,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="medium">
         <color indexed="64"/>
@@ -1443,6 +1468,77 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1453,7 +1549,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="153">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1580,9 +1676,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1595,7 +1688,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1605,7 +1698,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1621,22 +1714,13 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1675,28 +1759,94 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1705,113 +1855,35 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="38" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1870,32 +1942,79 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="45" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2207,254 +2326,254 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AK42"/>
-  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="11.5" customWidth="1"/>
-    <col min="2" max="2" width="13.1875" customWidth="1"/>
-    <col min="3" max="3" width="24.6875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.1875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29.625" customWidth="1"/>
-    <col min="9" max="9" width="24.1875" customWidth="1"/>
-    <col min="10" max="10" width="20.1875" customWidth="1"/>
-    <col min="11" max="11" width="12.625" style="23" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="35.625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.1875" customWidth="1"/>
-    <col min="14" max="14" width="24.125" customWidth="1"/>
+    <col min="2" max="2" width="13.19921875" customWidth="1"/>
+    <col min="3" max="3" width="24.69921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.19921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.59765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.09765625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.19921875" customWidth="1"/>
+    <col min="10" max="10" width="20.19921875" customWidth="1"/>
+    <col min="11" max="11" width="12.59765625" style="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="35.59765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.19921875" customWidth="1"/>
+    <col min="14" max="14" width="24.09765625" customWidth="1"/>
     <col min="15" max="15" width="38" customWidth="1"/>
-    <col min="16" max="16" width="24.125" customWidth="1"/>
-    <col min="17" max="17" width="12.125" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="24.125" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="34.125" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="21.625" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="24.625" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="42.625" hidden="1" customWidth="1"/>
-    <col min="23" max="25" width="21.625" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="15.125" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="12.125" hidden="1" customWidth="1"/>
-    <col min="28" max="28" width="24.125" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="10.625" hidden="1" customWidth="1"/>
-    <col min="30" max="30" width="31.125" hidden="1" customWidth="1"/>
-    <col min="31" max="32" width="18.625" hidden="1" customWidth="1"/>
-    <col min="33" max="33" width="12.625" hidden="1" customWidth="1"/>
-    <col min="34" max="34" width="18.125" hidden="1" customWidth="1"/>
-    <col min="35" max="35" width="21.125" hidden="1" customWidth="1"/>
-    <col min="36" max="36" width="24.625" hidden="1" customWidth="1"/>
-    <col min="37" max="37" width="8.625" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="24.09765625" customWidth="1"/>
+    <col min="17" max="17" width="12.09765625" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="24.09765625" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="34.09765625" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="21.59765625" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="24.59765625" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="42.59765625" hidden="1" customWidth="1"/>
+    <col min="23" max="25" width="21.59765625" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="15.09765625" hidden="1" customWidth="1"/>
+    <col min="27" max="27" width="12.09765625" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="24.09765625" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="10.59765625" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="31.09765625" hidden="1" customWidth="1"/>
+    <col min="31" max="32" width="18.59765625" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="12.59765625" hidden="1" customWidth="1"/>
+    <col min="34" max="34" width="18.09765625" hidden="1" customWidth="1"/>
+    <col min="35" max="35" width="21.09765625" hidden="1" customWidth="1"/>
+    <col min="36" max="36" width="24.59765625" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="8.59765625" hidden="1" customWidth="1"/>
     <col min="38" max="38" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="16.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="118" t="s">
+    <row r="1" spans="1:37" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="149" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
-      <c r="AC1" s="119"/>
-      <c r="AD1" s="119"/>
-      <c r="AE1" s="110"/>
-      <c r="AF1" s="110"/>
+      <c r="B1" s="150"/>
+      <c r="C1" s="150"/>
+      <c r="D1" s="150"/>
+      <c r="E1" s="150"/>
+      <c r="F1" s="150"/>
+      <c r="G1" s="150"/>
+      <c r="H1" s="150"/>
+      <c r="I1" s="150"/>
+      <c r="J1" s="150"/>
+      <c r="K1" s="150"/>
+      <c r="L1" s="151"/>
+      <c r="M1" s="147"/>
+      <c r="N1" s="147"/>
+      <c r="O1" s="147"/>
+      <c r="P1" s="147"/>
+      <c r="Q1" s="147"/>
+      <c r="R1" s="147"/>
+      <c r="S1" s="147"/>
+      <c r="T1" s="147"/>
+      <c r="U1" s="147"/>
+      <c r="V1" s="147"/>
+      <c r="W1" s="147"/>
+      <c r="X1" s="147"/>
+      <c r="Y1" s="147"/>
+      <c r="Z1" s="147"/>
+      <c r="AA1" s="147"/>
+      <c r="AB1" s="147"/>
+      <c r="AC1" s="147"/>
+      <c r="AD1" s="147"/>
+      <c r="AE1" s="77"/>
+      <c r="AF1" s="77"/>
       <c r="AG1" s="19"/>
       <c r="AH1" s="19"/>
       <c r="AI1" s="19"/>
       <c r="AJ1" s="20"/>
       <c r="AK1" s="20"/>
     </row>
-    <row r="2" spans="1:37" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A2" s="120"/>
-      <c r="B2" s="121"/>
-      <c r="C2" s="121"/>
-      <c r="D2" s="121"/>
-      <c r="E2" s="121"/>
-      <c r="F2" s="121"/>
-      <c r="G2" s="121"/>
-      <c r="H2" s="121"/>
-      <c r="I2" s="121"/>
-      <c r="J2" s="121"/>
-      <c r="K2" s="121"/>
-      <c r="L2" s="121"/>
-      <c r="M2" s="121"/>
-      <c r="N2" s="121"/>
-      <c r="O2" s="121"/>
-      <c r="P2" s="121"/>
-      <c r="Q2" s="121"/>
-      <c r="R2" s="121"/>
-      <c r="S2" s="121"/>
-      <c r="T2" s="121"/>
-      <c r="U2" s="121"/>
-      <c r="V2" s="121"/>
-      <c r="W2" s="121"/>
-      <c r="X2" s="121"/>
-      <c r="Y2" s="121"/>
-      <c r="Z2" s="121"/>
-      <c r="AA2" s="121"/>
-      <c r="AB2" s="121"/>
-      <c r="AC2" s="121"/>
-      <c r="AD2" s="121"/>
-      <c r="AE2" s="111"/>
-      <c r="AF2" s="111"/>
+    <row r="2" spans="1:37" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="152"/>
+      <c r="B2" s="153"/>
+      <c r="C2" s="153"/>
+      <c r="D2" s="153"/>
+      <c r="E2" s="153"/>
+      <c r="F2" s="153"/>
+      <c r="G2" s="153"/>
+      <c r="H2" s="153"/>
+      <c r="I2" s="153"/>
+      <c r="J2" s="153"/>
+      <c r="K2" s="153"/>
+      <c r="L2" s="154"/>
+      <c r="M2" s="148"/>
+      <c r="N2" s="148"/>
+      <c r="O2" s="148"/>
+      <c r="P2" s="148"/>
+      <c r="Q2" s="148"/>
+      <c r="R2" s="148"/>
+      <c r="S2" s="148"/>
+      <c r="T2" s="148"/>
+      <c r="U2" s="148"/>
+      <c r="V2" s="148"/>
+      <c r="W2" s="148"/>
+      <c r="X2" s="148"/>
+      <c r="Y2" s="148"/>
+      <c r="Z2" s="148"/>
+      <c r="AA2" s="148"/>
+      <c r="AB2" s="148"/>
+      <c r="AC2" s="148"/>
+      <c r="AD2" s="148"/>
+      <c r="AE2" s="78"/>
+      <c r="AF2" s="78"/>
       <c r="AG2" s="21"/>
       <c r="AH2" s="21"/>
       <c r="AI2" s="21"/>
       <c r="AJ2" s="22"/>
       <c r="AK2" s="22"/>
     </row>
-    <row r="3" spans="1:37" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A3" s="83" t="s">
+    <row r="3" spans="1:37" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="90" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="83"/>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83" t="s">
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90" t="s">
         <v>112</v>
       </c>
-      <c r="G3" s="83"/>
-      <c r="H3" s="83"/>
-      <c r="I3" s="83"/>
-      <c r="J3" s="83"/>
-      <c r="K3" s="84" t="s">
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="145" t="s">
         <v>113</v>
       </c>
-      <c r="L3" s="84"/>
-      <c r="M3" s="84"/>
-      <c r="N3" s="84"/>
-      <c r="O3" s="84"/>
-      <c r="P3" s="84"/>
-      <c r="AJ3" s="49"/>
-    </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.6">
-      <c r="A4" s="83"/>
-      <c r="B4" s="83"/>
-      <c r="C4" s="83"/>
-      <c r="D4" s="83"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="83"/>
-      <c r="G4" s="83"/>
-      <c r="H4" s="83"/>
-      <c r="I4" s="83"/>
-      <c r="J4" s="83"/>
-      <c r="K4" s="123" t="s">
+      <c r="L3" s="146"/>
+      <c r="M3" s="144"/>
+      <c r="N3" s="144"/>
+      <c r="O3" s="144"/>
+      <c r="P3" s="144"/>
+      <c r="AJ3" s="48"/>
+    </row>
+    <row r="4" spans="1:37" x14ac:dyDescent="0.4">
+      <c r="A4" s="90"/>
+      <c r="B4" s="90"/>
+      <c r="C4" s="90"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="88" t="s">
         <v>80</v>
       </c>
-      <c r="L4" s="123"/>
-      <c r="M4" s="123" t="s">
+      <c r="L4" s="88"/>
+      <c r="M4" s="88" t="s">
         <v>79</v>
       </c>
-      <c r="N4" s="123"/>
-      <c r="O4" s="123"/>
-      <c r="P4" s="124"/>
-      <c r="Q4" s="116" t="s">
+      <c r="N4" s="88"/>
+      <c r="O4" s="88"/>
+      <c r="P4" s="89"/>
+      <c r="Q4" s="84" t="s">
         <v>79</v>
       </c>
-      <c r="R4" s="117"/>
-      <c r="S4" s="117"/>
-      <c r="T4" s="117"/>
-      <c r="U4" s="117"/>
-      <c r="V4" s="117"/>
-      <c r="W4" s="117"/>
-      <c r="X4" s="117"/>
-      <c r="Y4" s="117"/>
-      <c r="Z4" s="117"/>
-      <c r="AA4" s="117"/>
-      <c r="AB4" s="117"/>
-      <c r="AC4" s="114" t="s">
+      <c r="R4" s="85"/>
+      <c r="S4" s="85"/>
+      <c r="T4" s="85"/>
+      <c r="U4" s="85"/>
+      <c r="V4" s="85"/>
+      <c r="W4" s="85"/>
+      <c r="X4" s="85"/>
+      <c r="Y4" s="85"/>
+      <c r="Z4" s="85"/>
+      <c r="AA4" s="85"/>
+      <c r="AB4" s="85"/>
+      <c r="AC4" s="81" t="s">
         <v>93</v>
       </c>
-      <c r="AD4" s="114"/>
-      <c r="AE4" s="114"/>
-      <c r="AF4" s="114"/>
-      <c r="AG4" s="114"/>
-      <c r="AH4" s="114"/>
-      <c r="AI4" s="114"/>
-      <c r="AJ4" s="115"/>
-      <c r="AK4" s="106" t="s">
+      <c r="AD4" s="81"/>
+      <c r="AE4" s="81"/>
+      <c r="AF4" s="81"/>
+      <c r="AG4" s="81"/>
+      <c r="AH4" s="81"/>
+      <c r="AI4" s="81"/>
+      <c r="AJ4" s="82"/>
+      <c r="AK4" s="96" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:37" ht="16.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A5" s="83"/>
-      <c r="B5" s="83"/>
-      <c r="C5" s="83"/>
-      <c r="D5" s="83"/>
-      <c r="E5" s="83"/>
-      <c r="F5" s="91" t="s">
+    <row r="5" spans="1:37" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="90"/>
+      <c r="B5" s="90"/>
+      <c r="C5" s="90"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="90"/>
+      <c r="F5" s="83" t="s">
         <v>107</v>
       </c>
-      <c r="G5" s="112"/>
-      <c r="H5" s="112"/>
-      <c r="I5" s="112"/>
-      <c r="J5" s="112"/>
-      <c r="K5" s="112" t="s">
+      <c r="G5" s="79"/>
+      <c r="H5" s="79"/>
+      <c r="I5" s="79"/>
+      <c r="J5" s="79"/>
+      <c r="K5" s="79" t="s">
         <v>106</v>
       </c>
-      <c r="L5" s="112"/>
-      <c r="M5" s="122" t="s">
+      <c r="L5" s="79"/>
+      <c r="M5" s="86" t="s">
         <v>111</v>
       </c>
-      <c r="N5" s="90"/>
-      <c r="O5" s="90"/>
-      <c r="P5" s="91"/>
-      <c r="Q5" s="91" t="s">
+      <c r="N5" s="87"/>
+      <c r="O5" s="87"/>
+      <c r="P5" s="83"/>
+      <c r="Q5" s="83" t="s">
         <v>92</v>
       </c>
-      <c r="R5" s="112"/>
-      <c r="S5" s="112"/>
-      <c r="T5" s="112"/>
-      <c r="U5" s="112"/>
-      <c r="V5" s="112"/>
-      <c r="W5" s="112"/>
-      <c r="X5" s="112"/>
-      <c r="Y5" s="112"/>
-      <c r="Z5" s="112"/>
-      <c r="AA5" s="112"/>
-      <c r="AB5" s="112"/>
-      <c r="AC5" s="112" t="s">
+      <c r="R5" s="79"/>
+      <c r="S5" s="79"/>
+      <c r="T5" s="79"/>
+      <c r="U5" s="79"/>
+      <c r="V5" s="79"/>
+      <c r="W5" s="79"/>
+      <c r="X5" s="79"/>
+      <c r="Y5" s="79"/>
+      <c r="Z5" s="79"/>
+      <c r="AA5" s="79"/>
+      <c r="AB5" s="79"/>
+      <c r="AC5" s="79" t="s">
         <v>94</v>
       </c>
-      <c r="AD5" s="112"/>
-      <c r="AE5" s="112"/>
-      <c r="AF5" s="112"/>
-      <c r="AG5" s="112"/>
-      <c r="AH5" s="112"/>
-      <c r="AI5" s="112"/>
-      <c r="AJ5" s="113"/>
-      <c r="AK5" s="107"/>
-    </row>
-    <row r="6" spans="1:37" ht="33.75" x14ac:dyDescent="0.6">
-      <c r="A6" s="89" t="s">
+      <c r="AD5" s="79"/>
+      <c r="AE5" s="79"/>
+      <c r="AF5" s="79"/>
+      <c r="AG5" s="79"/>
+      <c r="AH5" s="79"/>
+      <c r="AI5" s="79"/>
+      <c r="AJ5" s="80"/>
+      <c r="AK5" s="97"/>
+    </row>
+    <row r="6" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.4">
+      <c r="A6" s="107" t="s">
         <v>76</v>
       </c>
-      <c r="B6" s="90"/>
-      <c r="C6" s="91"/>
+      <c r="B6" s="87"/>
+      <c r="C6" s="83"/>
       <c r="D6" s="26" t="s">
         <v>0</v>
       </c>
@@ -2464,10 +2583,10 @@
       <c r="F6" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="G6" s="59" t="s">
+      <c r="G6" s="58" t="s">
         <v>91</v>
       </c>
-      <c r="H6" s="59" t="s">
+      <c r="H6" s="58" t="s">
         <v>166</v>
       </c>
       <c r="I6" s="26" t="s">
@@ -2479,7 +2598,7 @@
       <c r="K6" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="L6" s="27" t="s">
+      <c r="L6" s="58" t="s">
         <v>3</v>
       </c>
       <c r="M6" s="26" t="s">
@@ -2554,13 +2673,13 @@
       <c r="AJ6" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="AK6" s="107"/>
-    </row>
-    <row r="7" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="93" t="s">
+      <c r="AK6" s="97"/>
+    </row>
+    <row r="7" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="91" t="s">
         <v>102</v>
       </c>
-      <c r="B7" s="85" t="s">
+      <c r="B7" s="101" t="s">
         <v>104</v>
       </c>
       <c r="C7" s="24" t="s">
@@ -2575,21 +2694,25 @@
       <c r="F7" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="G7" s="60" t="s">
+      <c r="G7" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="H7" s="60" t="s">
-        <v>130</v>
+      <c r="H7" s="136" t="s">
+        <v>181</v>
       </c>
       <c r="I7" s="30" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="J7" s="24" t="s">
-        <v>181</v>
-      </c>
-      <c r="K7" s="30"/>
-      <c r="L7" s="31"/>
-      <c r="M7" s="30"/>
+        <v>175</v>
+      </c>
+      <c r="K7" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="L7" s="59" t="s">
+        <v>121</v>
+      </c>
+      <c r="M7" s="37"/>
       <c r="N7" s="31"/>
       <c r="O7" s="31"/>
       <c r="P7" s="30"/>
@@ -2612,16 +2735,16 @@
       <c r="AG7" s="32"/>
       <c r="AH7" s="32"/>
       <c r="AI7" s="31"/>
-      <c r="AJ7" s="50"/>
-      <c r="AK7" s="45"/>
-    </row>
-    <row r="8" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="94"/>
-      <c r="B8" s="86"/>
-      <c r="C8" s="85" t="s">
+      <c r="AJ7" s="49"/>
+      <c r="AK7" s="44"/>
+    </row>
+    <row r="8" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="155"/>
+      <c r="B8" s="101"/>
+      <c r="C8" s="101" t="s">
         <v>131</v>
       </c>
-      <c r="D8" s="66" t="s">
+      <c r="D8" s="30" t="s">
         <v>150</v>
       </c>
       <c r="E8" s="30" t="s">
@@ -2630,21 +2753,25 @@
       <c r="F8" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="G8" s="60" t="s">
+      <c r="G8" s="59" t="s">
         <v>122</v>
       </c>
-      <c r="H8" s="60" t="s">
+      <c r="H8" s="136" t="s">
+        <v>182</v>
+      </c>
+      <c r="I8" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="I8" s="30" t="s">
-        <v>173</v>
-      </c>
       <c r="J8" s="30" t="s">
-        <v>180</v>
-      </c>
-      <c r="K8" s="30"/>
-      <c r="L8" s="31"/>
-      <c r="M8" s="30"/>
+        <v>174</v>
+      </c>
+      <c r="K8" s="30" t="s">
+        <v>191</v>
+      </c>
+      <c r="L8" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="M8" s="37"/>
       <c r="N8" s="31"/>
       <c r="O8" s="31"/>
       <c r="P8" s="30"/>
@@ -2667,14 +2794,14 @@
       <c r="AG8" s="32"/>
       <c r="AH8" s="32"/>
       <c r="AI8" s="31"/>
-      <c r="AJ8" s="50"/>
-      <c r="AK8" s="45"/>
-    </row>
-    <row r="9" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="94"/>
-      <c r="B9" s="86"/>
-      <c r="C9" s="86"/>
-      <c r="D9" s="82" t="s">
+      <c r="AJ8" s="49"/>
+      <c r="AK8" s="44"/>
+    </row>
+    <row r="9" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="155"/>
+      <c r="B9" s="101"/>
+      <c r="C9" s="101"/>
+      <c r="D9" s="30" t="s">
         <v>21</v>
       </c>
       <c r="E9" s="30" t="s">
@@ -2683,21 +2810,25 @@
       <c r="F9" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="G9" s="60" t="s">
+      <c r="G9" s="59" t="s">
         <v>123</v>
       </c>
-      <c r="H9" s="60" t="s">
+      <c r="H9" s="136" t="s">
+        <v>183</v>
+      </c>
+      <c r="I9" s="30" t="s">
         <v>168</v>
       </c>
-      <c r="I9" s="30" t="s">
-        <v>174</v>
-      </c>
       <c r="J9" s="30" t="s">
-        <v>182</v>
-      </c>
-      <c r="K9" s="30"/>
-      <c r="L9" s="31"/>
-      <c r="M9" s="30"/>
+        <v>176</v>
+      </c>
+      <c r="K9" s="99" t="s">
+        <v>192</v>
+      </c>
+      <c r="L9" s="142" t="s">
+        <v>201</v>
+      </c>
+      <c r="M9" s="37"/>
       <c r="N9" s="31"/>
       <c r="O9" s="31"/>
       <c r="P9" s="30"/>
@@ -2720,16 +2851,16 @@
       <c r="AG9" s="30"/>
       <c r="AH9" s="30"/>
       <c r="AI9" s="24"/>
-      <c r="AJ9" s="51"/>
-      <c r="AK9" s="46"/>
-    </row>
-    <row r="10" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="94"/>
-      <c r="B10" s="86"/>
-      <c r="C10" s="44" t="s">
+      <c r="AJ9" s="50"/>
+      <c r="AK9" s="45"/>
+    </row>
+    <row r="10" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="155"/>
+      <c r="B10" s="101"/>
+      <c r="C10" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="D10" s="66" t="s">
+      <c r="D10" s="30" t="s">
         <v>151</v>
       </c>
       <c r="E10" s="30" t="s">
@@ -2738,21 +2869,21 @@
       <c r="F10" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="G10" s="60" t="s">
+      <c r="G10" s="59" t="s">
         <v>124</v>
       </c>
-      <c r="H10" s="60" t="s">
-        <v>169</v>
+      <c r="H10" s="136" t="s">
+        <v>184</v>
       </c>
       <c r="I10" s="30" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="J10" s="30" t="s">
-        <v>182</v>
-      </c>
-      <c r="K10" s="30"/>
-      <c r="L10" s="31"/>
-      <c r="M10" s="30"/>
+        <v>176</v>
+      </c>
+      <c r="K10" s="99"/>
+      <c r="L10" s="142"/>
+      <c r="M10" s="37"/>
       <c r="N10" s="31"/>
       <c r="O10" s="31"/>
       <c r="P10" s="30"/>
@@ -2775,39 +2906,27 @@
       <c r="AG10" s="30"/>
       <c r="AH10" s="30"/>
       <c r="AI10" s="24"/>
-      <c r="AJ10" s="51"/>
-      <c r="AK10" s="46"/>
-    </row>
-    <row r="11" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="94"/>
-      <c r="B11" s="86"/>
-      <c r="C11" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="D11" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="E11" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="F11" s="30" t="s">
-        <v>117</v>
-      </c>
-      <c r="G11" s="60" t="s">
-        <v>125</v>
-      </c>
-      <c r="H11" s="60" t="s">
-        <v>170</v>
-      </c>
-      <c r="I11" s="30" t="s">
-        <v>175</v>
-      </c>
-      <c r="J11" s="24" t="s">
-        <v>183</v>
-      </c>
-      <c r="K11" s="30"/>
-      <c r="L11" s="31"/>
-      <c r="M11" s="30"/>
+      <c r="AJ10" s="50"/>
+      <c r="AK10" s="45"/>
+    </row>
+    <row r="11" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="155"/>
+      <c r="B11" s="101"/>
+      <c r="C11" s="156"/>
+      <c r="D11" s="157"/>
+      <c r="E11" s="157"/>
+      <c r="F11" s="157"/>
+      <c r="G11" s="157"/>
+      <c r="H11" s="157"/>
+      <c r="I11" s="157"/>
+      <c r="J11" s="158"/>
+      <c r="K11" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="L11" s="59" t="s">
+        <v>202</v>
+      </c>
+      <c r="M11" s="37"/>
       <c r="N11" s="31"/>
       <c r="O11" s="31"/>
       <c r="P11" s="30"/>
@@ -2830,39 +2949,27 @@
       <c r="AG11" s="30"/>
       <c r="AH11" s="30"/>
       <c r="AI11" s="24"/>
-      <c r="AJ11" s="51"/>
-      <c r="AK11" s="46"/>
-    </row>
-    <row r="12" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A12" s="94"/>
-      <c r="B12" s="86"/>
-      <c r="C12" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="D12" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="E12" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="F12" s="30" t="s">
-        <v>118</v>
-      </c>
-      <c r="G12" s="60" t="s">
-        <v>126</v>
-      </c>
-      <c r="H12" s="60" t="s">
-        <v>171</v>
-      </c>
-      <c r="I12" s="30" t="s">
-        <v>176</v>
-      </c>
-      <c r="J12" s="30" t="s">
-        <v>184</v>
-      </c>
-      <c r="K12" s="30"/>
-      <c r="L12" s="31"/>
-      <c r="M12" s="30"/>
+      <c r="AJ11" s="50"/>
+      <c r="AK11" s="45"/>
+    </row>
+    <row r="12" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="155"/>
+      <c r="B12" s="101"/>
+      <c r="C12" s="159"/>
+      <c r="D12" s="160"/>
+      <c r="E12" s="160"/>
+      <c r="F12" s="160"/>
+      <c r="G12" s="160"/>
+      <c r="H12" s="160"/>
+      <c r="I12" s="160"/>
+      <c r="J12" s="161"/>
+      <c r="K12" s="30" t="s">
+        <v>194</v>
+      </c>
+      <c r="L12" s="59" t="s">
+        <v>203</v>
+      </c>
+      <c r="M12" s="37"/>
       <c r="N12" s="31"/>
       <c r="O12" s="31"/>
       <c r="P12" s="30"/>
@@ -2885,39 +2992,43 @@
       <c r="AG12" s="30"/>
       <c r="AH12" s="30"/>
       <c r="AI12" s="24"/>
-      <c r="AJ12" s="51"/>
-      <c r="AK12" s="46"/>
-    </row>
-    <row r="13" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A13" s="94"/>
-      <c r="B13" s="92"/>
+      <c r="AJ12" s="50"/>
+      <c r="AK12" s="45"/>
+    </row>
+    <row r="13" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="155"/>
+      <c r="B13" s="101"/>
       <c r="C13" s="24" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F13" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="G13" s="60" t="s">
-        <v>127</v>
-      </c>
-      <c r="H13" s="60" t="s">
-        <v>172</v>
+        <v>117</v>
+      </c>
+      <c r="G13" s="59" t="s">
+        <v>125</v>
+      </c>
+      <c r="H13" s="136" t="s">
+        <v>185</v>
       </c>
       <c r="I13" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="J13" s="24" t="s">
         <v>177</v>
       </c>
-      <c r="J13" s="24" t="s">
-        <v>185</v>
-      </c>
-      <c r="K13" s="24"/>
-      <c r="L13" s="31"/>
-      <c r="M13" s="24"/>
+      <c r="K13" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="L13" s="59" t="s">
+        <v>125</v>
+      </c>
+      <c r="M13" s="141"/>
       <c r="N13" s="31"/>
       <c r="O13" s="31"/>
       <c r="P13" s="24"/>
@@ -2940,41 +3051,43 @@
       <c r="AG13" s="30"/>
       <c r="AH13" s="30"/>
       <c r="AI13" s="24"/>
-      <c r="AJ13" s="51"/>
-      <c r="AK13" s="46"/>
-    </row>
-    <row r="14" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A14" s="94"/>
-      <c r="B14" s="85" t="s">
-        <v>136</v>
-      </c>
-      <c r="C14" s="78" t="s">
-        <v>137</v>
-      </c>
-      <c r="D14" s="24" t="s">
-        <v>31</v>
+      <c r="AJ13" s="50"/>
+      <c r="AK13" s="45"/>
+    </row>
+    <row r="14" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="155"/>
+      <c r="B14" s="101"/>
+      <c r="C14" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="D14" s="30" t="s">
+        <v>148</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>164</v>
+        <v>134</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>163</v>
-      </c>
-      <c r="G14" s="60" t="s">
-        <v>128</v>
-      </c>
-      <c r="H14" s="60" t="s">
-        <v>164</v>
+        <v>118</v>
+      </c>
+      <c r="G14" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="H14" s="136" t="s">
+        <v>186</v>
       </c>
       <c r="I14" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="J14" s="30" t="s">
         <v>178</v>
       </c>
-      <c r="J14" s="30" t="s">
-        <v>180</v>
-      </c>
-      <c r="K14" s="30"/>
-      <c r="L14" s="31"/>
-      <c r="M14" s="30"/>
+      <c r="K14" s="30" t="s">
+        <v>196</v>
+      </c>
+      <c r="L14" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="M14" s="37"/>
       <c r="N14" s="31"/>
       <c r="O14" s="31"/>
       <c r="P14" s="30"/>
@@ -2998,38 +3111,42 @@
       <c r="AH14" s="30"/>
       <c r="AI14" s="30"/>
       <c r="AJ14" s="36"/>
-      <c r="AK14" s="46"/>
-    </row>
-    <row r="15" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A15" s="95"/>
-      <c r="B15" s="92"/>
+      <c r="AK14" s="45"/>
+    </row>
+    <row r="15" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="155"/>
+      <c r="B15" s="101"/>
       <c r="C15" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="D15" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="66" t="s">
-        <v>165</v>
+        <v>135</v>
+      </c>
+      <c r="D15" s="30" t="s">
+        <v>149</v>
+      </c>
+      <c r="E15" s="24" t="s">
+        <v>135</v>
       </c>
       <c r="F15" s="30" t="s">
-        <v>120</v>
-      </c>
-      <c r="G15" s="81" t="s">
-        <v>129</v>
-      </c>
-      <c r="H15" s="81" t="s">
-        <v>165</v>
+        <v>119</v>
+      </c>
+      <c r="G15" s="59" t="s">
+        <v>127</v>
+      </c>
+      <c r="H15" s="136" t="s">
+        <v>187</v>
       </c>
       <c r="I15" s="30" t="s">
+        <v>171</v>
+      </c>
+      <c r="J15" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="J15" s="30" t="s">
-        <v>181</v>
-      </c>
-      <c r="K15" s="30"/>
-      <c r="L15" s="30"/>
-      <c r="M15" s="30"/>
+      <c r="K15" s="30" t="s">
+        <v>197</v>
+      </c>
+      <c r="L15" s="59" t="s">
+        <v>127</v>
+      </c>
+      <c r="M15" s="37"/>
       <c r="N15" s="30"/>
       <c r="O15" s="30"/>
       <c r="P15" s="30"/>
@@ -3053,110 +3170,150 @@
       <c r="AH15" s="30"/>
       <c r="AI15" s="30"/>
       <c r="AJ15" s="36"/>
-      <c r="AK15" s="46"/>
-    </row>
-    <row r="16" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A16" s="56" t="s">
-        <v>78</v>
-      </c>
-      <c r="B16" s="64" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" s="58"/>
-      <c r="D16" s="80" t="s">
-        <v>152</v>
+      <c r="AK15" s="45"/>
+    </row>
+    <row r="16" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="155"/>
+      <c r="B16" s="101" t="s">
+        <v>136</v>
+      </c>
+      <c r="C16" s="74" t="s">
+        <v>137</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>31</v>
       </c>
       <c r="E16" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="I16" s="56"/>
-      <c r="J16" s="56"/>
-      <c r="K16" s="30"/>
-      <c r="L16" s="30"/>
-      <c r="M16" s="30"/>
+        <v>164</v>
+      </c>
+      <c r="F16" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="G16" s="59" t="s">
+        <v>128</v>
+      </c>
+      <c r="H16" s="136" t="s">
+        <v>188</v>
+      </c>
+      <c r="I16" s="30" t="s">
+        <v>172</v>
+      </c>
+      <c r="J16" s="30" t="s">
+        <v>174</v>
+      </c>
+      <c r="K16" s="30" t="s">
+        <v>198</v>
+      </c>
+      <c r="L16" s="59" t="s">
+        <v>128</v>
+      </c>
+      <c r="M16" s="37"/>
       <c r="N16" s="30"/>
       <c r="O16" s="30"/>
       <c r="P16" s="30"/>
-      <c r="Q16" s="102"/>
-      <c r="R16" s="104"/>
-      <c r="S16" s="96"/>
-      <c r="T16" s="96"/>
-      <c r="U16" s="96"/>
-      <c r="V16" s="98"/>
-      <c r="W16" s="96"/>
-      <c r="X16" s="96"/>
-      <c r="Y16" s="96"/>
-      <c r="Z16" s="96"/>
-      <c r="AA16" s="97"/>
-      <c r="AB16" s="96"/>
-      <c r="AC16" s="97"/>
+      <c r="Q16" s="91"/>
+      <c r="R16" s="93"/>
+      <c r="S16" s="95"/>
+      <c r="T16" s="95"/>
+      <c r="U16" s="95"/>
+      <c r="V16" s="104"/>
+      <c r="W16" s="95"/>
+      <c r="X16" s="95"/>
+      <c r="Y16" s="95"/>
+      <c r="Z16" s="95"/>
+      <c r="AA16" s="99"/>
+      <c r="AB16" s="95"/>
+      <c r="AC16" s="99"/>
       <c r="AD16" s="101"/>
-      <c r="AE16" s="97"/>
-      <c r="AF16" s="97"/>
-      <c r="AG16" s="97"/>
-      <c r="AH16" s="97"/>
-      <c r="AI16" s="97"/>
-      <c r="AJ16" s="109"/>
-      <c r="AK16" s="108"/>
-    </row>
-    <row r="17" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A17" s="56"/>
-      <c r="B17" s="79"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="80" t="s">
-        <v>153</v>
-      </c>
-      <c r="E17" s="24" t="s">
-        <v>140</v>
-      </c>
-      <c r="I17" s="65"/>
-      <c r="J17" s="64"/>
-      <c r="K17" s="66"/>
-      <c r="L17" s="66"/>
-      <c r="M17" s="66"/>
-      <c r="N17" s="66"/>
-      <c r="O17" s="66"/>
-      <c r="P17" s="66"/>
-      <c r="Q17" s="103"/>
-      <c r="R17" s="105"/>
-      <c r="S17" s="96"/>
-      <c r="T17" s="96"/>
-      <c r="U17" s="96"/>
-      <c r="V17" s="96"/>
-      <c r="W17" s="96"/>
-      <c r="X17" s="96"/>
-      <c r="Y17" s="96"/>
-      <c r="Z17" s="96"/>
-      <c r="AA17" s="96"/>
-      <c r="AB17" s="96"/>
-      <c r="AC17" s="97"/>
-      <c r="AD17" s="97"/>
-      <c r="AE17" s="97"/>
-      <c r="AF17" s="97"/>
-      <c r="AG17" s="97"/>
-      <c r="AH17" s="97"/>
-      <c r="AI17" s="97"/>
-      <c r="AJ17" s="109"/>
-      <c r="AK17" s="108"/>
-    </row>
-    <row r="18" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A18" s="56"/>
-      <c r="B18" s="79"/>
-      <c r="C18" s="58"/>
-      <c r="D18" s="30" t="s">
-        <v>154</v>
+      <c r="AE16" s="99"/>
+      <c r="AF16" s="99"/>
+      <c r="AG16" s="99"/>
+      <c r="AH16" s="99"/>
+      <c r="AI16" s="99"/>
+      <c r="AJ16" s="100"/>
+      <c r="AK16" s="98"/>
+    </row>
+    <row r="17" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="92"/>
+      <c r="B17" s="101"/>
+      <c r="C17" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="D17" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="F17" s="30" t="s">
+        <v>120</v>
+      </c>
+      <c r="G17" s="59" t="s">
+        <v>129</v>
+      </c>
+      <c r="H17" s="136" t="s">
+        <v>189</v>
+      </c>
+      <c r="I17" s="30" t="s">
+        <v>173</v>
+      </c>
+      <c r="J17" s="30" t="s">
+        <v>175</v>
+      </c>
+      <c r="K17" s="30" t="s">
+        <v>199</v>
+      </c>
+      <c r="L17" s="59" t="s">
+        <v>129</v>
+      </c>
+      <c r="M17" s="76"/>
+      <c r="N17" s="62"/>
+      <c r="O17" s="62"/>
+      <c r="P17" s="62"/>
+      <c r="Q17" s="92"/>
+      <c r="R17" s="94"/>
+      <c r="S17" s="95"/>
+      <c r="T17" s="95"/>
+      <c r="U17" s="95"/>
+      <c r="V17" s="95"/>
+      <c r="W17" s="95"/>
+      <c r="X17" s="95"/>
+      <c r="Y17" s="95"/>
+      <c r="Z17" s="95"/>
+      <c r="AA17" s="95"/>
+      <c r="AB17" s="95"/>
+      <c r="AC17" s="99"/>
+      <c r="AD17" s="99"/>
+      <c r="AE17" s="99"/>
+      <c r="AF17" s="99"/>
+      <c r="AG17" s="99"/>
+      <c r="AH17" s="99"/>
+      <c r="AI17" s="99"/>
+      <c r="AJ17" s="100"/>
+      <c r="AK17" s="98"/>
+    </row>
+    <row r="18" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="137" t="s">
+        <v>78</v>
+      </c>
+      <c r="B18" s="101" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" s="140"/>
+      <c r="D18" s="75" t="s">
+        <v>152</v>
       </c>
       <c r="E18" s="24" t="s">
-        <v>141</v>
-      </c>
-      <c r="F18" s="58"/>
-      <c r="G18" s="58"/>
-      <c r="H18" s="58"/>
-      <c r="I18" s="56"/>
-      <c r="J18" s="57"/>
-      <c r="K18" s="30"/>
+        <v>139</v>
+      </c>
+      <c r="F18" s="57"/>
+      <c r="G18" s="57"/>
+      <c r="H18" s="57"/>
+      <c r="I18" s="55"/>
+      <c r="J18" s="56"/>
+      <c r="K18" s="143"/>
       <c r="L18" s="30"/>
-      <c r="M18" s="30"/>
+      <c r="M18" s="37"/>
       <c r="N18" s="30"/>
       <c r="O18" s="30"/>
       <c r="P18" s="30"/>
@@ -3180,26 +3337,26 @@
       <c r="AH18" s="30"/>
       <c r="AI18" s="30"/>
       <c r="AJ18" s="36"/>
-      <c r="AK18" s="46"/>
-    </row>
-    <row r="19" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A19" s="56"/>
-      <c r="B19" s="79"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="30" t="s">
-        <v>155</v>
+      <c r="AK18" s="45"/>
+    </row>
+    <row r="19" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="138"/>
+      <c r="B19" s="101"/>
+      <c r="C19" s="140"/>
+      <c r="D19" s="75" t="s">
+        <v>153</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>142</v>
-      </c>
-      <c r="F19" s="56"/>
-      <c r="G19" s="57"/>
-      <c r="H19" s="57"/>
-      <c r="I19" s="56"/>
-      <c r="J19" s="57"/>
+        <v>140</v>
+      </c>
+      <c r="F19" s="55"/>
+      <c r="G19" s="56"/>
+      <c r="H19" s="56"/>
+      <c r="I19" s="55"/>
+      <c r="J19" s="56"/>
       <c r="K19" s="30"/>
       <c r="L19" s="30"/>
-      <c r="M19" s="30"/>
+      <c r="M19" s="37"/>
       <c r="N19" s="30"/>
       <c r="O19" s="30"/>
       <c r="P19" s="30"/>
@@ -3207,7 +3364,7 @@
       <c r="R19" s="35"/>
       <c r="S19" s="33"/>
       <c r="T19" s="33"/>
-      <c r="U19" s="96"/>
+      <c r="U19" s="95"/>
       <c r="V19" s="35"/>
       <c r="W19" s="35"/>
       <c r="X19" s="35"/>
@@ -3223,26 +3380,26 @@
       <c r="AH19" s="30"/>
       <c r="AI19" s="30"/>
       <c r="AJ19" s="36"/>
-      <c r="AK19" s="46"/>
-    </row>
-    <row r="20" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A20" s="56"/>
-      <c r="B20" s="61"/>
-      <c r="C20" s="58"/>
-      <c r="D20" s="24" t="s">
-        <v>156</v>
+      <c r="AK19" s="45"/>
+    </row>
+    <row r="20" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="138"/>
+      <c r="B20" s="101"/>
+      <c r="C20" s="140"/>
+      <c r="D20" s="30" t="s">
+        <v>154</v>
       </c>
       <c r="E20" s="24" t="s">
-        <v>143</v>
-      </c>
-      <c r="F20" s="56"/>
-      <c r="G20" s="57"/>
-      <c r="H20" s="57"/>
-      <c r="I20" s="56"/>
-      <c r="J20" s="57"/>
+        <v>141</v>
+      </c>
+      <c r="F20" s="55"/>
+      <c r="G20" s="56"/>
+      <c r="H20" s="56"/>
+      <c r="I20" s="55"/>
+      <c r="J20" s="56"/>
       <c r="K20" s="30"/>
       <c r="L20" s="30"/>
-      <c r="M20" s="30"/>
+      <c r="M20" s="37"/>
       <c r="N20" s="30"/>
       <c r="O20" s="30"/>
       <c r="P20" s="30"/>
@@ -3250,7 +3407,7 @@
       <c r="R20" s="35"/>
       <c r="S20" s="33"/>
       <c r="T20" s="33"/>
-      <c r="U20" s="96"/>
+      <c r="U20" s="95"/>
       <c r="V20" s="25"/>
       <c r="W20" s="35"/>
       <c r="X20" s="35"/>
@@ -3266,28 +3423,26 @@
       <c r="AH20" s="30"/>
       <c r="AI20" s="30"/>
       <c r="AJ20" s="36"/>
-      <c r="AK20" s="46"/>
-    </row>
-    <row r="21" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A21" s="56"/>
-      <c r="B21" s="64" t="s">
-        <v>136</v>
-      </c>
-      <c r="C21" s="58"/>
-      <c r="D21" s="24" t="s">
-        <v>157</v>
+      <c r="AK20" s="45"/>
+    </row>
+    <row r="21" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="138"/>
+      <c r="B21" s="101"/>
+      <c r="C21" s="140"/>
+      <c r="D21" s="30" t="s">
+        <v>155</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>146</v>
-      </c>
-      <c r="F21" s="56"/>
-      <c r="G21" s="57"/>
-      <c r="H21" s="57"/>
-      <c r="I21" s="56"/>
-      <c r="J21" s="57"/>
+        <v>142</v>
+      </c>
+      <c r="F21" s="55"/>
+      <c r="G21" s="56"/>
+      <c r="H21" s="56"/>
+      <c r="I21" s="55"/>
+      <c r="J21" s="56"/>
       <c r="K21" s="30"/>
       <c r="L21" s="30"/>
-      <c r="M21" s="30"/>
+      <c r="M21" s="37"/>
       <c r="N21" s="30"/>
       <c r="O21" s="30"/>
       <c r="P21" s="30"/>
@@ -3310,27 +3465,27 @@
       <c r="AG21" s="30"/>
       <c r="AH21" s="30"/>
       <c r="AI21" s="24"/>
-      <c r="AJ21" s="51"/>
-      <c r="AK21" s="46"/>
-    </row>
-    <row r="22" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A22" s="56"/>
-      <c r="B22" s="79"/>
-      <c r="C22" s="58"/>
+      <c r="AJ21" s="50"/>
+      <c r="AK21" s="45"/>
+    </row>
+    <row r="22" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="138"/>
+      <c r="B22" s="101"/>
+      <c r="C22" s="140"/>
       <c r="D22" s="24" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E22" s="24" t="s">
-        <v>144</v>
-      </c>
-      <c r="F22" s="56"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="57"/>
-      <c r="I22" s="56"/>
-      <c r="J22" s="57"/>
+        <v>143</v>
+      </c>
+      <c r="F22" s="55"/>
+      <c r="G22" s="56"/>
+      <c r="H22" s="56"/>
+      <c r="I22" s="55"/>
+      <c r="J22" s="56"/>
       <c r="K22" s="30"/>
       <c r="L22" s="30"/>
-      <c r="M22" s="30"/>
+      <c r="M22" s="37"/>
       <c r="N22" s="30"/>
       <c r="O22" s="30"/>
       <c r="P22" s="30"/>
@@ -3353,27 +3508,29 @@
       <c r="AG22" s="30"/>
       <c r="AH22" s="30"/>
       <c r="AI22" s="24"/>
-      <c r="AJ22" s="51"/>
-      <c r="AK22" s="46"/>
-    </row>
-    <row r="23" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A23" s="56"/>
-      <c r="B23" s="61"/>
-      <c r="C23" s="58"/>
+      <c r="AJ22" s="50"/>
+      <c r="AK22" s="45"/>
+    </row>
+    <row r="23" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="138"/>
+      <c r="B23" s="101" t="s">
+        <v>136</v>
+      </c>
+      <c r="C23" s="140"/>
       <c r="D23" s="24" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>145</v>
-      </c>
-      <c r="F23" s="56"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="56"/>
-      <c r="J23" s="57"/>
+        <v>146</v>
+      </c>
+      <c r="F23" s="55"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="55"/>
+      <c r="J23" s="56"/>
       <c r="K23" s="30"/>
       <c r="L23" s="30"/>
-      <c r="M23" s="30"/>
+      <c r="M23" s="37"/>
       <c r="N23" s="30"/>
       <c r="O23" s="30"/>
       <c r="P23" s="30"/>
@@ -3396,18 +3553,27 @@
       <c r="AG23" s="30"/>
       <c r="AH23" s="30"/>
       <c r="AI23" s="24"/>
-      <c r="AJ23" s="51"/>
-      <c r="AK23" s="46"/>
-    </row>
-    <row r="24" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="F24" s="56"/>
-      <c r="G24" s="57"/>
-      <c r="H24" s="57"/>
-      <c r="I24" s="56"/>
-      <c r="J24" s="57"/>
+      <c r="AJ23" s="50"/>
+      <c r="AK23" s="45"/>
+    </row>
+    <row r="24" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="138"/>
+      <c r="B24" s="101"/>
+      <c r="C24" s="140"/>
+      <c r="D24" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="E24" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F24" s="55"/>
+      <c r="G24" s="56"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="55"/>
+      <c r="J24" s="56"/>
       <c r="K24" s="30"/>
       <c r="L24" s="24"/>
-      <c r="M24" s="30"/>
+      <c r="M24" s="37"/>
       <c r="N24" s="24"/>
       <c r="O24" s="24"/>
       <c r="P24" s="30"/>
@@ -3431,17 +3597,26 @@
       <c r="AH24" s="30"/>
       <c r="AI24" s="30"/>
       <c r="AJ24" s="36"/>
-      <c r="AK24" s="46"/>
-    </row>
-    <row r="25" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="F25" s="56"/>
-      <c r="G25" s="57"/>
-      <c r="H25" s="57"/>
-      <c r="I25" s="56"/>
-      <c r="J25" s="57"/>
+      <c r="AK24" s="45"/>
+    </row>
+    <row r="25" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="139"/>
+      <c r="B25" s="101"/>
+      <c r="C25" s="140"/>
+      <c r="D25" s="24" t="s">
+        <v>159</v>
+      </c>
+      <c r="E25" s="24" t="s">
+        <v>145</v>
+      </c>
+      <c r="F25" s="55"/>
+      <c r="G25" s="56"/>
+      <c r="H25" s="56"/>
+      <c r="I25" s="55"/>
+      <c r="J25" s="56"/>
       <c r="K25" s="30"/>
       <c r="L25" s="24"/>
-      <c r="M25" s="30"/>
+      <c r="M25" s="37"/>
       <c r="N25" s="24"/>
       <c r="O25" s="24"/>
       <c r="P25" s="30"/>
@@ -3465,25 +3640,25 @@
       <c r="AH25" s="30"/>
       <c r="AI25" s="30"/>
       <c r="AJ25" s="36"/>
-      <c r="AK25" s="46"/>
-    </row>
-    <row r="26" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A26" s="68"/>
-      <c r="B26" s="67"/>
-      <c r="C26" s="67"/>
-      <c r="D26" s="67"/>
-      <c r="E26" s="68"/>
-      <c r="F26" s="68"/>
-      <c r="G26" s="67"/>
-      <c r="H26" s="67"/>
-      <c r="I26" s="68"/>
-      <c r="J26" s="67"/>
-      <c r="K26" s="69"/>
-      <c r="L26" s="70"/>
-      <c r="M26" s="69"/>
-      <c r="N26" s="70"/>
-      <c r="O26" s="70"/>
-      <c r="P26" s="69"/>
+      <c r="AK25" s="45"/>
+    </row>
+    <row r="26" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="64"/>
+      <c r="B26" s="63"/>
+      <c r="C26" s="63"/>
+      <c r="D26" s="63"/>
+      <c r="E26" s="64"/>
+      <c r="F26" s="64"/>
+      <c r="G26" s="63"/>
+      <c r="H26" s="63"/>
+      <c r="I26" s="64"/>
+      <c r="J26" s="63"/>
+      <c r="K26" s="65"/>
+      <c r="L26" s="66"/>
+      <c r="M26" s="65"/>
+      <c r="N26" s="66"/>
+      <c r="O26" s="66"/>
+      <c r="P26" s="65"/>
       <c r="Q26" s="34"/>
       <c r="R26" s="33"/>
       <c r="S26" s="35"/>
@@ -3504,27 +3679,27 @@
       <c r="AH26" s="30"/>
       <c r="AI26" s="30"/>
       <c r="AJ26" s="36"/>
-      <c r="AK26" s="46"/>
-    </row>
-    <row r="27" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A27" s="68"/>
-      <c r="B27" s="67"/>
-      <c r="C27" s="67"/>
-      <c r="D27" s="67"/>
-      <c r="E27" s="68"/>
-      <c r="F27" s="68"/>
-      <c r="G27" s="67"/>
-      <c r="H27" s="67"/>
-      <c r="I27" s="68"/>
-      <c r="J27" s="67"/>
-      <c r="K27" s="69"/>
-      <c r="L27" s="70"/>
-      <c r="M27" s="69"/>
-      <c r="N27" s="70"/>
-      <c r="O27" s="70"/>
-      <c r="P27" s="69"/>
-      <c r="Q27" s="99"/>
-      <c r="R27" s="100"/>
+      <c r="AK26" s="45"/>
+    </row>
+    <row r="27" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="64"/>
+      <c r="B27" s="63"/>
+      <c r="C27" s="63"/>
+      <c r="D27" s="63"/>
+      <c r="E27" s="64"/>
+      <c r="F27" s="64"/>
+      <c r="G27" s="63"/>
+      <c r="H27" s="63"/>
+      <c r="I27" s="64"/>
+      <c r="J27" s="63"/>
+      <c r="K27" s="65"/>
+      <c r="L27" s="66"/>
+      <c r="M27" s="65"/>
+      <c r="N27" s="66"/>
+      <c r="O27" s="66"/>
+      <c r="P27" s="65"/>
+      <c r="Q27" s="102"/>
+      <c r="R27" s="103"/>
       <c r="S27" s="35"/>
       <c r="T27" s="35"/>
       <c r="U27" s="35"/>
@@ -3533,8 +3708,8 @@
       <c r="X27" s="35"/>
       <c r="Y27" s="35"/>
       <c r="Z27" s="35"/>
-      <c r="AA27" s="97"/>
-      <c r="AB27" s="97"/>
+      <c r="AA27" s="99"/>
+      <c r="AB27" s="99"/>
       <c r="AC27" s="30"/>
       <c r="AD27" s="30"/>
       <c r="AE27" s="30"/>
@@ -3543,27 +3718,27 @@
       <c r="AH27" s="30"/>
       <c r="AI27" s="30"/>
       <c r="AJ27" s="36"/>
-      <c r="AK27" s="47"/>
-    </row>
-    <row r="28" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A28" s="68"/>
-      <c r="B28" s="67"/>
-      <c r="C28" s="67"/>
-      <c r="D28" s="67"/>
-      <c r="E28" s="68"/>
-      <c r="F28" s="68"/>
-      <c r="G28" s="67"/>
-      <c r="H28" s="67"/>
-      <c r="I28" s="68"/>
-      <c r="J28" s="67"/>
-      <c r="K28" s="69"/>
-      <c r="L28" s="70"/>
-      <c r="M28" s="69"/>
-      <c r="N28" s="70"/>
-      <c r="O28" s="70"/>
-      <c r="P28" s="69"/>
-      <c r="Q28" s="99"/>
-      <c r="R28" s="100"/>
+      <c r="AK27" s="46"/>
+    </row>
+    <row r="28" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="64"/>
+      <c r="B28" s="63"/>
+      <c r="C28" s="63"/>
+      <c r="D28" s="63"/>
+      <c r="E28" s="64"/>
+      <c r="F28" s="64"/>
+      <c r="G28" s="63"/>
+      <c r="H28" s="63"/>
+      <c r="I28" s="64"/>
+      <c r="J28" s="63"/>
+      <c r="K28" s="65"/>
+      <c r="L28" s="66"/>
+      <c r="M28" s="65"/>
+      <c r="N28" s="66"/>
+      <c r="O28" s="66"/>
+      <c r="P28" s="65"/>
+      <c r="Q28" s="102"/>
+      <c r="R28" s="103"/>
       <c r="S28" s="35"/>
       <c r="T28" s="35"/>
       <c r="U28" s="35"/>
@@ -3572,8 +3747,8 @@
       <c r="X28" s="35"/>
       <c r="Y28" s="35"/>
       <c r="Z28" s="35"/>
-      <c r="AA28" s="97"/>
-      <c r="AB28" s="97"/>
+      <c r="AA28" s="99"/>
+      <c r="AB28" s="99"/>
       <c r="AC28" s="30"/>
       <c r="AD28" s="30"/>
       <c r="AE28" s="30"/>
@@ -3582,27 +3757,27 @@
       <c r="AH28" s="30"/>
       <c r="AI28" s="30"/>
       <c r="AJ28" s="36"/>
-      <c r="AK28" s="47"/>
-    </row>
-    <row r="29" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A29" s="68"/>
-      <c r="B29" s="67"/>
-      <c r="C29" s="67"/>
-      <c r="D29" s="67"/>
-      <c r="E29" s="68"/>
-      <c r="F29" s="68"/>
-      <c r="G29" s="67"/>
-      <c r="H29" s="67"/>
-      <c r="I29" s="68"/>
-      <c r="J29" s="67"/>
-      <c r="K29" s="69"/>
-      <c r="L29" s="70"/>
-      <c r="M29" s="69"/>
-      <c r="N29" s="70"/>
-      <c r="O29" s="70"/>
-      <c r="P29" s="69"/>
-      <c r="Q29" s="99"/>
-      <c r="R29" s="100"/>
+      <c r="AK28" s="46"/>
+    </row>
+    <row r="29" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="64"/>
+      <c r="B29" s="63"/>
+      <c r="C29" s="63"/>
+      <c r="D29" s="63"/>
+      <c r="E29" s="64"/>
+      <c r="F29" s="64"/>
+      <c r="G29" s="63"/>
+      <c r="H29" s="63"/>
+      <c r="I29" s="64"/>
+      <c r="J29" s="63"/>
+      <c r="K29" s="65"/>
+      <c r="L29" s="66"/>
+      <c r="M29" s="65"/>
+      <c r="N29" s="66"/>
+      <c r="O29" s="66"/>
+      <c r="P29" s="65"/>
+      <c r="Q29" s="102"/>
+      <c r="R29" s="103"/>
       <c r="S29" s="35"/>
       <c r="T29" s="35"/>
       <c r="U29" s="35"/>
@@ -3611,8 +3786,8 @@
       <c r="X29" s="35"/>
       <c r="Y29" s="35"/>
       <c r="Z29" s="35"/>
-      <c r="AA29" s="97"/>
-      <c r="AB29" s="97"/>
+      <c r="AA29" s="99"/>
+      <c r="AB29" s="99"/>
       <c r="AC29" s="30"/>
       <c r="AD29" s="30"/>
       <c r="AE29" s="30"/>
@@ -3621,27 +3796,27 @@
       <c r="AH29" s="30"/>
       <c r="AI29" s="30"/>
       <c r="AJ29" s="36"/>
-      <c r="AK29" s="47"/>
-    </row>
-    <row r="30" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A30" s="68"/>
-      <c r="B30" s="67"/>
-      <c r="C30" s="67"/>
-      <c r="D30" s="67"/>
-      <c r="E30" s="68"/>
-      <c r="F30" s="68"/>
-      <c r="G30" s="67"/>
-      <c r="H30" s="67"/>
-      <c r="I30" s="68"/>
-      <c r="J30" s="67"/>
-      <c r="K30" s="69"/>
-      <c r="L30" s="70"/>
-      <c r="M30" s="69"/>
-      <c r="N30" s="70"/>
-      <c r="O30" s="70"/>
-      <c r="P30" s="69"/>
-      <c r="Q30" s="99"/>
-      <c r="R30" s="100"/>
+      <c r="AK29" s="46"/>
+    </row>
+    <row r="30" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="64"/>
+      <c r="B30" s="63"/>
+      <c r="C30" s="63"/>
+      <c r="D30" s="63"/>
+      <c r="E30" s="64"/>
+      <c r="F30" s="64"/>
+      <c r="G30" s="63"/>
+      <c r="H30" s="63"/>
+      <c r="I30" s="64"/>
+      <c r="J30" s="63"/>
+      <c r="K30" s="65"/>
+      <c r="L30" s="66"/>
+      <c r="M30" s="65"/>
+      <c r="N30" s="66"/>
+      <c r="O30" s="66"/>
+      <c r="P30" s="65"/>
+      <c r="Q30" s="102"/>
+      <c r="R30" s="103"/>
       <c r="S30" s="35"/>
       <c r="T30" s="35"/>
       <c r="U30" s="35"/>
@@ -3650,8 +3825,8 @@
       <c r="X30" s="35"/>
       <c r="Y30" s="35"/>
       <c r="Z30" s="35"/>
-      <c r="AA30" s="97"/>
-      <c r="AB30" s="97"/>
+      <c r="AA30" s="99"/>
+      <c r="AB30" s="99"/>
       <c r="AC30" s="30"/>
       <c r="AD30" s="30"/>
       <c r="AE30" s="30"/>
@@ -3660,24 +3835,24 @@
       <c r="AH30" s="30"/>
       <c r="AI30" s="30"/>
       <c r="AJ30" s="36"/>
-      <c r="AK30" s="47"/>
-    </row>
-    <row r="31" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="D31" s="70"/>
-      <c r="E31" s="70"/>
-      <c r="F31" s="70"/>
-      <c r="G31" s="70"/>
-      <c r="H31" s="70"/>
-      <c r="I31" s="70"/>
-      <c r="J31" s="70"/>
-      <c r="K31" s="69"/>
-      <c r="L31" s="70"/>
-      <c r="M31" s="69"/>
-      <c r="N31" s="70"/>
-      <c r="O31" s="70"/>
-      <c r="P31" s="69"/>
-      <c r="Q31" s="99"/>
-      <c r="R31" s="100"/>
+      <c r="AK30" s="46"/>
+    </row>
+    <row r="31" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D31" s="66"/>
+      <c r="E31" s="66"/>
+      <c r="F31" s="66"/>
+      <c r="G31" s="66"/>
+      <c r="H31" s="66"/>
+      <c r="I31" s="66"/>
+      <c r="J31" s="66"/>
+      <c r="K31" s="65"/>
+      <c r="L31" s="66"/>
+      <c r="M31" s="65"/>
+      <c r="N31" s="66"/>
+      <c r="O31" s="66"/>
+      <c r="P31" s="65"/>
+      <c r="Q31" s="102"/>
+      <c r="R31" s="103"/>
       <c r="S31" s="35"/>
       <c r="T31" s="35"/>
       <c r="U31" s="35"/>
@@ -3686,8 +3861,8 @@
       <c r="X31" s="35"/>
       <c r="Y31" s="35"/>
       <c r="Z31" s="35"/>
-      <c r="AA31" s="97"/>
-      <c r="AB31" s="97"/>
+      <c r="AA31" s="99"/>
+      <c r="AB31" s="99"/>
       <c r="AC31" s="30"/>
       <c r="AD31" s="30"/>
       <c r="AE31" s="30"/>
@@ -3696,22 +3871,22 @@
       <c r="AH31" s="30"/>
       <c r="AI31" s="30"/>
       <c r="AJ31" s="36"/>
-      <c r="AK31" s="47"/>
-    </row>
-    <row r="32" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="D32" s="67"/>
-      <c r="E32" s="67"/>
-      <c r="F32" s="67"/>
-      <c r="G32" s="67"/>
-      <c r="H32" s="67"/>
-      <c r="I32" s="70"/>
-      <c r="J32" s="87"/>
-      <c r="K32" s="69"/>
-      <c r="L32" s="69"/>
-      <c r="M32" s="69"/>
-      <c r="N32" s="69"/>
-      <c r="O32" s="69"/>
-      <c r="P32" s="69"/>
+      <c r="AK31" s="46"/>
+    </row>
+    <row r="32" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D32" s="63"/>
+      <c r="E32" s="63"/>
+      <c r="F32" s="63"/>
+      <c r="G32" s="63"/>
+      <c r="H32" s="63"/>
+      <c r="I32" s="66"/>
+      <c r="J32" s="105"/>
+      <c r="K32" s="65"/>
+      <c r="L32" s="65"/>
+      <c r="M32" s="65"/>
+      <c r="N32" s="65"/>
+      <c r="O32" s="65"/>
+      <c r="P32" s="65"/>
       <c r="Q32" s="37"/>
       <c r="R32" s="33"/>
       <c r="S32" s="35"/>
@@ -3732,22 +3907,22 @@
       <c r="AH32" s="30"/>
       <c r="AI32" s="30"/>
       <c r="AJ32" s="36"/>
-      <c r="AK32" s="47"/>
-    </row>
-    <row r="33" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="D33" s="67"/>
-      <c r="E33" s="67"/>
-      <c r="F33" s="67"/>
-      <c r="G33" s="67"/>
-      <c r="H33" s="67"/>
-      <c r="I33" s="70"/>
-      <c r="J33" s="87"/>
-      <c r="K33" s="69"/>
-      <c r="L33" s="69"/>
-      <c r="M33" s="69"/>
-      <c r="N33" s="69"/>
-      <c r="O33" s="69"/>
-      <c r="P33" s="69"/>
+      <c r="AK32" s="46"/>
+    </row>
+    <row r="33" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D33" s="63"/>
+      <c r="E33" s="63"/>
+      <c r="F33" s="63"/>
+      <c r="G33" s="63"/>
+      <c r="H33" s="63"/>
+      <c r="I33" s="66"/>
+      <c r="J33" s="105"/>
+      <c r="K33" s="65"/>
+      <c r="L33" s="65"/>
+      <c r="M33" s="65"/>
+      <c r="N33" s="65"/>
+      <c r="O33" s="65"/>
+      <c r="P33" s="65"/>
       <c r="Q33" s="37"/>
       <c r="R33" s="33"/>
       <c r="S33" s="35"/>
@@ -3768,22 +3943,22 @@
       <c r="AH33" s="30"/>
       <c r="AI33" s="30"/>
       <c r="AJ33" s="36"/>
-      <c r="AK33" s="47"/>
-    </row>
-    <row r="34" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="D34" s="70"/>
-      <c r="E34" s="70"/>
-      <c r="F34" s="70"/>
-      <c r="G34" s="70"/>
-      <c r="H34" s="70"/>
-      <c r="I34" s="70"/>
-      <c r="J34" s="70"/>
-      <c r="K34" s="69"/>
-      <c r="L34" s="69"/>
-      <c r="M34" s="69"/>
-      <c r="N34" s="69"/>
-      <c r="O34" s="69"/>
-      <c r="P34" s="69"/>
+      <c r="AK33" s="46"/>
+    </row>
+    <row r="34" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D34" s="66"/>
+      <c r="E34" s="66"/>
+      <c r="F34" s="66"/>
+      <c r="G34" s="66"/>
+      <c r="H34" s="66"/>
+      <c r="I34" s="66"/>
+      <c r="J34" s="66"/>
+      <c r="K34" s="65"/>
+      <c r="L34" s="65"/>
+      <c r="M34" s="65"/>
+      <c r="N34" s="65"/>
+      <c r="O34" s="65"/>
+      <c r="P34" s="65"/>
       <c r="Q34" s="37"/>
       <c r="R34" s="33"/>
       <c r="S34" s="35"/>
@@ -3804,22 +3979,22 @@
       <c r="AH34" s="30"/>
       <c r="AI34" s="30"/>
       <c r="AJ34" s="36"/>
-      <c r="AK34" s="47"/>
-    </row>
-    <row r="35" spans="1:37" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="D35" s="71"/>
-      <c r="E35" s="72"/>
-      <c r="F35" s="70"/>
-      <c r="G35" s="70"/>
-      <c r="H35" s="70"/>
-      <c r="I35" s="70"/>
-      <c r="J35" s="70"/>
-      <c r="K35" s="69"/>
-      <c r="L35" s="69"/>
-      <c r="M35" s="69"/>
-      <c r="N35" s="69"/>
-      <c r="O35" s="69"/>
-      <c r="P35" s="69"/>
+      <c r="AK34" s="46"/>
+    </row>
+    <row r="35" spans="1:37" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="D35" s="67"/>
+      <c r="E35" s="68"/>
+      <c r="F35" s="66"/>
+      <c r="G35" s="66"/>
+      <c r="H35" s="66"/>
+      <c r="I35" s="66"/>
+      <c r="J35" s="66"/>
+      <c r="K35" s="65"/>
+      <c r="L35" s="65"/>
+      <c r="M35" s="65"/>
+      <c r="N35" s="65"/>
+      <c r="O35" s="65"/>
+      <c r="P35" s="65"/>
       <c r="Q35" s="39"/>
       <c r="R35" s="40"/>
       <c r="S35" s="41"/>
@@ -3839,23 +4014,23 @@
       <c r="AG35" s="42"/>
       <c r="AH35" s="42"/>
       <c r="AI35" s="42"/>
-      <c r="AJ35" s="52"/>
-      <c r="AK35" s="48"/>
-    </row>
-    <row r="36" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="D36" s="73"/>
-      <c r="E36" s="74"/>
-      <c r="F36" s="69"/>
-      <c r="G36" s="69"/>
-      <c r="H36" s="69"/>
-      <c r="I36" s="69"/>
-      <c r="J36" s="88"/>
-      <c r="K36" s="69"/>
-      <c r="L36" s="69"/>
-      <c r="M36" s="69"/>
-      <c r="N36" s="69"/>
-      <c r="O36" s="69"/>
-      <c r="P36" s="69"/>
+      <c r="AJ35" s="51"/>
+      <c r="AK35" s="47"/>
+    </row>
+    <row r="36" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D36" s="69"/>
+      <c r="E36" s="70"/>
+      <c r="F36" s="65"/>
+      <c r="G36" s="65"/>
+      <c r="H36" s="65"/>
+      <c r="I36" s="65"/>
+      <c r="J36" s="106"/>
+      <c r="K36" s="65"/>
+      <c r="L36" s="65"/>
+      <c r="M36" s="65"/>
+      <c r="N36" s="65"/>
+      <c r="O36" s="65"/>
+      <c r="P36" s="65"/>
       <c r="Q36" s="43"/>
       <c r="R36" s="43"/>
       <c r="S36" s="43"/>
@@ -3875,23 +4050,23 @@
       <c r="AG36" s="43"/>
       <c r="AH36" s="43"/>
       <c r="AI36" s="43"/>
-      <c r="AJ36" s="53"/>
+      <c r="AJ36" s="52"/>
       <c r="AK36" s="43"/>
     </row>
-    <row r="37" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="D37" s="73"/>
-      <c r="E37" s="74"/>
-      <c r="F37" s="69"/>
-      <c r="G37" s="69"/>
-      <c r="H37" s="69"/>
-      <c r="I37" s="69"/>
-      <c r="J37" s="88"/>
-      <c r="K37" s="69"/>
-      <c r="L37" s="69"/>
-      <c r="M37" s="69"/>
-      <c r="N37" s="69"/>
-      <c r="O37" s="69"/>
-      <c r="P37" s="69"/>
+    <row r="37" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D37" s="69"/>
+      <c r="E37" s="70"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="65"/>
+      <c r="H37" s="65"/>
+      <c r="I37" s="65"/>
+      <c r="J37" s="106"/>
+      <c r="K37" s="65"/>
+      <c r="L37" s="65"/>
+      <c r="M37" s="65"/>
+      <c r="N37" s="65"/>
+      <c r="O37" s="65"/>
+      <c r="P37" s="65"/>
       <c r="Q37" s="43"/>
       <c r="R37" s="43"/>
       <c r="S37" s="43"/>
@@ -3911,23 +4086,23 @@
       <c r="AG37" s="43"/>
       <c r="AH37" s="43"/>
       <c r="AI37" s="43"/>
-      <c r="AJ37" s="53"/>
+      <c r="AJ37" s="52"/>
       <c r="AK37" s="43"/>
     </row>
-    <row r="38" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="D38" s="68"/>
-      <c r="E38" s="68"/>
-      <c r="F38" s="68"/>
-      <c r="G38" s="68"/>
-      <c r="H38" s="68"/>
-      <c r="I38" s="68"/>
-      <c r="J38" s="68"/>
-      <c r="K38" s="75"/>
-      <c r="L38" s="69"/>
-      <c r="M38" s="76"/>
-      <c r="N38" s="69"/>
-      <c r="O38" s="69"/>
-      <c r="P38" s="77"/>
+    <row r="38" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D38" s="64"/>
+      <c r="E38" s="64"/>
+      <c r="F38" s="64"/>
+      <c r="G38" s="64"/>
+      <c r="H38" s="64"/>
+      <c r="I38" s="64"/>
+      <c r="J38" s="64"/>
+      <c r="K38" s="71"/>
+      <c r="L38" s="65"/>
+      <c r="M38" s="72"/>
+      <c r="N38" s="65"/>
+      <c r="O38" s="65"/>
+      <c r="P38" s="73"/>
       <c r="Q38" s="43"/>
       <c r="R38" s="43"/>
       <c r="S38" s="43"/>
@@ -3947,25 +4122,25 @@
       <c r="AG38" s="43"/>
       <c r="AH38" s="43"/>
       <c r="AI38" s="43"/>
-      <c r="AJ38" s="53"/>
+      <c r="AJ38" s="52"/>
       <c r="AK38" s="43"/>
     </row>
-    <row r="39" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A39" s="62"/>
-      <c r="C39" s="68"/>
-      <c r="D39" s="68"/>
-      <c r="E39" s="68"/>
-      <c r="F39" s="68"/>
-      <c r="G39" s="68"/>
-      <c r="H39" s="68"/>
-      <c r="I39" s="68"/>
-      <c r="J39" s="68"/>
-      <c r="K39" s="75"/>
-      <c r="L39" s="69"/>
-      <c r="M39" s="76"/>
-      <c r="N39" s="69"/>
-      <c r="O39" s="69"/>
-      <c r="P39" s="77"/>
+    <row r="39" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A39" s="60"/>
+      <c r="C39" s="64"/>
+      <c r="D39" s="64"/>
+      <c r="E39" s="64"/>
+      <c r="F39" s="64"/>
+      <c r="G39" s="64"/>
+      <c r="H39" s="64"/>
+      <c r="I39" s="64"/>
+      <c r="J39" s="64"/>
+      <c r="K39" s="71"/>
+      <c r="L39" s="65"/>
+      <c r="M39" s="72"/>
+      <c r="N39" s="65"/>
+      <c r="O39" s="65"/>
+      <c r="P39" s="73"/>
       <c r="Q39" s="43"/>
       <c r="R39" s="43"/>
       <c r="S39" s="43"/>
@@ -3985,25 +4160,25 @@
       <c r="AG39" s="43"/>
       <c r="AH39" s="43"/>
       <c r="AI39" s="43"/>
-      <c r="AJ39" s="53"/>
+      <c r="AJ39" s="52"/>
       <c r="AK39" s="43"/>
     </row>
-    <row r="40" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A40" s="62"/>
-      <c r="C40" s="68"/>
-      <c r="D40" s="68"/>
-      <c r="E40" s="68"/>
-      <c r="F40" s="68"/>
-      <c r="G40" s="68"/>
-      <c r="H40" s="68"/>
-      <c r="I40" s="68"/>
-      <c r="J40" s="68"/>
-      <c r="K40" s="71"/>
-      <c r="L40" s="69"/>
-      <c r="M40" s="76"/>
-      <c r="N40" s="69"/>
-      <c r="O40" s="69"/>
-      <c r="P40" s="77"/>
+    <row r="40" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A40" s="60"/>
+      <c r="C40" s="64"/>
+      <c r="D40" s="64"/>
+      <c r="E40" s="64"/>
+      <c r="F40" s="64"/>
+      <c r="G40" s="64"/>
+      <c r="H40" s="64"/>
+      <c r="I40" s="64"/>
+      <c r="J40" s="64"/>
+      <c r="K40" s="67"/>
+      <c r="L40" s="65"/>
+      <c r="M40" s="72"/>
+      <c r="N40" s="65"/>
+      <c r="O40" s="65"/>
+      <c r="P40" s="73"/>
       <c r="Q40" s="43"/>
       <c r="R40" s="43"/>
       <c r="S40" s="43"/>
@@ -4023,26 +4198,26 @@
       <c r="AG40" s="43"/>
       <c r="AH40" s="43"/>
       <c r="AI40" s="43"/>
-      <c r="AJ40" s="53"/>
+      <c r="AJ40" s="52"/>
       <c r="AK40" s="43"/>
     </row>
-    <row r="41" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A41" s="62"/>
-      <c r="B41" s="67"/>
-      <c r="C41" s="68"/>
-      <c r="D41" s="68"/>
-      <c r="E41" s="68"/>
-      <c r="F41" s="68"/>
-      <c r="G41" s="68"/>
-      <c r="H41" s="68"/>
-      <c r="I41" s="68"/>
-      <c r="J41" s="68"/>
-      <c r="K41" s="75"/>
-      <c r="L41" s="69"/>
-      <c r="M41" s="76"/>
-      <c r="N41" s="69"/>
-      <c r="O41" s="69"/>
-      <c r="P41" s="77"/>
+    <row r="41" spans="1:37" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A41" s="60"/>
+      <c r="B41" s="63"/>
+      <c r="C41" s="64"/>
+      <c r="D41" s="64"/>
+      <c r="E41" s="64"/>
+      <c r="F41" s="64"/>
+      <c r="G41" s="64"/>
+      <c r="H41" s="64"/>
+      <c r="I41" s="64"/>
+      <c r="J41" s="64"/>
+      <c r="K41" s="71"/>
+      <c r="L41" s="65"/>
+      <c r="M41" s="72"/>
+      <c r="N41" s="65"/>
+      <c r="O41" s="65"/>
+      <c r="P41" s="73"/>
       <c r="Q41" s="43"/>
       <c r="R41" s="43"/>
       <c r="S41" s="43"/>
@@ -4062,62 +4237,82 @@
       <c r="AG41" s="43"/>
       <c r="AH41" s="43"/>
       <c r="AI41" s="43"/>
-      <c r="AJ41" s="53"/>
+      <c r="AJ41" s="52"/>
       <c r="AK41" s="43"/>
     </row>
-    <row r="42" spans="1:37" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A42" s="63"/>
-      <c r="C42" s="68"/>
-      <c r="D42" s="68"/>
-      <c r="E42" s="68"/>
-      <c r="F42" s="68"/>
-      <c r="G42" s="68"/>
-      <c r="H42" s="68"/>
-      <c r="I42" s="68"/>
-      <c r="J42" s="68"/>
-      <c r="K42" s="72"/>
-      <c r="L42" s="69"/>
-      <c r="M42" s="76"/>
-      <c r="N42" s="69"/>
-      <c r="O42" s="69"/>
-      <c r="P42" s="77"/>
-      <c r="Q42" s="54"/>
-      <c r="R42" s="54"/>
-      <c r="S42" s="54"/>
-      <c r="T42" s="54"/>
-      <c r="U42" s="54"/>
-      <c r="V42" s="54"/>
-      <c r="W42" s="54"/>
-      <c r="X42" s="54"/>
-      <c r="Y42" s="54"/>
-      <c r="Z42" s="54"/>
-      <c r="AA42" s="54"/>
-      <c r="AB42" s="54"/>
-      <c r="AC42" s="54"/>
-      <c r="AD42" s="54"/>
-      <c r="AE42" s="54"/>
-      <c r="AF42" s="54"/>
-      <c r="AG42" s="54"/>
-      <c r="AH42" s="54"/>
-      <c r="AI42" s="54"/>
-      <c r="AJ42" s="55"/>
+    <row r="42" spans="1:37" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A42" s="61"/>
+      <c r="C42" s="64"/>
+      <c r="D42" s="64"/>
+      <c r="E42" s="64"/>
+      <c r="F42" s="64"/>
+      <c r="G42" s="64"/>
+      <c r="H42" s="64"/>
+      <c r="I42" s="64"/>
+      <c r="J42" s="64"/>
+      <c r="K42" s="68"/>
+      <c r="L42" s="65"/>
+      <c r="M42" s="72"/>
+      <c r="N42" s="65"/>
+      <c r="O42" s="65"/>
+      <c r="P42" s="73"/>
+      <c r="Q42" s="53"/>
+      <c r="R42" s="53"/>
+      <c r="S42" s="53"/>
+      <c r="T42" s="53"/>
+      <c r="U42" s="53"/>
+      <c r="V42" s="53"/>
+      <c r="W42" s="53"/>
+      <c r="X42" s="53"/>
+      <c r="Y42" s="53"/>
+      <c r="Z42" s="53"/>
+      <c r="AA42" s="53"/>
+      <c r="AB42" s="53"/>
+      <c r="AC42" s="53"/>
+      <c r="AD42" s="53"/>
+      <c r="AE42" s="53"/>
+      <c r="AF42" s="53"/>
+      <c r="AG42" s="53"/>
+      <c r="AH42" s="53"/>
+      <c r="AI42" s="53"/>
+      <c r="AJ42" s="54"/>
       <c r="AK42" s="43"/>
     </row>
   </sheetData>
-  <mergeCells count="55">
-    <mergeCell ref="AE1:AF1"/>
-    <mergeCell ref="AE2:AF2"/>
-    <mergeCell ref="AC5:AJ5"/>
-    <mergeCell ref="AC4:AJ4"/>
-    <mergeCell ref="F5:J5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="Q4:AB4"/>
-    <mergeCell ref="Q5:AB5"/>
-    <mergeCell ref="A1:AD2"/>
-    <mergeCell ref="M5:P5"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:P4"/>
-    <mergeCell ref="A3:E5"/>
+  <mergeCells count="62">
+    <mergeCell ref="A7:A17"/>
+    <mergeCell ref="A18:A25"/>
+    <mergeCell ref="C11:J12"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="J32:J33"/>
+    <mergeCell ref="J36:J37"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="B7:B15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="B18:B22"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="C18:C25"/>
+    <mergeCell ref="AA31:AB31"/>
+    <mergeCell ref="AA30:AB30"/>
+    <mergeCell ref="AA27:AB27"/>
+    <mergeCell ref="AA28:AB28"/>
+    <mergeCell ref="F3:J4"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="Q31:R31"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="Q28:R28"/>
+    <mergeCell ref="Q29:R29"/>
+    <mergeCell ref="U19:U20"/>
+    <mergeCell ref="Z16:Z17"/>
+    <mergeCell ref="U16:U17"/>
+    <mergeCell ref="AD16:AD17"/>
+    <mergeCell ref="AC16:AC17"/>
+    <mergeCell ref="Q30:R30"/>
+    <mergeCell ref="AA29:AB29"/>
+    <mergeCell ref="V16:V17"/>
+    <mergeCell ref="AA16:AA17"/>
     <mergeCell ref="Q16:Q17"/>
     <mergeCell ref="R16:R17"/>
     <mergeCell ref="AB16:AB17"/>
@@ -4134,32 +4329,19 @@
     <mergeCell ref="W16:W17"/>
     <mergeCell ref="X16:X17"/>
     <mergeCell ref="Y16:Y17"/>
-    <mergeCell ref="Z16:Z17"/>
-    <mergeCell ref="U16:U17"/>
-    <mergeCell ref="AD16:AD17"/>
-    <mergeCell ref="AC16:AC17"/>
-    <mergeCell ref="Q30:R30"/>
-    <mergeCell ref="Q31:R31"/>
-    <mergeCell ref="Q27:R27"/>
-    <mergeCell ref="Q28:R28"/>
-    <mergeCell ref="Q29:R29"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="AA29:AB29"/>
-    <mergeCell ref="V16:V17"/>
-    <mergeCell ref="AA16:AA17"/>
-    <mergeCell ref="AA31:AB31"/>
-    <mergeCell ref="AA30:AB30"/>
-    <mergeCell ref="AA27:AB27"/>
-    <mergeCell ref="AA28:AB28"/>
-    <mergeCell ref="F3:J4"/>
-    <mergeCell ref="K3:P3"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="J32:J33"/>
-    <mergeCell ref="J36:J37"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="B7:B13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="A7:A15"/>
+    <mergeCell ref="AE1:AF1"/>
+    <mergeCell ref="AE2:AF2"/>
+    <mergeCell ref="AC5:AJ5"/>
+    <mergeCell ref="AC4:AJ4"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="Q4:AB4"/>
+    <mergeCell ref="Q5:AB5"/>
+    <mergeCell ref="M5:P5"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:P4"/>
+    <mergeCell ref="A3:E5"/>
+    <mergeCell ref="A1:L2"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4173,109 +4355,109 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P17"/>
-  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.375" customWidth="1"/>
-    <col min="2" max="2" width="15.875" customWidth="1"/>
-    <col min="3" max="3" width="6.375" customWidth="1"/>
-    <col min="4" max="4" width="26.875" customWidth="1"/>
-    <col min="5" max="5" width="7.125" customWidth="1"/>
-    <col min="6" max="6" width="22.625" customWidth="1"/>
-    <col min="7" max="7" width="9.375" customWidth="1"/>
-    <col min="8" max="8" width="21.6875" customWidth="1"/>
+    <col min="1" max="1" width="11.3984375" customWidth="1"/>
+    <col min="2" max="2" width="15.8984375" customWidth="1"/>
+    <col min="3" max="3" width="6.3984375" customWidth="1"/>
+    <col min="4" max="4" width="26.8984375" customWidth="1"/>
+    <col min="5" max="5" width="7.09765625" customWidth="1"/>
+    <col min="6" max="6" width="22.59765625" customWidth="1"/>
+    <col min="7" max="7" width="9.3984375" customWidth="1"/>
+    <col min="8" max="8" width="21.69921875" customWidth="1"/>
     <col min="9" max="9" width="6" customWidth="1"/>
-    <col min="10" max="10" width="16.375" customWidth="1"/>
+    <col min="10" max="10" width="16.3984375" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="5.6875" customWidth="1"/>
-    <col min="13" max="13" width="13.875" customWidth="1"/>
-    <col min="14" max="14" width="11.1875" customWidth="1"/>
-    <col min="15" max="16" width="12.875" customWidth="1"/>
+    <col min="12" max="12" width="5.69921875" customWidth="1"/>
+    <col min="13" max="13" width="13.8984375" customWidth="1"/>
+    <col min="14" max="14" width="11.19921875" customWidth="1"/>
+    <col min="15" max="16" width="12.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="136" t="s">
+    <row r="1" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="128" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="137"/>
-      <c r="C1" s="137"/>
-      <c r="D1" s="137"/>
-      <c r="E1" s="137"/>
-      <c r="F1" s="137"/>
-      <c r="G1" s="137"/>
-      <c r="H1" s="137"/>
-      <c r="I1" s="137"/>
-      <c r="J1" s="137"/>
-      <c r="K1" s="137"/>
-      <c r="L1" s="137"/>
-      <c r="M1" s="110" t="s">
+      <c r="B1" s="129"/>
+      <c r="C1" s="129"/>
+      <c r="D1" s="129"/>
+      <c r="E1" s="129"/>
+      <c r="F1" s="129"/>
+      <c r="G1" s="129"/>
+      <c r="H1" s="129"/>
+      <c r="I1" s="129"/>
+      <c r="J1" s="129"/>
+      <c r="K1" s="129"/>
+      <c r="L1" s="129"/>
+      <c r="M1" s="77" t="s">
         <v>49</v>
       </c>
-      <c r="N1" s="110"/>
-      <c r="O1" s="110" t="s">
+      <c r="N1" s="77"/>
+      <c r="O1" s="77" t="s">
         <v>51</v>
       </c>
-      <c r="P1" s="134"/>
-    </row>
-    <row r="2" spans="1:16" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A2" s="138"/>
-      <c r="B2" s="139"/>
-      <c r="C2" s="139"/>
-      <c r="D2" s="139"/>
-      <c r="E2" s="139"/>
-      <c r="F2" s="139"/>
-      <c r="G2" s="139"/>
-      <c r="H2" s="139"/>
-      <c r="I2" s="139"/>
-      <c r="J2" s="139"/>
-      <c r="K2" s="139"/>
-      <c r="L2" s="139"/>
-      <c r="M2" s="111" t="s">
+      <c r="P1" s="126"/>
+    </row>
+    <row r="2" spans="1:16" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="130"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="131"/>
+      <c r="D2" s="131"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="131"/>
+      <c r="G2" s="131"/>
+      <c r="H2" s="131"/>
+      <c r="I2" s="131"/>
+      <c r="J2" s="131"/>
+      <c r="K2" s="131"/>
+      <c r="L2" s="131"/>
+      <c r="M2" s="78" t="s">
         <v>50</v>
       </c>
-      <c r="N2" s="111"/>
-      <c r="O2" s="111"/>
-      <c r="P2" s="135"/>
-    </row>
-    <row r="3" spans="1:16" ht="17.25" thickBot="1" x14ac:dyDescent="0.65"/>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.6">
-      <c r="A4" s="140" t="s">
+      <c r="N2" s="78"/>
+      <c r="O2" s="78"/>
+      <c r="P2" s="127"/>
+    </row>
+    <row r="3" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.45"/>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A4" s="132" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="141"/>
-      <c r="C4" s="141"/>
-      <c r="D4" s="142"/>
-      <c r="E4" s="143" t="s">
+      <c r="B4" s="133"/>
+      <c r="C4" s="133"/>
+      <c r="D4" s="134"/>
+      <c r="E4" s="135" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="142"/>
-      <c r="G4" s="143" t="s">
+      <c r="F4" s="134"/>
+      <c r="G4" s="135" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="142"/>
-      <c r="I4" s="143" t="s">
+      <c r="H4" s="134"/>
+      <c r="I4" s="135" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="142"/>
-      <c r="K4" s="143" t="s">
+      <c r="J4" s="134"/>
+      <c r="K4" s="135" t="s">
         <v>26</v>
       </c>
-      <c r="L4" s="142"/>
+      <c r="L4" s="134"/>
       <c r="M4" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="143" t="s">
+      <c r="N4" s="135" t="s">
         <v>28</v>
       </c>
-      <c r="O4" s="142"/>
-      <c r="P4" s="125" t="s">
+      <c r="O4" s="134"/>
+      <c r="P4" s="117" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A5" s="127" t="s">
+    <row r="5" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="119" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="128"/>
+      <c r="B5" s="120"/>
       <c r="C5" s="15" t="s">
         <v>0</v>
       </c>
@@ -4315,10 +4497,10 @@
       <c r="O5" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="P5" s="126"/>
-    </row>
-    <row r="6" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="129" t="s">
+      <c r="P5" s="118"/>
+    </row>
+    <row r="6" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="121" t="s">
         <v>36</v>
       </c>
       <c r="B6" s="11" t="s">
@@ -4347,9 +4529,9 @@
       <c r="O6" s="5"/>
       <c r="P6" s="6"/>
     </row>
-    <row r="7" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="129"/>
-      <c r="B7" s="144" t="s">
+    <row r="7" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="121"/>
+      <c r="B7" s="114" t="s">
         <v>53</v>
       </c>
       <c r="C7" s="5" t="s">
@@ -4358,47 +4540,47 @@
       <c r="D7" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="146"/>
-      <c r="F7" s="146"/>
-      <c r="G7" s="148" t="s">
+      <c r="E7" s="110"/>
+      <c r="F7" s="110"/>
+      <c r="G7" s="116" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="144" t="s">
+      <c r="H7" s="114" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="146"/>
-      <c r="J7" s="146"/>
-      <c r="K7" s="146"/>
-      <c r="L7" s="146"/>
-      <c r="M7" s="146"/>
-      <c r="N7" s="146"/>
-      <c r="O7" s="146"/>
-      <c r="P7" s="149"/>
-    </row>
-    <row r="8" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="130"/>
-      <c r="B8" s="145"/>
+      <c r="I7" s="110"/>
+      <c r="J7" s="110"/>
+      <c r="K7" s="110"/>
+      <c r="L7" s="110"/>
+      <c r="M7" s="110"/>
+      <c r="N7" s="110"/>
+      <c r="O7" s="110"/>
+      <c r="P7" s="108"/>
+    </row>
+    <row r="8" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="122"/>
+      <c r="B8" s="115"/>
       <c r="C8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="147"/>
-      <c r="F8" s="147"/>
-      <c r="G8" s="148"/>
-      <c r="H8" s="145"/>
-      <c r="I8" s="147"/>
-      <c r="J8" s="147"/>
-      <c r="K8" s="147"/>
-      <c r="L8" s="147"/>
-      <c r="M8" s="147"/>
-      <c r="N8" s="147"/>
-      <c r="O8" s="147"/>
-      <c r="P8" s="150"/>
-    </row>
-    <row r="9" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="130"/>
+      <c r="E8" s="111"/>
+      <c r="F8" s="111"/>
+      <c r="G8" s="116"/>
+      <c r="H8" s="115"/>
+      <c r="I8" s="111"/>
+      <c r="J8" s="111"/>
+      <c r="K8" s="111"/>
+      <c r="L8" s="111"/>
+      <c r="M8" s="111"/>
+      <c r="N8" s="111"/>
+      <c r="O8" s="111"/>
+      <c r="P8" s="109"/>
+    </row>
+    <row r="9" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="122"/>
       <c r="B9" s="16" t="s">
         <v>54</v>
       </c>
@@ -4425,9 +4607,9 @@
       <c r="O9" s="1"/>
       <c r="P9" s="2"/>
     </row>
-    <row r="10" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="130"/>
-      <c r="B10" s="144" t="s">
+    <row r="10" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="122"/>
+      <c r="B10" s="114" t="s">
         <v>56</v>
       </c>
       <c r="C10" s="9" t="s">
@@ -4436,47 +4618,47 @@
       <c r="D10" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="146"/>
-      <c r="F10" s="146"/>
-      <c r="G10" s="151" t="s">
+      <c r="E10" s="110"/>
+      <c r="F10" s="110"/>
+      <c r="G10" s="112" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="144" t="s">
+      <c r="H10" s="114" t="s">
         <v>41</v>
       </c>
-      <c r="I10" s="146"/>
-      <c r="J10" s="146"/>
-      <c r="K10" s="146"/>
-      <c r="L10" s="146"/>
-      <c r="M10" s="146"/>
-      <c r="N10" s="146"/>
-      <c r="O10" s="146"/>
-      <c r="P10" s="149"/>
-    </row>
-    <row r="11" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="130"/>
-      <c r="B11" s="145"/>
+      <c r="I10" s="110"/>
+      <c r="J10" s="110"/>
+      <c r="K10" s="110"/>
+      <c r="L10" s="110"/>
+      <c r="M10" s="110"/>
+      <c r="N10" s="110"/>
+      <c r="O10" s="110"/>
+      <c r="P10" s="108"/>
+    </row>
+    <row r="11" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="122"/>
+      <c r="B11" s="115"/>
       <c r="C11" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="147"/>
-      <c r="F11" s="147"/>
-      <c r="G11" s="152"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="147"/>
-      <c r="J11" s="147"/>
-      <c r="K11" s="147"/>
-      <c r="L11" s="147"/>
-      <c r="M11" s="147"/>
-      <c r="N11" s="147"/>
-      <c r="O11" s="147"/>
-      <c r="P11" s="150"/>
-    </row>
-    <row r="12" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A12" s="130"/>
+      <c r="E11" s="111"/>
+      <c r="F11" s="111"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="115"/>
+      <c r="I11" s="111"/>
+      <c r="J11" s="111"/>
+      <c r="K11" s="111"/>
+      <c r="L11" s="111"/>
+      <c r="M11" s="111"/>
+      <c r="N11" s="111"/>
+      <c r="O11" s="111"/>
+      <c r="P11" s="109"/>
+    </row>
+    <row r="12" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="122"/>
       <c r="B12" s="12" t="s">
         <v>55</v>
       </c>
@@ -4503,8 +4685,8 @@
       <c r="O12" s="1"/>
       <c r="P12" s="2"/>
     </row>
-    <row r="13" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A13" s="131"/>
+    <row r="13" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="123"/>
       <c r="B13" s="12" t="s">
         <v>57</v>
       </c>
@@ -4531,8 +4713,8 @@
       <c r="O13" s="1"/>
       <c r="P13" s="2"/>
     </row>
-    <row r="14" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A14" s="132" t="s">
+    <row r="14" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="124" t="s">
         <v>37</v>
       </c>
       <c r="B14" s="12" t="s">
@@ -4561,8 +4743,8 @@
       <c r="O14" s="1"/>
       <c r="P14" s="2"/>
     </row>
-    <row r="15" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A15" s="130"/>
+    <row r="15" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="122"/>
       <c r="B15" s="12" t="s">
         <v>58</v>
       </c>
@@ -4589,8 +4771,8 @@
       <c r="O15" s="1"/>
       <c r="P15" s="2"/>
     </row>
-    <row r="16" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A16" s="130"/>
+    <row r="16" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="122"/>
       <c r="B16" s="12" t="s">
         <v>60</v>
       </c>
@@ -4617,8 +4799,8 @@
       <c r="O16" s="1"/>
       <c r="P16" s="2"/>
     </row>
-    <row r="17" spans="1:16" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A17" s="133"/>
+    <row r="17" spans="1:16" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="125"/>
       <c r="B17" s="13" t="s">
         <v>61</v>
       </c>
@@ -4647,6 +4829,31 @@
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="P4:P5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A6:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="J7:J8"/>
     <mergeCell ref="P7:P8"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="F7:F8"/>
@@ -4663,31 +4870,6 @@
     <mergeCell ref="N10:N11"/>
     <mergeCell ref="O10:O11"/>
     <mergeCell ref="K7:K8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="O7:O8"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="P4:P5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="O1:P1"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="A1:L2"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="B7:B8"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
AM (bce-01, sqd-01 수정), RTM (설계 bce 식별자 추가), Uml (설계 BCE/C;ass diagram 작성
</commit_message>
<xml_diff>
--- a/Document/요구사항추적표(RTM).xlsx
+++ b/Document/요구사항추적표(RTM).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rlaal\Documents\FalshTalk\Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A04F7A0F-A12A-4D2A-8909-F9E8977575C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07974FE4-73F4-4F6A-863B-3A32B2866D1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="230">
   <si>
     <t>번호</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -410,20 +410,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>분석 모델링
-(AM)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>설계단계</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>설계 기술서
-(SDD)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>서브시스템</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -854,6 +840,75 @@
   </si>
   <si>
     <t>SQD-04</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>회원 탈퇴</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SQD-07</t>
+  </si>
+  <si>
+    <t>SMD-01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SMD-02</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SMD-03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SMD-04</t>
+  </si>
+  <si>
+    <t>SMD-06</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SMD-05</t>
+  </si>
+  <si>
+    <t>SMD-05</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>시스템 설계</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>설계기술서 (SDD)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>설계 BCE</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRD-01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRD-02</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRD-03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRD-04</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRD-06</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRD-05</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1011,7 +1066,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="48">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -1361,21 +1416,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color auto="1"/>
@@ -1428,19 +1468,6 @@
       <right/>
       <top style="thin">
         <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
       </top>
       <bottom style="thin">
         <color auto="1"/>
@@ -1570,18 +1597,20 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color auto="1"/>
+      <right style="medium">
+        <color indexed="64"/>
       </right>
       <top/>
-      <bottom/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -1596,7 +1625,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="179">
+  <cellXfs count="159">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1680,7 +1709,7 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1695,16 +1724,13 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1723,29 +1749,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1758,10 +1771,7 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1819,41 +1829,94 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="45" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1864,133 +1927,148 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="42" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="41" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1999,121 +2077,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="42" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="47" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="46" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="41" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2425,7 +2392,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AL42"/>
+  <dimension ref="A1:AQ42"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="11.5" customWidth="1"/>
@@ -2440,7 +2407,7 @@
     <col min="10" max="10" width="20.19921875" customWidth="1"/>
     <col min="11" max="11" width="12.59765625" style="23" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="35.59765625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.19921875" customWidth="1"/>
+    <col min="13" max="13" width="23.59765625" customWidth="1"/>
     <col min="14" max="14" width="18.796875" customWidth="1"/>
     <col min="15" max="15" width="15" customWidth="1"/>
     <col min="16" max="16" width="24.09765625" customWidth="1"/>
@@ -2462,223 +2429,255 @@
     <col min="35" max="35" width="21.09765625" hidden="1" customWidth="1"/>
     <col min="36" max="36" width="24.59765625" hidden="1" customWidth="1"/>
     <col min="37" max="37" width="8.59765625" hidden="1" customWidth="1"/>
-    <col min="38" max="38" width="13.296875" customWidth="1"/>
+    <col min="38" max="38" width="11.19921875" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="0" hidden="1" customWidth="1"/>
+    <col min="40" max="40" width="15" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="14.8984375" customWidth="1"/>
+    <col min="43" max="43" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="86" t="s">
-        <v>109</v>
-      </c>
-      <c r="B1" s="87"/>
-      <c r="C1" s="87"/>
-      <c r="D1" s="87"/>
-      <c r="E1" s="87"/>
-      <c r="F1" s="87"/>
-      <c r="G1" s="87"/>
-      <c r="H1" s="87"/>
-      <c r="I1" s="87"/>
-      <c r="J1" s="87"/>
-      <c r="K1" s="87"/>
-      <c r="L1" s="87"/>
-      <c r="M1" s="87"/>
-      <c r="N1" s="87"/>
-      <c r="O1" s="87"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="77"/>
-      <c r="R1" s="77"/>
-      <c r="S1" s="77"/>
-      <c r="T1" s="77"/>
-      <c r="U1" s="77"/>
-      <c r="V1" s="77"/>
-      <c r="W1" s="77"/>
-      <c r="X1" s="77"/>
-      <c r="Y1" s="77"/>
-      <c r="Z1" s="77"/>
-      <c r="AA1" s="77"/>
-      <c r="AB1" s="77"/>
-      <c r="AC1" s="77"/>
-      <c r="AD1" s="77"/>
-      <c r="AE1" s="92"/>
-      <c r="AF1" s="92"/>
+    <row r="1" spans="1:43" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="109" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="110"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="111"/>
+      <c r="Q1" s="70"/>
+      <c r="R1" s="70"/>
+      <c r="S1" s="70"/>
+      <c r="T1" s="70"/>
+      <c r="U1" s="70"/>
+      <c r="V1" s="70"/>
+      <c r="W1" s="70"/>
+      <c r="X1" s="70"/>
+      <c r="Y1" s="70"/>
+      <c r="Z1" s="70"/>
+      <c r="AA1" s="70"/>
+      <c r="AB1" s="70"/>
+      <c r="AC1" s="70"/>
+      <c r="AD1" s="70"/>
+      <c r="AE1" s="104"/>
+      <c r="AF1" s="104"/>
       <c r="AG1" s="19"/>
       <c r="AH1" s="19"/>
       <c r="AI1" s="19"/>
       <c r="AJ1" s="20"/>
       <c r="AK1" s="20"/>
-      <c r="AL1" s="79"/>
-    </row>
-    <row r="2" spans="1:38" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="89"/>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="90"/>
-      <c r="H2" s="90"/>
-      <c r="I2" s="90"/>
-      <c r="J2" s="90"/>
-      <c r="K2" s="90"/>
-      <c r="L2" s="90"/>
-      <c r="M2" s="90"/>
-      <c r="N2" s="90"/>
-      <c r="O2" s="90"/>
-      <c r="P2" s="91"/>
-      <c r="Q2" s="78"/>
-      <c r="R2" s="78"/>
-      <c r="S2" s="78"/>
-      <c r="T2" s="78"/>
-      <c r="U2" s="78"/>
-      <c r="V2" s="78"/>
-      <c r="W2" s="78"/>
-      <c r="X2" s="78"/>
-      <c r="Y2" s="78"/>
-      <c r="Z2" s="78"/>
-      <c r="AA2" s="78"/>
-      <c r="AB2" s="78"/>
-      <c r="AC2" s="78"/>
-      <c r="AD2" s="78"/>
-      <c r="AE2" s="93"/>
-      <c r="AF2" s="93"/>
+      <c r="AL1" s="72"/>
+    </row>
+    <row r="2" spans="1:43" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="112"/>
+      <c r="B2" s="113"/>
+      <c r="C2" s="113"/>
+      <c r="D2" s="113"/>
+      <c r="E2" s="113"/>
+      <c r="F2" s="113"/>
+      <c r="G2" s="113"/>
+      <c r="H2" s="113"/>
+      <c r="I2" s="113"/>
+      <c r="J2" s="113"/>
+      <c r="K2" s="113"/>
+      <c r="L2" s="113"/>
+      <c r="M2" s="113"/>
+      <c r="N2" s="113"/>
+      <c r="O2" s="113"/>
+      <c r="P2" s="114"/>
+      <c r="Q2" s="71"/>
+      <c r="R2" s="71"/>
+      <c r="S2" s="71"/>
+      <c r="T2" s="71"/>
+      <c r="U2" s="71"/>
+      <c r="V2" s="71"/>
+      <c r="W2" s="71"/>
+      <c r="X2" s="71"/>
+      <c r="Y2" s="71"/>
+      <c r="Z2" s="71"/>
+      <c r="AA2" s="71"/>
+      <c r="AB2" s="71"/>
+      <c r="AC2" s="71"/>
+      <c r="AD2" s="71"/>
+      <c r="AE2" s="105"/>
+      <c r="AF2" s="105"/>
       <c r="AG2" s="21"/>
       <c r="AH2" s="21"/>
       <c r="AI2" s="21"/>
       <c r="AJ2" s="22"/>
       <c r="AK2" s="22"/>
-      <c r="AL2" s="79"/>
-    </row>
-    <row r="3" spans="1:38" ht="18" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="82" t="s">
+      <c r="AL2" s="72"/>
+    </row>
+    <row r="3" spans="1:43" x14ac:dyDescent="0.4">
+      <c r="A3" s="96" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="96"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96" t="s">
         <v>108</v>
       </c>
-      <c r="B3" s="82"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="82"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="82" t="s">
-        <v>111</v>
-      </c>
-      <c r="G3" s="82"/>
-      <c r="H3" s="82"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="82"/>
-      <c r="K3" s="83" t="s">
-        <v>112</v>
-      </c>
-      <c r="L3" s="84"/>
-      <c r="M3" s="84"/>
-      <c r="N3" s="84"/>
-      <c r="O3" s="84"/>
-      <c r="P3" s="85"/>
-      <c r="AJ3" s="48"/>
-    </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.4">
-      <c r="A4" s="82"/>
-      <c r="B4" s="82"/>
-      <c r="C4" s="82"/>
-      <c r="D4" s="82"/>
-      <c r="E4" s="82"/>
-      <c r="F4" s="82"/>
-      <c r="G4" s="82"/>
-      <c r="H4" s="82"/>
-      <c r="I4" s="82"/>
-      <c r="J4" s="82"/>
-      <c r="K4" s="103" t="s">
+      <c r="G3" s="96"/>
+      <c r="H3" s="96"/>
+      <c r="I3" s="96"/>
+      <c r="J3" s="96"/>
+      <c r="K3" s="124" t="s">
+        <v>109</v>
+      </c>
+      <c r="L3" s="125"/>
+      <c r="M3" s="125"/>
+      <c r="N3" s="125"/>
+      <c r="O3" s="125"/>
+      <c r="P3" s="125"/>
+      <c r="Q3" s="125"/>
+      <c r="R3" s="125"/>
+      <c r="S3" s="125"/>
+      <c r="T3" s="125"/>
+      <c r="U3" s="125"/>
+      <c r="V3" s="125"/>
+      <c r="W3" s="125"/>
+      <c r="X3" s="125"/>
+      <c r="Y3" s="125"/>
+      <c r="Z3" s="125"/>
+      <c r="AA3" s="125"/>
+      <c r="AB3" s="125"/>
+      <c r="AC3" s="125"/>
+      <c r="AD3" s="125"/>
+      <c r="AE3" s="125"/>
+      <c r="AF3" s="125"/>
+      <c r="AG3" s="125"/>
+      <c r="AH3" s="125"/>
+      <c r="AI3" s="125"/>
+      <c r="AJ3" s="125"/>
+      <c r="AK3" s="125"/>
+      <c r="AL3" s="125"/>
+      <c r="AM3" s="125"/>
+      <c r="AN3" s="125"/>
+      <c r="AO3" s="125"/>
+      <c r="AP3" s="125"/>
+    </row>
+    <row r="4" spans="1:43" x14ac:dyDescent="0.4">
+      <c r="A4" s="96"/>
+      <c r="B4" s="96"/>
+      <c r="C4" s="96"/>
+      <c r="D4" s="96"/>
+      <c r="E4" s="96"/>
+      <c r="F4" s="96"/>
+      <c r="G4" s="96"/>
+      <c r="H4" s="96"/>
+      <c r="I4" s="96"/>
+      <c r="J4" s="96"/>
+      <c r="K4" s="107" t="s">
         <v>80</v>
       </c>
-      <c r="L4" s="103"/>
-      <c r="M4" s="103" t="s">
+      <c r="L4" s="107"/>
+      <c r="M4" s="96" t="s">
         <v>79</v>
       </c>
-      <c r="N4" s="103"/>
-      <c r="O4" s="103"/>
-      <c r="P4" s="104"/>
-      <c r="Q4" s="99" t="s">
-        <v>79</v>
-      </c>
-      <c r="R4" s="100"/>
-      <c r="S4" s="100"/>
-      <c r="T4" s="100"/>
-      <c r="U4" s="100"/>
-      <c r="V4" s="100"/>
-      <c r="W4" s="100"/>
-      <c r="X4" s="100"/>
-      <c r="Y4" s="100"/>
-      <c r="Z4" s="100"/>
-      <c r="AA4" s="100"/>
-      <c r="AB4" s="100"/>
-      <c r="AC4" s="96" t="s">
-        <v>93</v>
-      </c>
+      <c r="N4" s="96"/>
+      <c r="O4" s="96"/>
+      <c r="P4" s="96"/>
+      <c r="Q4" s="96"/>
+      <c r="R4" s="96"/>
+      <c r="S4" s="96"/>
+      <c r="T4" s="96"/>
+      <c r="U4" s="96"/>
+      <c r="V4" s="96"/>
+      <c r="W4" s="96"/>
+      <c r="X4" s="96"/>
+      <c r="Y4" s="96"/>
+      <c r="Z4" s="96"/>
+      <c r="AA4" s="96"/>
+      <c r="AB4" s="96"/>
+      <c r="AC4" s="96"/>
       <c r="AD4" s="96"/>
       <c r="AE4" s="96"/>
       <c r="AF4" s="96"/>
       <c r="AG4" s="96"/>
       <c r="AH4" s="96"/>
       <c r="AI4" s="96"/>
-      <c r="AJ4" s="97"/>
-      <c r="AK4" s="107" t="s">
-        <v>8</v>
-      </c>
-      <c r="AL4" s="80"/>
-    </row>
-    <row r="5" spans="1:38" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="82"/>
-      <c r="B5" s="82"/>
-      <c r="C5" s="82"/>
-      <c r="D5" s="82"/>
-      <c r="E5" s="82"/>
-      <c r="F5" s="98" t="s">
+      <c r="AJ4" s="96"/>
+      <c r="AK4" s="96"/>
+      <c r="AL4" s="96"/>
+      <c r="AM4" s="96"/>
+      <c r="AN4" s="96"/>
+      <c r="AO4" s="96"/>
+      <c r="AP4" s="96"/>
+      <c r="AQ4" s="83" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="96"/>
+      <c r="B5" s="96"/>
+      <c r="C5" s="96"/>
+      <c r="D5" s="96"/>
+      <c r="E5" s="96"/>
+      <c r="F5" s="87" t="s">
+        <v>104</v>
+      </c>
+      <c r="G5" s="106"/>
+      <c r="H5" s="106"/>
+      <c r="I5" s="106"/>
+      <c r="J5" s="106"/>
+      <c r="K5" s="106" t="s">
+        <v>103</v>
+      </c>
+      <c r="L5" s="102"/>
+      <c r="M5" s="106" t="s">
         <v>107</v>
       </c>
-      <c r="G5" s="94"/>
-      <c r="H5" s="94"/>
-      <c r="I5" s="94"/>
-      <c r="J5" s="94"/>
-      <c r="K5" s="94" t="s">
-        <v>106</v>
-      </c>
-      <c r="L5" s="94"/>
-      <c r="M5" s="101" t="s">
-        <v>110</v>
-      </c>
-      <c r="N5" s="102"/>
-      <c r="O5" s="102"/>
-      <c r="P5" s="98"/>
-      <c r="Q5" s="98" t="s">
-        <v>92</v>
-      </c>
-      <c r="R5" s="94"/>
-      <c r="S5" s="94"/>
-      <c r="T5" s="94"/>
-      <c r="U5" s="94"/>
-      <c r="V5" s="94"/>
-      <c r="W5" s="94"/>
-      <c r="X5" s="94"/>
-      <c r="Y5" s="94"/>
-      <c r="Z5" s="94"/>
-      <c r="AA5" s="94"/>
-      <c r="AB5" s="94"/>
-      <c r="AC5" s="94" t="s">
-        <v>94</v>
-      </c>
-      <c r="AD5" s="94"/>
-      <c r="AE5" s="94"/>
-      <c r="AF5" s="94"/>
-      <c r="AG5" s="94"/>
-      <c r="AH5" s="94"/>
-      <c r="AI5" s="94"/>
-      <c r="AJ5" s="95"/>
-      <c r="AK5" s="108"/>
-      <c r="AL5" s="80"/>
-    </row>
-    <row r="6" spans="1:38" ht="34.799999999999997" x14ac:dyDescent="0.4">
-      <c r="A6" s="121" t="s">
+      <c r="N5" s="106"/>
+      <c r="O5" s="106"/>
+      <c r="P5" s="106"/>
+      <c r="Q5" s="106"/>
+      <c r="R5" s="106"/>
+      <c r="S5" s="106"/>
+      <c r="T5" s="106"/>
+      <c r="U5" s="106"/>
+      <c r="V5" s="106"/>
+      <c r="W5" s="106"/>
+      <c r="X5" s="106"/>
+      <c r="Y5" s="106"/>
+      <c r="Z5" s="106"/>
+      <c r="AA5" s="106"/>
+      <c r="AB5" s="106"/>
+      <c r="AC5" s="106"/>
+      <c r="AD5" s="106"/>
+      <c r="AE5" s="106"/>
+      <c r="AF5" s="106"/>
+      <c r="AG5" s="106"/>
+      <c r="AH5" s="106"/>
+      <c r="AI5" s="106"/>
+      <c r="AJ5" s="106"/>
+      <c r="AK5" s="106"/>
+      <c r="AL5" s="106"/>
+      <c r="AM5" s="106"/>
+      <c r="AN5" s="106"/>
+      <c r="AO5" s="106"/>
+      <c r="AP5" s="106"/>
+      <c r="AQ5" s="83" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="6" spans="1:43" ht="34.799999999999997" x14ac:dyDescent="0.4">
+      <c r="A6" s="85" t="s">
         <v>76</v>
       </c>
-      <c r="B6" s="102"/>
-      <c r="C6" s="98"/>
+      <c r="B6" s="86"/>
+      <c r="C6" s="87"/>
       <c r="D6" s="26" t="s">
         <v>0</v>
       </c>
@@ -2688,14 +2687,14 @@
       <c r="F6" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="G6" s="58" t="s">
+      <c r="G6" s="52" t="s">
         <v>91</v>
       </c>
-      <c r="H6" s="58" t="s">
-        <v>165</v>
+      <c r="H6" s="52" t="s">
+        <v>162</v>
       </c>
       <c r="I6" s="26" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="J6" s="26" t="s">
         <v>81</v>
@@ -2703,14 +2702,14 @@
       <c r="K6" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="L6" s="58" t="s">
+      <c r="L6" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="M6" s="101" t="s">
+      <c r="M6" s="102" t="s">
         <v>83</v>
       </c>
-      <c r="N6" s="102"/>
-      <c r="O6" s="98"/>
+      <c r="N6" s="86"/>
+      <c r="O6" s="87"/>
       <c r="P6" s="27" t="s">
         <v>87</v>
       </c>
@@ -2754,77 +2753,90 @@
         <v>2</v>
       </c>
       <c r="AD6" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE6" s="26" t="s">
+        <v>93</v>
+      </c>
+      <c r="AF6" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="AG6" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="AE6" s="26" t="s">
+      <c r="AH6" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="AF6" s="27" t="s">
+      <c r="AI6" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="AG6" s="27" t="s">
+      <c r="AJ6" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="AH6" s="27" t="s">
-        <v>99</v>
-      </c>
-      <c r="AI6" s="26" t="s">
-        <v>100</v>
-      </c>
-      <c r="AJ6" s="28" t="s">
-        <v>101</v>
-      </c>
-      <c r="AK6" s="108"/>
+      <c r="AK6" s="81"/>
       <c r="AL6" s="27" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="7" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="115" t="s">
-        <v>102</v>
-      </c>
-      <c r="B7" s="111" t="s">
-        <v>104</v>
+      <c r="AM6" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="AN6" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="AO6" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="AP6" s="27"/>
+      <c r="AQ6" s="82" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="7" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="91" t="s">
+        <v>99</v>
+      </c>
+      <c r="B7" s="91" t="s">
+        <v>101</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D7" s="30" t="s">
         <v>71</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="F7" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="G7" s="59" t="s">
-        <v>120</v>
-      </c>
-      <c r="H7" s="75" t="s">
-        <v>180</v>
+        <v>100</v>
+      </c>
+      <c r="G7" s="76" t="s">
+        <v>117</v>
+      </c>
+      <c r="H7" s="68" t="s">
+        <v>177</v>
       </c>
       <c r="I7" s="30" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="J7" s="24" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="K7" s="30" t="s">
-        <v>189</v>
-      </c>
-      <c r="L7" s="59" t="s">
-        <v>120</v>
-      </c>
-      <c r="M7" s="162" t="s">
-        <v>203</v>
-      </c>
-      <c r="N7" s="163"/>
-      <c r="O7" s="164"/>
-      <c r="P7" s="124" t="s">
-        <v>209</v>
-      </c>
-      <c r="Q7" s="34"/>
+        <v>186</v>
+      </c>
+      <c r="L7" s="76" t="s">
+        <v>117</v>
+      </c>
+      <c r="M7" s="108" t="s">
+        <v>200</v>
+      </c>
+      <c r="N7" s="108"/>
+      <c r="O7" s="108"/>
+      <c r="P7" s="95" t="s">
+        <v>206</v>
+      </c>
+      <c r="Q7" s="32"/>
       <c r="R7" s="33"/>
       <c r="S7" s="33"/>
       <c r="T7" s="33"/>
@@ -2833,7 +2845,7 @@
       <c r="W7" s="33"/>
       <c r="X7" s="33"/>
       <c r="Y7" s="33"/>
-      <c r="Z7" s="35"/>
+      <c r="Z7" s="34"/>
       <c r="AA7" s="32"/>
       <c r="AB7" s="33"/>
       <c r="AC7" s="32"/>
@@ -2843,48 +2855,55 @@
       <c r="AG7" s="32"/>
       <c r="AH7" s="32"/>
       <c r="AI7" s="31"/>
-      <c r="AJ7" s="49"/>
-      <c r="AK7" s="44"/>
-      <c r="AL7" s="72"/>
-    </row>
-    <row r="8" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="123"/>
-      <c r="B8" s="111"/>
-      <c r="C8" s="111" t="s">
-        <v>130</v>
+      <c r="AJ7" s="31"/>
+      <c r="AK7" s="32"/>
+      <c r="AL7" s="32"/>
+      <c r="AM7" s="51"/>
+      <c r="AN7" s="130" t="s">
+        <v>214</v>
+      </c>
+      <c r="AQ7" s="157" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="8" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="115"/>
+      <c r="B8" s="115"/>
+      <c r="C8" s="89" t="s">
+        <v>127</v>
       </c>
       <c r="D8" s="30" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="F8" s="30" t="s">
-        <v>113</v>
-      </c>
-      <c r="G8" s="59" t="s">
-        <v>121</v>
-      </c>
-      <c r="H8" s="75" t="s">
-        <v>181</v>
+        <v>110</v>
+      </c>
+      <c r="G8" s="76" t="s">
+        <v>118</v>
+      </c>
+      <c r="H8" s="68" t="s">
+        <v>178</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="J8" s="30" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="K8" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="L8" s="59" t="s">
-        <v>199</v>
-      </c>
-      <c r="M8" s="165"/>
-      <c r="N8" s="166"/>
-      <c r="O8" s="167"/>
-      <c r="P8" s="125"/>
-      <c r="Q8" s="34"/>
+        <v>187</v>
+      </c>
+      <c r="L8" s="76" t="s">
+        <v>196</v>
+      </c>
+      <c r="M8" s="108"/>
+      <c r="N8" s="108"/>
+      <c r="O8" s="108"/>
+      <c r="P8" s="95"/>
+      <c r="Q8" s="32"/>
       <c r="R8" s="33"/>
       <c r="S8" s="33"/>
       <c r="T8" s="33"/>
@@ -2893,7 +2912,7 @@
       <c r="W8" s="33"/>
       <c r="X8" s="33"/>
       <c r="Y8" s="33"/>
-      <c r="Z8" s="35"/>
+      <c r="Z8" s="34"/>
       <c r="AA8" s="32"/>
       <c r="AB8" s="33"/>
       <c r="AC8" s="32"/>
@@ -2903,46 +2922,49 @@
       <c r="AG8" s="32"/>
       <c r="AH8" s="32"/>
       <c r="AI8" s="31"/>
-      <c r="AJ8" s="49"/>
-      <c r="AK8" s="44"/>
-      <c r="AL8" s="72"/>
-    </row>
-    <row r="9" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="123"/>
-      <c r="B9" s="111"/>
-      <c r="C9" s="111"/>
+      <c r="AJ8" s="31"/>
+      <c r="AK8" s="32"/>
+      <c r="AL8" s="32"/>
+      <c r="AM8" s="51"/>
+      <c r="AN8" s="130"/>
+      <c r="AQ8" s="157"/>
+    </row>
+    <row r="9" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="115"/>
+      <c r="B9" s="115"/>
+      <c r="C9" s="89"/>
       <c r="D9" s="30" t="s">
         <v>21</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F9" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="G9" s="59" t="s">
-        <v>122</v>
-      </c>
-      <c r="H9" s="75" t="s">
-        <v>182</v>
+        <v>111</v>
+      </c>
+      <c r="G9" s="76" t="s">
+        <v>119</v>
+      </c>
+      <c r="H9" s="68" t="s">
+        <v>179</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J9" s="30" t="s">
-        <v>175</v>
-      </c>
-      <c r="K9" s="105" t="s">
-        <v>191</v>
-      </c>
-      <c r="L9" s="119" t="s">
-        <v>200</v>
-      </c>
-      <c r="M9" s="165"/>
-      <c r="N9" s="166"/>
-      <c r="O9" s="167"/>
-      <c r="P9" s="125"/>
-      <c r="Q9" s="34"/>
+        <v>172</v>
+      </c>
+      <c r="K9" s="95" t="s">
+        <v>188</v>
+      </c>
+      <c r="L9" s="76" t="s">
+        <v>197</v>
+      </c>
+      <c r="M9" s="108"/>
+      <c r="N9" s="108"/>
+      <c r="O9" s="108"/>
+      <c r="P9" s="95"/>
+      <c r="Q9" s="32"/>
       <c r="R9" s="33"/>
       <c r="S9" s="33"/>
       <c r="T9" s="33"/>
@@ -2951,7 +2973,7 @@
       <c r="W9" s="33"/>
       <c r="X9" s="33"/>
       <c r="Y9" s="33"/>
-      <c r="Z9" s="35"/>
+      <c r="Z9" s="34"/>
       <c r="AA9" s="32"/>
       <c r="AB9" s="33"/>
       <c r="AC9" s="30"/>
@@ -2961,44 +2983,47 @@
       <c r="AG9" s="30"/>
       <c r="AH9" s="30"/>
       <c r="AI9" s="24"/>
-      <c r="AJ9" s="50"/>
-      <c r="AK9" s="45"/>
-      <c r="AL9" s="64"/>
-    </row>
-    <row r="10" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="123"/>
-      <c r="B10" s="111"/>
+      <c r="AJ9" s="24"/>
+      <c r="AK9" s="30"/>
+      <c r="AL9" s="30"/>
+      <c r="AM9" s="51"/>
+      <c r="AN9" s="130"/>
+      <c r="AQ9" s="157"/>
+    </row>
+    <row r="10" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="115"/>
+      <c r="B10" s="115"/>
       <c r="C10" s="24" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E10" s="30" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F10" s="30" t="s">
-        <v>115</v>
-      </c>
-      <c r="G10" s="59" t="s">
-        <v>123</v>
-      </c>
-      <c r="H10" s="75" t="s">
-        <v>183</v>
+        <v>112</v>
+      </c>
+      <c r="G10" s="76" t="s">
+        <v>120</v>
+      </c>
+      <c r="H10" s="68" t="s">
+        <v>180</v>
       </c>
       <c r="I10" s="30" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J10" s="30" t="s">
-        <v>175</v>
-      </c>
-      <c r="K10" s="105"/>
-      <c r="L10" s="119"/>
-      <c r="M10" s="165"/>
-      <c r="N10" s="166"/>
-      <c r="O10" s="167"/>
-      <c r="P10" s="125"/>
-      <c r="Q10" s="34"/>
+        <v>172</v>
+      </c>
+      <c r="K10" s="95"/>
+      <c r="L10" s="76"/>
+      <c r="M10" s="108"/>
+      <c r="N10" s="108"/>
+      <c r="O10" s="108"/>
+      <c r="P10" s="95"/>
+      <c r="Q10" s="32"/>
       <c r="R10" s="33"/>
       <c r="S10" s="33"/>
       <c r="T10" s="33"/>
@@ -3007,7 +3032,7 @@
       <c r="W10" s="33"/>
       <c r="X10" s="33"/>
       <c r="Y10" s="33"/>
-      <c r="Z10" s="35"/>
+      <c r="Z10" s="34"/>
       <c r="AA10" s="32"/>
       <c r="AB10" s="33"/>
       <c r="AC10" s="30"/>
@@ -3017,32 +3042,35 @@
       <c r="AG10" s="30"/>
       <c r="AH10" s="30"/>
       <c r="AI10" s="24"/>
-      <c r="AJ10" s="50"/>
-      <c r="AK10" s="45"/>
-      <c r="AL10" s="64"/>
-    </row>
-    <row r="11" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="123"/>
-      <c r="B11" s="111"/>
-      <c r="C11" s="127"/>
-      <c r="D11" s="128"/>
-      <c r="E11" s="128"/>
-      <c r="F11" s="128"/>
-      <c r="G11" s="128"/>
-      <c r="H11" s="128"/>
-      <c r="I11" s="128"/>
-      <c r="J11" s="129"/>
+      <c r="AJ10" s="24"/>
+      <c r="AK10" s="30"/>
+      <c r="AL10" s="30"/>
+      <c r="AM10" s="51"/>
+      <c r="AN10" s="130"/>
+      <c r="AQ10" s="157"/>
+    </row>
+    <row r="11" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="115"/>
+      <c r="B11" s="115"/>
+      <c r="C11" s="88"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="88"/>
+      <c r="F11" s="88"/>
+      <c r="G11" s="88"/>
+      <c r="H11" s="88"/>
+      <c r="I11" s="88"/>
+      <c r="J11" s="88"/>
       <c r="K11" s="30" t="s">
-        <v>192</v>
-      </c>
-      <c r="L11" s="59" t="s">
-        <v>201</v>
-      </c>
-      <c r="M11" s="168"/>
-      <c r="N11" s="169"/>
-      <c r="O11" s="170"/>
-      <c r="P11" s="126"/>
-      <c r="Q11" s="34"/>
+        <v>189</v>
+      </c>
+      <c r="L11" s="76" t="s">
+        <v>198</v>
+      </c>
+      <c r="M11" s="108"/>
+      <c r="N11" s="108"/>
+      <c r="O11" s="108"/>
+      <c r="P11" s="95"/>
+      <c r="Q11" s="32"/>
       <c r="R11" s="33"/>
       <c r="S11" s="33"/>
       <c r="T11" s="33"/>
@@ -3051,7 +3079,7 @@
       <c r="W11" s="33"/>
       <c r="X11" s="33"/>
       <c r="Y11" s="33"/>
-      <c r="Z11" s="35"/>
+      <c r="Z11" s="34"/>
       <c r="AA11" s="32"/>
       <c r="AB11" s="33"/>
       <c r="AC11" s="30"/>
@@ -3061,36 +3089,41 @@
       <c r="AG11" s="30"/>
       <c r="AH11" s="30"/>
       <c r="AI11" s="24"/>
-      <c r="AJ11" s="50"/>
-      <c r="AK11" s="45"/>
-      <c r="AL11" s="64"/>
-    </row>
-    <row r="12" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="123"/>
-      <c r="B12" s="111"/>
-      <c r="C12" s="130"/>
-      <c r="D12" s="131"/>
-      <c r="E12" s="131"/>
-      <c r="F12" s="131"/>
-      <c r="G12" s="131"/>
-      <c r="H12" s="131"/>
-      <c r="I12" s="131"/>
-      <c r="J12" s="132"/>
+      <c r="AJ11" s="24"/>
+      <c r="AK11" s="30"/>
+      <c r="AL11" s="30"/>
+      <c r="AM11" s="51"/>
+      <c r="AN11" s="130" t="s">
+        <v>215</v>
+      </c>
+      <c r="AQ11" s="157"/>
+    </row>
+    <row r="12" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="115"/>
+      <c r="B12" s="115"/>
+      <c r="C12" s="88"/>
+      <c r="D12" s="88"/>
+      <c r="E12" s="88"/>
+      <c r="F12" s="88"/>
+      <c r="G12" s="88"/>
+      <c r="H12" s="88"/>
+      <c r="I12" s="88"/>
+      <c r="J12" s="88"/>
       <c r="K12" s="30" t="s">
-        <v>193</v>
-      </c>
-      <c r="L12" s="59" t="s">
-        <v>202</v>
-      </c>
-      <c r="M12" s="171" t="s">
-        <v>208</v>
-      </c>
-      <c r="N12" s="172"/>
-      <c r="O12" s="173"/>
+        <v>190</v>
+      </c>
+      <c r="L12" s="76" t="s">
+        <v>199</v>
+      </c>
+      <c r="M12" s="108" t="s">
+        <v>205</v>
+      </c>
+      <c r="N12" s="108"/>
+      <c r="O12" s="108"/>
       <c r="P12" s="30" t="s">
-        <v>210</v>
-      </c>
-      <c r="Q12" s="34"/>
+        <v>207</v>
+      </c>
+      <c r="Q12" s="32"/>
       <c r="R12" s="33"/>
       <c r="S12" s="33"/>
       <c r="T12" s="33"/>
@@ -3099,7 +3132,7 @@
       <c r="W12" s="33"/>
       <c r="X12" s="33"/>
       <c r="Y12" s="33"/>
-      <c r="Z12" s="35"/>
+      <c r="Z12" s="34"/>
       <c r="AA12" s="32"/>
       <c r="AB12" s="33"/>
       <c r="AC12" s="30"/>
@@ -3109,52 +3142,57 @@
       <c r="AG12" s="30"/>
       <c r="AH12" s="30"/>
       <c r="AI12" s="24"/>
-      <c r="AJ12" s="50"/>
-      <c r="AK12" s="45"/>
-      <c r="AL12" s="64"/>
-    </row>
-    <row r="13" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="123"/>
-      <c r="B13" s="111"/>
+      <c r="AJ12" s="24"/>
+      <c r="AK12" s="30"/>
+      <c r="AL12" s="30"/>
+      <c r="AM12" s="51"/>
+      <c r="AN12" s="130"/>
+      <c r="AQ12" s="157" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="13" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="115"/>
+      <c r="B13" s="115"/>
       <c r="C13" s="24" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F13" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="G13" s="59" t="s">
-        <v>124</v>
-      </c>
-      <c r="H13" s="75" t="s">
-        <v>184</v>
+        <v>113</v>
+      </c>
+      <c r="G13" s="76" t="s">
+        <v>121</v>
+      </c>
+      <c r="H13" s="68" t="s">
+        <v>181</v>
       </c>
       <c r="I13" s="30" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="K13" s="30" t="s">
-        <v>194</v>
-      </c>
-      <c r="L13" s="59" t="s">
-        <v>124</v>
-      </c>
-      <c r="M13" s="174" t="s">
-        <v>205</v>
-      </c>
-      <c r="N13" s="112"/>
-      <c r="O13" s="113"/>
+        <v>191</v>
+      </c>
+      <c r="L13" s="76" t="s">
+        <v>121</v>
+      </c>
+      <c r="M13" s="95" t="s">
+        <v>202</v>
+      </c>
+      <c r="N13" s="95"/>
+      <c r="O13" s="95"/>
       <c r="P13" s="30" t="s">
-        <v>214</v>
-      </c>
-      <c r="Q13" s="34"/>
+        <v>211</v>
+      </c>
+      <c r="Q13" s="32"/>
       <c r="R13" s="33"/>
       <c r="S13" s="33"/>
       <c r="T13" s="33"/>
@@ -3163,7 +3201,7 @@
       <c r="W13" s="33"/>
       <c r="X13" s="33"/>
       <c r="Y13" s="33"/>
-      <c r="Z13" s="35"/>
+      <c r="Z13" s="34"/>
       <c r="AA13" s="32"/>
       <c r="AB13" s="33"/>
       <c r="AC13" s="30"/>
@@ -3173,52 +3211,59 @@
       <c r="AG13" s="30"/>
       <c r="AH13" s="30"/>
       <c r="AI13" s="24"/>
-      <c r="AJ13" s="50"/>
-      <c r="AK13" s="45"/>
-      <c r="AL13" s="64"/>
-    </row>
-    <row r="14" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="123"/>
-      <c r="B14" s="111"/>
-      <c r="C14" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="D14" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="E14" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="F14" s="30" t="s">
-        <v>117</v>
-      </c>
-      <c r="G14" s="59" t="s">
-        <v>125</v>
-      </c>
-      <c r="H14" s="75" t="s">
-        <v>185</v>
-      </c>
-      <c r="I14" s="30" t="s">
-        <v>169</v>
-      </c>
-      <c r="J14" s="30" t="s">
-        <v>177</v>
-      </c>
-      <c r="K14" s="30" t="s">
-        <v>195</v>
-      </c>
-      <c r="L14" s="59" t="s">
-        <v>125</v>
-      </c>
-      <c r="M14" s="171" t="s">
-        <v>207</v>
-      </c>
-      <c r="N14" s="172"/>
-      <c r="O14" s="173"/>
-      <c r="P14" s="30" t="s">
-        <v>211</v>
-      </c>
-      <c r="Q14" s="34"/>
+      <c r="AJ13" s="24"/>
+      <c r="AK13" s="30"/>
+      <c r="AL13" s="30"/>
+      <c r="AM13" s="51"/>
+      <c r="AN13" s="79" t="s">
+        <v>220</v>
+      </c>
+      <c r="AQ13" s="157" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="14" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="115"/>
+      <c r="B14" s="115"/>
+      <c r="C14" s="91" t="s">
+        <v>130</v>
+      </c>
+      <c r="D14" s="93" t="s">
+        <v>144</v>
+      </c>
+      <c r="E14" s="91" t="s">
+        <v>130</v>
+      </c>
+      <c r="F14" s="93" t="s">
+        <v>114</v>
+      </c>
+      <c r="G14" s="126" t="s">
+        <v>122</v>
+      </c>
+      <c r="H14" s="128" t="s">
+        <v>182</v>
+      </c>
+      <c r="I14" s="93" t="s">
+        <v>166</v>
+      </c>
+      <c r="J14" s="93" t="s">
+        <v>174</v>
+      </c>
+      <c r="K14" s="93" t="s">
+        <v>192</v>
+      </c>
+      <c r="L14" s="76" t="s">
+        <v>122</v>
+      </c>
+      <c r="M14" s="108" t="s">
+        <v>204</v>
+      </c>
+      <c r="N14" s="108"/>
+      <c r="O14" s="108"/>
+      <c r="P14" s="95" t="s">
+        <v>208</v>
+      </c>
+      <c r="Q14" s="32"/>
       <c r="R14" s="33"/>
       <c r="S14" s="33"/>
       <c r="T14" s="33"/>
@@ -3237,52 +3282,35 @@
       <c r="AG14" s="30"/>
       <c r="AH14" s="30"/>
       <c r="AI14" s="30"/>
-      <c r="AJ14" s="36"/>
-      <c r="AK14" s="45"/>
-      <c r="AL14" s="64"/>
-    </row>
-    <row r="15" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="123"/>
-      <c r="B15" s="111"/>
-      <c r="C15" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="D15" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="E15" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="F15" s="30" t="s">
-        <v>118</v>
-      </c>
-      <c r="G15" s="59" t="s">
-        <v>126</v>
-      </c>
-      <c r="H15" s="75" t="s">
-        <v>186</v>
-      </c>
-      <c r="I15" s="30" t="s">
-        <v>170</v>
-      </c>
-      <c r="J15" s="24" t="s">
-        <v>178</v>
-      </c>
-      <c r="K15" s="30" t="s">
-        <v>196</v>
-      </c>
-      <c r="L15" s="59" t="s">
-        <v>126</v>
-      </c>
-      <c r="M15" s="174" t="s">
-        <v>206</v>
-      </c>
-      <c r="N15" s="112"/>
-      <c r="O15" s="113"/>
-      <c r="P15" s="30" t="s">
-        <v>212</v>
-      </c>
-      <c r="Q15" s="34"/>
+      <c r="AJ14" s="30"/>
+      <c r="AK14" s="30"/>
+      <c r="AL14" s="30"/>
+      <c r="AM14" s="51"/>
+      <c r="AN14" s="79" t="s">
+        <v>216</v>
+      </c>
+      <c r="AQ14" s="158" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="15" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="115"/>
+      <c r="B15" s="115"/>
+      <c r="C15" s="92"/>
+      <c r="D15" s="94"/>
+      <c r="E15" s="92"/>
+      <c r="F15" s="94"/>
+      <c r="G15" s="127"/>
+      <c r="H15" s="129"/>
+      <c r="I15" s="94"/>
+      <c r="J15" s="94"/>
+      <c r="K15" s="94"/>
+      <c r="L15" s="76"/>
+      <c r="M15" s="108"/>
+      <c r="N15" s="108"/>
+      <c r="O15" s="108"/>
+      <c r="P15" s="95"/>
+      <c r="Q15" s="32"/>
       <c r="R15" s="33"/>
       <c r="S15" s="33"/>
       <c r="T15" s="33"/>
@@ -3291,7 +3319,7 @@
       <c r="W15" s="33"/>
       <c r="X15" s="33"/>
       <c r="Y15" s="33"/>
-      <c r="Z15" s="35"/>
+      <c r="Z15" s="34"/>
       <c r="AA15" s="32"/>
       <c r="AB15" s="33"/>
       <c r="AC15" s="30"/>
@@ -3301,173 +3329,208 @@
       <c r="AG15" s="30"/>
       <c r="AH15" s="30"/>
       <c r="AI15" s="30"/>
-      <c r="AJ15" s="36"/>
-      <c r="AK15" s="45"/>
-      <c r="AL15" s="64"/>
-    </row>
-    <row r="16" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="123"/>
-      <c r="B16" s="111" t="s">
-        <v>135</v>
-      </c>
-      <c r="C16" s="73" t="s">
-        <v>136</v>
-      </c>
-      <c r="D16" s="24" t="s">
+      <c r="AJ15" s="30"/>
+      <c r="AK15" s="30"/>
+      <c r="AL15" s="30"/>
+      <c r="AM15" s="51"/>
+      <c r="AN15" s="79" t="s">
+        <v>217</v>
+      </c>
+      <c r="AQ15" s="158"/>
+    </row>
+    <row r="16" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="115"/>
+      <c r="B16" s="116"/>
+      <c r="C16" s="24" t="s">
+        <v>131</v>
+      </c>
+      <c r="D16" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>131</v>
+      </c>
+      <c r="F16" s="30" t="s">
+        <v>115</v>
+      </c>
+      <c r="G16" s="76" t="s">
+        <v>123</v>
+      </c>
+      <c r="H16" s="68" t="s">
+        <v>183</v>
+      </c>
+      <c r="I16" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="J16" s="24" t="s">
+        <v>175</v>
+      </c>
+      <c r="K16" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="L16" s="76" t="s">
+        <v>123</v>
+      </c>
+      <c r="M16" s="95" t="s">
+        <v>203</v>
+      </c>
+      <c r="N16" s="95"/>
+      <c r="O16" s="95"/>
+      <c r="P16" s="30" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q16" s="95"/>
+      <c r="R16" s="101"/>
+      <c r="S16" s="101"/>
+      <c r="T16" s="101"/>
+      <c r="U16" s="101"/>
+      <c r="V16" s="103"/>
+      <c r="W16" s="101"/>
+      <c r="X16" s="101"/>
+      <c r="Y16" s="101"/>
+      <c r="Z16" s="101"/>
+      <c r="AA16" s="95"/>
+      <c r="AB16" s="101"/>
+      <c r="AC16" s="95"/>
+      <c r="AD16" s="89"/>
+      <c r="AE16" s="95"/>
+      <c r="AF16" s="95"/>
+      <c r="AG16" s="95"/>
+      <c r="AH16" s="95"/>
+      <c r="AI16" s="95"/>
+      <c r="AJ16" s="95"/>
+      <c r="AK16" s="95"/>
+      <c r="AL16" s="30"/>
+      <c r="AM16" s="51"/>
+      <c r="AN16" s="79" t="s">
+        <v>219</v>
+      </c>
+      <c r="AQ16" s="157" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="17" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="115"/>
+      <c r="B17" s="91" t="s">
+        <v>132</v>
+      </c>
+      <c r="C17" s="66" t="s">
+        <v>133</v>
+      </c>
+      <c r="D17" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="F16" s="30" t="s">
-        <v>162</v>
-      </c>
-      <c r="G16" s="59" t="s">
-        <v>127</v>
-      </c>
-      <c r="H16" s="75" t="s">
-        <v>187</v>
-      </c>
-      <c r="I16" s="30" t="s">
+      <c r="E17" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="F17" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="G17" s="76" t="s">
+        <v>124</v>
+      </c>
+      <c r="H17" s="68" t="s">
+        <v>184</v>
+      </c>
+      <c r="I17" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="J17" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="K17" s="30" t="s">
+        <v>194</v>
+      </c>
+      <c r="L17" s="76" t="s">
+        <v>124</v>
+      </c>
+      <c r="M17" s="117" t="s">
+        <v>201</v>
+      </c>
+      <c r="N17" s="118"/>
+      <c r="O17" s="119"/>
+      <c r="P17" s="30" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q17" s="95"/>
+      <c r="R17" s="101"/>
+      <c r="S17" s="101"/>
+      <c r="T17" s="101"/>
+      <c r="U17" s="101"/>
+      <c r="V17" s="101"/>
+      <c r="W17" s="101"/>
+      <c r="X17" s="101"/>
+      <c r="Y17" s="101"/>
+      <c r="Z17" s="101"/>
+      <c r="AA17" s="101"/>
+      <c r="AB17" s="101"/>
+      <c r="AC17" s="95"/>
+      <c r="AD17" s="95"/>
+      <c r="AE17" s="95"/>
+      <c r="AF17" s="95"/>
+      <c r="AG17" s="95"/>
+      <c r="AH17" s="95"/>
+      <c r="AI17" s="95"/>
+      <c r="AJ17" s="95"/>
+      <c r="AK17" s="95"/>
+      <c r="AL17" s="30"/>
+      <c r="AM17" s="51"/>
+      <c r="AN17" s="79"/>
+      <c r="AQ17" s="158" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="18" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="116"/>
+      <c r="B18" s="116"/>
+      <c r="C18" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="D18" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="F18" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="G18" s="76" t="s">
+        <v>125</v>
+      </c>
+      <c r="H18" s="68" t="s">
+        <v>185</v>
+      </c>
+      <c r="I18" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="J18" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="J16" s="30" t="s">
-        <v>173</v>
-      </c>
-      <c r="K16" s="30" t="s">
-        <v>197</v>
-      </c>
-      <c r="L16" s="59" t="s">
-        <v>127</v>
-      </c>
-      <c r="M16" s="175" t="s">
-        <v>204</v>
-      </c>
-      <c r="N16" s="176"/>
-      <c r="O16" s="115"/>
-      <c r="P16" s="124" t="s">
+      <c r="K18" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="L18" s="76" t="s">
+        <v>212</v>
+      </c>
+      <c r="M18" s="120"/>
+      <c r="N18" s="99"/>
+      <c r="O18" s="100"/>
+      <c r="P18" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="Q16" s="115"/>
-      <c r="R16" s="117"/>
-      <c r="S16" s="106"/>
-      <c r="T16" s="106"/>
-      <c r="U16" s="106"/>
-      <c r="V16" s="114"/>
-      <c r="W16" s="106"/>
-      <c r="X16" s="106"/>
-      <c r="Y16" s="106"/>
-      <c r="Z16" s="106"/>
-      <c r="AA16" s="105"/>
-      <c r="AB16" s="106"/>
-      <c r="AC16" s="105"/>
-      <c r="AD16" s="111"/>
-      <c r="AE16" s="105"/>
-      <c r="AF16" s="105"/>
-      <c r="AG16" s="105"/>
-      <c r="AH16" s="105"/>
-      <c r="AI16" s="105"/>
-      <c r="AJ16" s="110"/>
-      <c r="AK16" s="109"/>
-      <c r="AL16" s="64"/>
-    </row>
-    <row r="17" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="116"/>
-      <c r="B17" s="111"/>
-      <c r="C17" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="D17" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" s="30" t="s">
-        <v>164</v>
-      </c>
-      <c r="F17" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="G17" s="59" t="s">
-        <v>128</v>
-      </c>
-      <c r="H17" s="75" t="s">
-        <v>188</v>
-      </c>
-      <c r="I17" s="30" t="s">
-        <v>172</v>
-      </c>
-      <c r="J17" s="30" t="s">
-        <v>174</v>
-      </c>
-      <c r="K17" s="30" t="s">
-        <v>198</v>
-      </c>
-      <c r="L17" s="59" t="s">
-        <v>128</v>
-      </c>
-      <c r="M17" s="177"/>
-      <c r="N17" s="178"/>
-      <c r="O17" s="116"/>
-      <c r="P17" s="126"/>
-      <c r="Q17" s="116"/>
-      <c r="R17" s="118"/>
-      <c r="S17" s="106"/>
-      <c r="T17" s="106"/>
-      <c r="U17" s="106"/>
-      <c r="V17" s="106"/>
-      <c r="W17" s="106"/>
-      <c r="X17" s="106"/>
-      <c r="Y17" s="106"/>
-      <c r="Z17" s="106"/>
-      <c r="AA17" s="106"/>
-      <c r="AB17" s="106"/>
-      <c r="AC17" s="105"/>
-      <c r="AD17" s="105"/>
-      <c r="AE17" s="105"/>
-      <c r="AF17" s="105"/>
-      <c r="AG17" s="105"/>
-      <c r="AH17" s="105"/>
-      <c r="AI17" s="105"/>
-      <c r="AJ17" s="110"/>
-      <c r="AK17" s="109"/>
-      <c r="AL17" s="64"/>
-    </row>
-    <row r="18" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="124" t="s">
-        <v>78</v>
-      </c>
-      <c r="B18" s="111" t="s">
-        <v>104</v>
-      </c>
-      <c r="C18" s="122"/>
-      <c r="D18" s="74" t="s">
-        <v>151</v>
-      </c>
-      <c r="E18" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="F18" s="57"/>
-      <c r="G18" s="57"/>
-      <c r="H18" s="57"/>
-      <c r="I18" s="55"/>
-      <c r="J18" s="56"/>
-      <c r="K18" s="76"/>
-      <c r="L18" s="30"/>
-      <c r="M18" s="37"/>
-      <c r="N18" s="30"/>
-      <c r="O18" s="30"/>
-      <c r="P18" s="30"/>
-      <c r="Q18" s="37"/>
-      <c r="R18" s="35"/>
+      <c r="Q18" s="30"/>
+      <c r="R18" s="34"/>
       <c r="S18" s="33"/>
       <c r="T18" s="33"/>
-      <c r="U18" s="35"/>
+      <c r="U18" s="34"/>
       <c r="V18" s="25"/>
-      <c r="W18" s="35"/>
-      <c r="X18" s="35"/>
-      <c r="Y18" s="35"/>
-      <c r="Z18" s="35"/>
+      <c r="W18" s="34"/>
+      <c r="X18" s="34"/>
+      <c r="Y18" s="34"/>
+      <c r="Z18" s="34"/>
       <c r="AA18" s="30"/>
-      <c r="AB18" s="35"/>
+      <c r="AB18" s="34"/>
       <c r="AC18" s="30"/>
       <c r="AD18" s="24"/>
       <c r="AE18" s="30"/>
@@ -3475,43 +3538,50 @@
       <c r="AG18" s="30"/>
       <c r="AH18" s="30"/>
       <c r="AI18" s="30"/>
-      <c r="AJ18" s="36"/>
-      <c r="AK18" s="45"/>
-      <c r="AL18" s="64"/>
-    </row>
-    <row r="19" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="125"/>
-      <c r="B19" s="111"/>
-      <c r="C19" s="122"/>
-      <c r="D19" s="74" t="s">
-        <v>152</v>
+      <c r="AJ18" s="30"/>
+      <c r="AK18" s="30"/>
+      <c r="AL18" s="30"/>
+      <c r="AM18" s="51"/>
+      <c r="AN18" s="79"/>
+      <c r="AQ18" s="158"/>
+    </row>
+    <row r="19" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="91" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="91" t="s">
+        <v>101</v>
+      </c>
+      <c r="C19" s="121"/>
+      <c r="D19" s="67" t="s">
+        <v>148</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="F19" s="55"/>
-      <c r="G19" s="56"/>
-      <c r="H19" s="56"/>
-      <c r="I19" s="55"/>
-      <c r="J19" s="56"/>
-      <c r="K19" s="30"/>
+        <v>135</v>
+      </c>
+      <c r="F19" s="51"/>
+      <c r="G19" s="51"/>
+      <c r="H19" s="51"/>
+      <c r="I19" s="49"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="69"/>
       <c r="L19" s="30"/>
-      <c r="M19" s="37"/>
+      <c r="M19" s="30"/>
       <c r="N19" s="30"/>
       <c r="O19" s="30"/>
       <c r="P19" s="30"/>
-      <c r="Q19" s="37"/>
-      <c r="R19" s="35"/>
+      <c r="Q19" s="30"/>
+      <c r="R19" s="34"/>
       <c r="S19" s="33"/>
       <c r="T19" s="33"/>
-      <c r="U19" s="106"/>
-      <c r="V19" s="35"/>
-      <c r="W19" s="35"/>
-      <c r="X19" s="35"/>
-      <c r="Y19" s="35"/>
-      <c r="Z19" s="35"/>
+      <c r="U19" s="101"/>
+      <c r="V19" s="34"/>
+      <c r="W19" s="34"/>
+      <c r="X19" s="34"/>
+      <c r="Y19" s="34"/>
+      <c r="Z19" s="34"/>
       <c r="AA19" s="30"/>
-      <c r="AB19" s="35"/>
+      <c r="AB19" s="34"/>
       <c r="AC19" s="30"/>
       <c r="AD19" s="24"/>
       <c r="AE19" s="30"/>
@@ -3519,43 +3589,46 @@
       <c r="AG19" s="30"/>
       <c r="AH19" s="30"/>
       <c r="AI19" s="30"/>
-      <c r="AJ19" s="36"/>
-      <c r="AK19" s="45"/>
-      <c r="AL19" s="64"/>
-    </row>
-    <row r="20" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="125"/>
-      <c r="B20" s="111"/>
+      <c r="AJ19" s="30"/>
+      <c r="AK19" s="30"/>
+      <c r="AL19" s="30"/>
+      <c r="AM19" s="51"/>
+      <c r="AN19" s="79"/>
+      <c r="AQ19" s="51"/>
+    </row>
+    <row r="20" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="115"/>
+      <c r="B20" s="115"/>
       <c r="C20" s="122"/>
-      <c r="D20" s="30" t="s">
-        <v>153</v>
+      <c r="D20" s="67" t="s">
+        <v>149</v>
       </c>
       <c r="E20" s="24" t="s">
-        <v>140</v>
-      </c>
-      <c r="F20" s="55"/>
-      <c r="G20" s="56"/>
-      <c r="H20" s="56"/>
-      <c r="I20" s="55"/>
-      <c r="J20" s="56"/>
+        <v>136</v>
+      </c>
+      <c r="F20" s="49"/>
+      <c r="G20" s="50"/>
+      <c r="H20" s="50"/>
+      <c r="I20" s="49"/>
+      <c r="J20" s="50"/>
       <c r="K20" s="30"/>
       <c r="L20" s="30"/>
-      <c r="M20" s="37"/>
+      <c r="M20" s="30"/>
       <c r="N20" s="30"/>
       <c r="O20" s="30"/>
       <c r="P20" s="30"/>
-      <c r="Q20" s="37"/>
-      <c r="R20" s="35"/>
+      <c r="Q20" s="30"/>
+      <c r="R20" s="34"/>
       <c r="S20" s="33"/>
       <c r="T20" s="33"/>
-      <c r="U20" s="106"/>
+      <c r="U20" s="101"/>
       <c r="V20" s="25"/>
-      <c r="W20" s="35"/>
-      <c r="X20" s="35"/>
-      <c r="Y20" s="35"/>
-      <c r="Z20" s="35"/>
+      <c r="W20" s="34"/>
+      <c r="X20" s="34"/>
+      <c r="Y20" s="34"/>
+      <c r="Z20" s="34"/>
       <c r="AA20" s="30"/>
-      <c r="AB20" s="35"/>
+      <c r="AB20" s="34"/>
       <c r="AC20" s="30"/>
       <c r="AD20" s="24"/>
       <c r="AE20" s="30"/>
@@ -3563,32 +3636,35 @@
       <c r="AG20" s="30"/>
       <c r="AH20" s="30"/>
       <c r="AI20" s="30"/>
-      <c r="AJ20" s="36"/>
-      <c r="AK20" s="45"/>
-      <c r="AL20" s="64"/>
-    </row>
-    <row r="21" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="125"/>
-      <c r="B21" s="111"/>
+      <c r="AJ20" s="30"/>
+      <c r="AK20" s="30"/>
+      <c r="AL20" s="30"/>
+      <c r="AM20" s="51"/>
+      <c r="AN20" s="79"/>
+      <c r="AQ20" s="51"/>
+    </row>
+    <row r="21" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="115"/>
+      <c r="B21" s="115"/>
       <c r="C21" s="122"/>
       <c r="D21" s="30" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>141</v>
-      </c>
-      <c r="F21" s="55"/>
-      <c r="G21" s="56"/>
-      <c r="H21" s="56"/>
-      <c r="I21" s="55"/>
-      <c r="J21" s="56"/>
+        <v>137</v>
+      </c>
+      <c r="F21" s="49"/>
+      <c r="G21" s="50"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="49"/>
+      <c r="J21" s="50"/>
       <c r="K21" s="30"/>
       <c r="L21" s="30"/>
-      <c r="M21" s="37"/>
+      <c r="M21" s="30"/>
       <c r="N21" s="30"/>
       <c r="O21" s="30"/>
       <c r="P21" s="30"/>
-      <c r="Q21" s="34"/>
+      <c r="Q21" s="32"/>
       <c r="R21" s="33"/>
       <c r="S21" s="33"/>
       <c r="T21" s="33"/>
@@ -3597,7 +3673,7 @@
       <c r="W21" s="33"/>
       <c r="X21" s="33"/>
       <c r="Y21" s="33"/>
-      <c r="Z21" s="35"/>
+      <c r="Z21" s="34"/>
       <c r="AA21" s="32"/>
       <c r="AB21" s="33"/>
       <c r="AC21" s="30"/>
@@ -3607,32 +3683,35 @@
       <c r="AG21" s="30"/>
       <c r="AH21" s="30"/>
       <c r="AI21" s="24"/>
-      <c r="AJ21" s="50"/>
-      <c r="AK21" s="45"/>
-      <c r="AL21" s="64"/>
-    </row>
-    <row r="22" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="125"/>
-      <c r="B22" s="111"/>
+      <c r="AJ21" s="24"/>
+      <c r="AK21" s="30"/>
+      <c r="AL21" s="30"/>
+      <c r="AM21" s="51"/>
+      <c r="AN21" s="79"/>
+      <c r="AQ21" s="51"/>
+    </row>
+    <row r="22" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="115"/>
+      <c r="B22" s="115"/>
       <c r="C22" s="122"/>
-      <c r="D22" s="24" t="s">
-        <v>155</v>
+      <c r="D22" s="30" t="s">
+        <v>151</v>
       </c>
       <c r="E22" s="24" t="s">
-        <v>142</v>
-      </c>
-      <c r="F22" s="55"/>
-      <c r="G22" s="56"/>
-      <c r="H22" s="56"/>
-      <c r="I22" s="55"/>
-      <c r="J22" s="56"/>
+        <v>138</v>
+      </c>
+      <c r="F22" s="49"/>
+      <c r="G22" s="50"/>
+      <c r="H22" s="50"/>
+      <c r="I22" s="49"/>
+      <c r="J22" s="50"/>
       <c r="K22" s="30"/>
       <c r="L22" s="30"/>
-      <c r="M22" s="37"/>
+      <c r="M22" s="30"/>
       <c r="N22" s="30"/>
       <c r="O22" s="30"/>
       <c r="P22" s="30"/>
-      <c r="Q22" s="34"/>
+      <c r="Q22" s="32"/>
       <c r="R22" s="33"/>
       <c r="S22" s="33"/>
       <c r="T22" s="33"/>
@@ -3641,7 +3720,7 @@
       <c r="W22" s="33"/>
       <c r="X22" s="33"/>
       <c r="Y22" s="33"/>
-      <c r="Z22" s="35"/>
+      <c r="Z22" s="34"/>
       <c r="AA22" s="32"/>
       <c r="AB22" s="33"/>
       <c r="AC22" s="30"/>
@@ -3651,45 +3730,48 @@
       <c r="AG22" s="30"/>
       <c r="AH22" s="30"/>
       <c r="AI22" s="24"/>
-      <c r="AJ22" s="50"/>
-      <c r="AK22" s="45"/>
-      <c r="AL22" s="64"/>
-    </row>
-    <row r="23" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="125"/>
-      <c r="B23" s="111" t="s">
-        <v>135</v>
-      </c>
+      <c r="AJ22" s="24"/>
+      <c r="AK22" s="30"/>
+      <c r="AL22" s="30"/>
+      <c r="AM22" s="51"/>
+      <c r="AN22" s="79" t="s">
+        <v>218</v>
+      </c>
+      <c r="AQ22" s="51"/>
+    </row>
+    <row r="23" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="115"/>
+      <c r="B23" s="116"/>
       <c r="C23" s="122"/>
       <c r="D23" s="24" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>145</v>
-      </c>
-      <c r="F23" s="55"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="55"/>
-      <c r="J23" s="56"/>
+        <v>139</v>
+      </c>
+      <c r="F23" s="49"/>
+      <c r="G23" s="50"/>
+      <c r="H23" s="50"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="50"/>
       <c r="K23" s="30"/>
       <c r="L23" s="30"/>
-      <c r="M23" s="37"/>
+      <c r="M23" s="30"/>
       <c r="N23" s="30"/>
       <c r="O23" s="30"/>
       <c r="P23" s="30"/>
-      <c r="Q23" s="34"/>
-      <c r="R23" s="35"/>
+      <c r="Q23" s="32"/>
+      <c r="R23" s="34"/>
       <c r="S23" s="33"/>
       <c r="T23" s="33"/>
-      <c r="U23" s="35"/>
+      <c r="U23" s="34"/>
       <c r="V23" s="25"/>
-      <c r="W23" s="35"/>
-      <c r="X23" s="35"/>
-      <c r="Y23" s="35"/>
-      <c r="Z23" s="35"/>
+      <c r="W23" s="34"/>
+      <c r="X23" s="34"/>
+      <c r="Y23" s="34"/>
+      <c r="Z23" s="34"/>
       <c r="AA23" s="32"/>
-      <c r="AB23" s="35"/>
+      <c r="AB23" s="34"/>
       <c r="AC23" s="30"/>
       <c r="AD23" s="24"/>
       <c r="AE23" s="30"/>
@@ -3697,43 +3779,48 @@
       <c r="AG23" s="30"/>
       <c r="AH23" s="30"/>
       <c r="AI23" s="24"/>
-      <c r="AJ23" s="50"/>
-      <c r="AK23" s="45"/>
-      <c r="AL23" s="64"/>
-    </row>
-    <row r="24" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="125"/>
-      <c r="B24" s="111"/>
+      <c r="AJ23" s="24"/>
+      <c r="AK23" s="30"/>
+      <c r="AL23" s="30"/>
+      <c r="AM23" s="51"/>
+      <c r="AN23" s="80"/>
+      <c r="AQ23" s="51"/>
+    </row>
+    <row r="24" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="115"/>
+      <c r="B24" s="91" t="s">
+        <v>132</v>
+      </c>
       <c r="C24" s="122"/>
       <c r="D24" s="24" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>143</v>
-      </c>
-      <c r="F24" s="55"/>
-      <c r="G24" s="56"/>
-      <c r="H24" s="56"/>
-      <c r="I24" s="55"/>
-      <c r="J24" s="56"/>
+        <v>142</v>
+      </c>
+      <c r="F24" s="49"/>
+      <c r="G24" s="50"/>
+      <c r="H24" s="50"/>
+      <c r="I24" s="49"/>
+      <c r="J24" s="50"/>
       <c r="K24" s="30"/>
-      <c r="L24" s="24"/>
-      <c r="M24" s="37"/>
-      <c r="N24" s="24"/>
-      <c r="O24" s="24"/>
+      <c r="L24" s="30"/>
+      <c r="M24" s="30"/>
+      <c r="N24" s="30"/>
+      <c r="O24" s="30"/>
       <c r="P24" s="30"/>
-      <c r="Q24" s="37"/>
-      <c r="R24" s="35"/>
-      <c r="S24" s="35"/>
-      <c r="T24" s="35"/>
-      <c r="U24" s="35"/>
-      <c r="V24" s="35"/>
-      <c r="W24" s="35"/>
-      <c r="X24" s="35"/>
-      <c r="Y24" s="35"/>
-      <c r="Z24" s="35"/>
+      <c r="Q24" s="30"/>
+      <c r="R24" s="34"/>
+      <c r="S24" s="34"/>
+      <c r="T24" s="34"/>
+      <c r="U24" s="34"/>
+      <c r="V24" s="34"/>
+      <c r="W24" s="34"/>
+      <c r="X24" s="34"/>
+      <c r="Y24" s="34"/>
+      <c r="Z24" s="34"/>
       <c r="AA24" s="30"/>
-      <c r="AB24" s="35"/>
+      <c r="AB24" s="34"/>
       <c r="AC24" s="30"/>
       <c r="AD24" s="30"/>
       <c r="AE24" s="30"/>
@@ -3741,41 +3828,44 @@
       <c r="AG24" s="30"/>
       <c r="AH24" s="30"/>
       <c r="AI24" s="30"/>
-      <c r="AJ24" s="36"/>
-      <c r="AK24" s="45"/>
-      <c r="AL24" s="64"/>
-    </row>
-    <row r="25" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="126"/>
-      <c r="B25" s="111"/>
+      <c r="AJ24" s="30"/>
+      <c r="AK24" s="30"/>
+      <c r="AL24" s="30"/>
+      <c r="AM24" s="51"/>
+      <c r="AN24" s="51"/>
+      <c r="AQ24" s="51"/>
+    </row>
+    <row r="25" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="115"/>
+      <c r="B25" s="115"/>
       <c r="C25" s="122"/>
       <c r="D25" s="24" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E25" s="24" t="s">
-        <v>144</v>
-      </c>
-      <c r="F25" s="55"/>
-      <c r="G25" s="56"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="55"/>
-      <c r="J25" s="56"/>
+        <v>140</v>
+      </c>
+      <c r="F25" s="49"/>
+      <c r="G25" s="50"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="49"/>
+      <c r="J25" s="50"/>
       <c r="K25" s="30"/>
       <c r="L25" s="24"/>
-      <c r="M25" s="37"/>
+      <c r="M25" s="30"/>
       <c r="N25" s="24"/>
       <c r="O25" s="24"/>
       <c r="P25" s="30"/>
-      <c r="Q25" s="34"/>
+      <c r="Q25" s="32"/>
       <c r="R25" s="33"/>
-      <c r="S25" s="35"/>
-      <c r="T25" s="35"/>
-      <c r="U25" s="35"/>
-      <c r="V25" s="35"/>
-      <c r="W25" s="35"/>
-      <c r="X25" s="35"/>
-      <c r="Y25" s="35"/>
-      <c r="Z25" s="35"/>
+      <c r="S25" s="34"/>
+      <c r="T25" s="34"/>
+      <c r="U25" s="34"/>
+      <c r="V25" s="34"/>
+      <c r="W25" s="34"/>
+      <c r="X25" s="34"/>
+      <c r="Y25" s="34"/>
+      <c r="Z25" s="34"/>
       <c r="AA25" s="32"/>
       <c r="AB25" s="33"/>
       <c r="AC25" s="30"/>
@@ -3785,119 +3875,129 @@
       <c r="AG25" s="30"/>
       <c r="AH25" s="30"/>
       <c r="AI25" s="30"/>
-      <c r="AJ25" s="36"/>
-      <c r="AK25" s="45"/>
-      <c r="AL25" s="64"/>
-    </row>
-    <row r="26" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="63"/>
-      <c r="B26" s="62"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="62"/>
-      <c r="E26" s="63"/>
-      <c r="F26" s="63"/>
-      <c r="G26" s="62"/>
-      <c r="H26" s="62"/>
-      <c r="I26" s="63"/>
-      <c r="J26" s="62"/>
-      <c r="K26" s="64"/>
-      <c r="L26" s="65"/>
-      <c r="M26" s="64"/>
-      <c r="N26" s="65"/>
-      <c r="O26" s="65"/>
-      <c r="P26" s="64"/>
-      <c r="Q26" s="34"/>
+      <c r="AJ25" s="30"/>
+      <c r="AK25" s="30"/>
+      <c r="AL25" s="30"/>
+      <c r="AM25" s="51"/>
+      <c r="AN25" s="51"/>
+      <c r="AQ25" s="51"/>
+    </row>
+    <row r="26" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="116"/>
+      <c r="B26" s="116"/>
+      <c r="C26" s="123"/>
+      <c r="D26" s="24" t="s">
+        <v>155</v>
+      </c>
+      <c r="E26" s="24" t="s">
+        <v>141</v>
+      </c>
+      <c r="F26" s="49"/>
+      <c r="G26" s="50"/>
+      <c r="H26" s="50"/>
+      <c r="I26" s="49"/>
+      <c r="J26" s="50"/>
+      <c r="K26" s="30"/>
+      <c r="L26" s="24"/>
+      <c r="M26" s="30"/>
+      <c r="N26" s="24"/>
+      <c r="O26" s="24"/>
+      <c r="P26" s="30"/>
+      <c r="Q26" s="32"/>
       <c r="R26" s="33"/>
-      <c r="S26" s="35"/>
-      <c r="T26" s="35"/>
-      <c r="U26" s="35"/>
-      <c r="V26" s="35"/>
-      <c r="W26" s="35"/>
-      <c r="X26" s="35"/>
-      <c r="Y26" s="35"/>
-      <c r="Z26" s="35"/>
+      <c r="S26" s="34"/>
+      <c r="T26" s="34"/>
+      <c r="U26" s="34"/>
+      <c r="V26" s="34"/>
+      <c r="W26" s="34"/>
+      <c r="X26" s="34"/>
+      <c r="Y26" s="34"/>
+      <c r="Z26" s="34"/>
       <c r="AA26" s="32"/>
       <c r="AB26" s="33"/>
       <c r="AC26" s="32"/>
-      <c r="AD26" s="38"/>
+      <c r="AD26" s="37"/>
       <c r="AE26" s="30"/>
       <c r="AF26" s="32"/>
       <c r="AG26" s="32"/>
       <c r="AH26" s="30"/>
       <c r="AI26" s="30"/>
-      <c r="AJ26" s="36"/>
-      <c r="AK26" s="45"/>
-      <c r="AL26" s="64"/>
-    </row>
-    <row r="27" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="63"/>
-      <c r="B27" s="62"/>
-      <c r="C27" s="62"/>
-      <c r="D27" s="62"/>
-      <c r="E27" s="63"/>
-      <c r="F27" s="63"/>
-      <c r="G27" s="62"/>
-      <c r="H27" s="62"/>
-      <c r="I27" s="63"/>
-      <c r="J27" s="62"/>
-      <c r="K27" s="64"/>
-      <c r="L27" s="65"/>
-      <c r="M27" s="64"/>
-      <c r="N27" s="65"/>
-      <c r="O27" s="65"/>
-      <c r="P27" s="64"/>
-      <c r="Q27" s="112"/>
-      <c r="R27" s="113"/>
-      <c r="S27" s="35"/>
-      <c r="T27" s="35"/>
-      <c r="U27" s="35"/>
-      <c r="V27" s="35"/>
-      <c r="W27" s="35"/>
-      <c r="X27" s="35"/>
-      <c r="Y27" s="35"/>
-      <c r="Z27" s="35"/>
-      <c r="AA27" s="105"/>
-      <c r="AB27" s="105"/>
-      <c r="AC27" s="30"/>
-      <c r="AD27" s="30"/>
-      <c r="AE27" s="30"/>
-      <c r="AF27" s="30"/>
-      <c r="AG27" s="30"/>
-      <c r="AH27" s="30"/>
-      <c r="AI27" s="30"/>
-      <c r="AJ27" s="36"/>
-      <c r="AK27" s="46"/>
-      <c r="AL27" s="81"/>
-    </row>
-    <row r="28" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="63"/>
-      <c r="B28" s="62"/>
-      <c r="C28" s="62"/>
-      <c r="D28" s="62"/>
-      <c r="E28" s="63"/>
-      <c r="F28" s="63"/>
-      <c r="G28" s="62"/>
-      <c r="H28" s="62"/>
-      <c r="I28" s="63"/>
-      <c r="J28" s="62"/>
-      <c r="K28" s="64"/>
-      <c r="L28" s="65"/>
-      <c r="M28" s="64"/>
-      <c r="N28" s="65"/>
-      <c r="O28" s="65"/>
-      <c r="P28" s="64"/>
-      <c r="Q28" s="112"/>
-      <c r="R28" s="113"/>
-      <c r="S28" s="35"/>
-      <c r="T28" s="35"/>
-      <c r="U28" s="35"/>
-      <c r="V28" s="35"/>
-      <c r="W28" s="35"/>
-      <c r="X28" s="35"/>
-      <c r="Y28" s="35"/>
-      <c r="Z28" s="35"/>
-      <c r="AA28" s="105"/>
-      <c r="AB28" s="105"/>
+      <c r="AJ26" s="30"/>
+      <c r="AK26" s="30"/>
+      <c r="AL26" s="30"/>
+      <c r="AM26" s="51"/>
+      <c r="AN26" s="51"/>
+      <c r="AQ26" s="51"/>
+    </row>
+    <row r="27" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="56"/>
+      <c r="B27" s="55"/>
+      <c r="C27" s="55"/>
+      <c r="D27" s="55"/>
+      <c r="E27" s="56"/>
+      <c r="F27" s="56"/>
+      <c r="G27" s="55"/>
+      <c r="H27" s="55"/>
+      <c r="I27" s="56"/>
+      <c r="J27" s="55"/>
+      <c r="K27" s="57"/>
+      <c r="L27" s="58"/>
+      <c r="M27" s="57"/>
+      <c r="N27" s="58"/>
+      <c r="O27" s="58"/>
+      <c r="P27" s="57"/>
+      <c r="Q27" s="99"/>
+      <c r="R27" s="100"/>
+      <c r="S27" s="75"/>
+      <c r="T27" s="75"/>
+      <c r="U27" s="75"/>
+      <c r="V27" s="75"/>
+      <c r="W27" s="75"/>
+      <c r="X27" s="75"/>
+      <c r="Y27" s="75"/>
+      <c r="Z27" s="75"/>
+      <c r="AA27" s="94"/>
+      <c r="AB27" s="94"/>
+      <c r="AC27" s="74"/>
+      <c r="AD27" s="74"/>
+      <c r="AE27" s="74"/>
+      <c r="AF27" s="74"/>
+      <c r="AG27" s="74"/>
+      <c r="AH27" s="74"/>
+      <c r="AI27" s="74"/>
+      <c r="AJ27" s="77"/>
+      <c r="AK27" s="78"/>
+      <c r="AL27" s="73"/>
+    </row>
+    <row r="28" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="56"/>
+      <c r="B28" s="55"/>
+      <c r="C28" s="55"/>
+      <c r="D28" s="55"/>
+      <c r="E28" s="56"/>
+      <c r="F28" s="56"/>
+      <c r="G28" s="55"/>
+      <c r="H28" s="55"/>
+      <c r="I28" s="56"/>
+      <c r="J28" s="55"/>
+      <c r="K28" s="57"/>
+      <c r="L28" s="58"/>
+      <c r="M28" s="57"/>
+      <c r="N28" s="58"/>
+      <c r="O28" s="58"/>
+      <c r="P28" s="57"/>
+      <c r="Q28" s="97"/>
+      <c r="R28" s="98"/>
+      <c r="S28" s="34"/>
+      <c r="T28" s="34"/>
+      <c r="U28" s="34"/>
+      <c r="V28" s="34"/>
+      <c r="W28" s="34"/>
+      <c r="X28" s="34"/>
+      <c r="Y28" s="34"/>
+      <c r="Z28" s="34"/>
+      <c r="AA28" s="95"/>
+      <c r="AB28" s="95"/>
       <c r="AC28" s="30"/>
       <c r="AD28" s="30"/>
       <c r="AE28" s="30"/>
@@ -3905,39 +4005,39 @@
       <c r="AG28" s="30"/>
       <c r="AH28" s="30"/>
       <c r="AI28" s="30"/>
-      <c r="AJ28" s="36"/>
-      <c r="AK28" s="46"/>
-      <c r="AL28" s="81"/>
-    </row>
-    <row r="29" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="63"/>
-      <c r="B29" s="62"/>
-      <c r="C29" s="62"/>
-      <c r="D29" s="62"/>
-      <c r="E29" s="63"/>
-      <c r="F29" s="63"/>
-      <c r="G29" s="62"/>
-      <c r="H29" s="62"/>
-      <c r="I29" s="63"/>
-      <c r="J29" s="62"/>
-      <c r="K29" s="64"/>
-      <c r="L29" s="65"/>
-      <c r="M29" s="64"/>
-      <c r="N29" s="65"/>
-      <c r="O29" s="65"/>
-      <c r="P29" s="64"/>
-      <c r="Q29" s="112"/>
-      <c r="R29" s="113"/>
-      <c r="S29" s="35"/>
-      <c r="T29" s="35"/>
-      <c r="U29" s="35"/>
-      <c r="V29" s="35"/>
-      <c r="W29" s="35"/>
-      <c r="X29" s="35"/>
-      <c r="Y29" s="35"/>
-      <c r="Z29" s="35"/>
-      <c r="AA29" s="105"/>
-      <c r="AB29" s="105"/>
+      <c r="AJ28" s="35"/>
+      <c r="AK28" s="43"/>
+      <c r="AL28" s="73"/>
+    </row>
+    <row r="29" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="56"/>
+      <c r="B29" s="55"/>
+      <c r="C29" s="55"/>
+      <c r="D29" s="55"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="56"/>
+      <c r="G29" s="55"/>
+      <c r="H29" s="55"/>
+      <c r="I29" s="56"/>
+      <c r="J29" s="55"/>
+      <c r="K29" s="57"/>
+      <c r="L29" s="58"/>
+      <c r="M29" s="57"/>
+      <c r="N29" s="58"/>
+      <c r="O29" s="58"/>
+      <c r="P29" s="57"/>
+      <c r="Q29" s="97"/>
+      <c r="R29" s="98"/>
+      <c r="S29" s="34"/>
+      <c r="T29" s="34"/>
+      <c r="U29" s="34"/>
+      <c r="V29" s="34"/>
+      <c r="W29" s="34"/>
+      <c r="X29" s="34"/>
+      <c r="Y29" s="34"/>
+      <c r="Z29" s="34"/>
+      <c r="AA29" s="95"/>
+      <c r="AB29" s="95"/>
       <c r="AC29" s="30"/>
       <c r="AD29" s="30"/>
       <c r="AE29" s="30"/>
@@ -3945,39 +4045,39 @@
       <c r="AG29" s="30"/>
       <c r="AH29" s="30"/>
       <c r="AI29" s="30"/>
-      <c r="AJ29" s="36"/>
-      <c r="AK29" s="46"/>
-      <c r="AL29" s="81"/>
-    </row>
-    <row r="30" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="63"/>
-      <c r="B30" s="62"/>
-      <c r="C30" s="62"/>
-      <c r="D30" s="62"/>
-      <c r="E30" s="63"/>
-      <c r="F30" s="63"/>
-      <c r="G30" s="62"/>
-      <c r="H30" s="62"/>
-      <c r="I30" s="63"/>
-      <c r="J30" s="62"/>
-      <c r="K30" s="64"/>
-      <c r="L30" s="65"/>
-      <c r="M30" s="64"/>
-      <c r="N30" s="65"/>
-      <c r="O30" s="65"/>
-      <c r="P30" s="64"/>
-      <c r="Q30" s="112"/>
-      <c r="R30" s="113"/>
-      <c r="S30" s="35"/>
-      <c r="T30" s="35"/>
-      <c r="U30" s="35"/>
-      <c r="V30" s="35"/>
-      <c r="W30" s="35"/>
-      <c r="X30" s="35"/>
-      <c r="Y30" s="35"/>
-      <c r="Z30" s="35"/>
-      <c r="AA30" s="105"/>
-      <c r="AB30" s="105"/>
+      <c r="AJ29" s="35"/>
+      <c r="AK29" s="43"/>
+      <c r="AL29" s="73"/>
+    </row>
+    <row r="30" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="56"/>
+      <c r="B30" s="55"/>
+      <c r="C30" s="55"/>
+      <c r="D30" s="55"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
+      <c r="G30" s="55"/>
+      <c r="H30" s="55"/>
+      <c r="I30" s="56"/>
+      <c r="J30" s="55"/>
+      <c r="K30" s="57"/>
+      <c r="L30" s="58"/>
+      <c r="M30" s="57"/>
+      <c r="N30" s="58"/>
+      <c r="O30" s="58"/>
+      <c r="P30" s="57"/>
+      <c r="Q30" s="97"/>
+      <c r="R30" s="98"/>
+      <c r="S30" s="34"/>
+      <c r="T30" s="34"/>
+      <c r="U30" s="34"/>
+      <c r="V30" s="34"/>
+      <c r="W30" s="34"/>
+      <c r="X30" s="34"/>
+      <c r="Y30" s="34"/>
+      <c r="Z30" s="34"/>
+      <c r="AA30" s="95"/>
+      <c r="AB30" s="95"/>
       <c r="AC30" s="30"/>
       <c r="AD30" s="30"/>
       <c r="AE30" s="30"/>
@@ -3985,36 +4085,36 @@
       <c r="AG30" s="30"/>
       <c r="AH30" s="30"/>
       <c r="AI30" s="30"/>
-      <c r="AJ30" s="36"/>
-      <c r="AK30" s="46"/>
-      <c r="AL30" s="81"/>
-    </row>
-    <row r="31" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="D31" s="65"/>
-      <c r="E31" s="65"/>
-      <c r="F31" s="65"/>
-      <c r="G31" s="65"/>
-      <c r="H31" s="65"/>
-      <c r="I31" s="65"/>
-      <c r="J31" s="65"/>
-      <c r="K31" s="64"/>
-      <c r="L31" s="65"/>
-      <c r="M31" s="64"/>
-      <c r="N31" s="65"/>
-      <c r="O31" s="65"/>
-      <c r="P31" s="64"/>
-      <c r="Q31" s="112"/>
-      <c r="R31" s="113"/>
-      <c r="S31" s="35"/>
-      <c r="T31" s="35"/>
-      <c r="U31" s="35"/>
-      <c r="V31" s="35"/>
-      <c r="W31" s="35"/>
-      <c r="X31" s="35"/>
-      <c r="Y31" s="35"/>
-      <c r="Z31" s="35"/>
-      <c r="AA31" s="105"/>
-      <c r="AB31" s="105"/>
+      <c r="AJ30" s="35"/>
+      <c r="AK30" s="43"/>
+      <c r="AL30" s="73"/>
+    </row>
+    <row r="31" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D31" s="58"/>
+      <c r="E31" s="58"/>
+      <c r="F31" s="58"/>
+      <c r="G31" s="58"/>
+      <c r="H31" s="58"/>
+      <c r="I31" s="58"/>
+      <c r="J31" s="58"/>
+      <c r="K31" s="57"/>
+      <c r="L31" s="58"/>
+      <c r="M31" s="57"/>
+      <c r="N31" s="58"/>
+      <c r="O31" s="58"/>
+      <c r="P31" s="57"/>
+      <c r="Q31" s="97"/>
+      <c r="R31" s="98"/>
+      <c r="S31" s="34"/>
+      <c r="T31" s="34"/>
+      <c r="U31" s="34"/>
+      <c r="V31" s="34"/>
+      <c r="W31" s="34"/>
+      <c r="X31" s="34"/>
+      <c r="Y31" s="34"/>
+      <c r="Z31" s="34"/>
+      <c r="AA31" s="95"/>
+      <c r="AB31" s="95"/>
       <c r="AC31" s="30"/>
       <c r="AD31" s="30"/>
       <c r="AE31" s="30"/>
@@ -4022,34 +4122,34 @@
       <c r="AG31" s="30"/>
       <c r="AH31" s="30"/>
       <c r="AI31" s="30"/>
-      <c r="AJ31" s="36"/>
-      <c r="AK31" s="46"/>
-      <c r="AL31" s="81"/>
-    </row>
-    <row r="32" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="D32" s="62"/>
-      <c r="E32" s="62"/>
-      <c r="F32" s="62"/>
-      <c r="G32" s="62"/>
-      <c r="H32" s="62"/>
-      <c r="I32" s="65"/>
-      <c r="J32" s="133"/>
-      <c r="K32" s="64"/>
-      <c r="L32" s="64"/>
-      <c r="M32" s="64"/>
-      <c r="N32" s="64"/>
-      <c r="O32" s="64"/>
-      <c r="P32" s="64"/>
-      <c r="Q32" s="37"/>
+      <c r="AJ31" s="35"/>
+      <c r="AK31" s="43"/>
+      <c r="AL31" s="73"/>
+    </row>
+    <row r="32" spans="1:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D32" s="55"/>
+      <c r="E32" s="55"/>
+      <c r="F32" s="55"/>
+      <c r="G32" s="55"/>
+      <c r="H32" s="55"/>
+      <c r="I32" s="58"/>
+      <c r="J32" s="90"/>
+      <c r="K32" s="57"/>
+      <c r="L32" s="57"/>
+      <c r="M32" s="57"/>
+      <c r="N32" s="57"/>
+      <c r="O32" s="57"/>
+      <c r="P32" s="57"/>
+      <c r="Q32" s="36"/>
       <c r="R32" s="33"/>
-      <c r="S32" s="35"/>
-      <c r="T32" s="35"/>
-      <c r="U32" s="35"/>
-      <c r="V32" s="35"/>
-      <c r="W32" s="35"/>
-      <c r="X32" s="35"/>
-      <c r="Y32" s="35"/>
-      <c r="Z32" s="35"/>
+      <c r="S32" s="34"/>
+      <c r="T32" s="34"/>
+      <c r="U32" s="34"/>
+      <c r="V32" s="34"/>
+      <c r="W32" s="34"/>
+      <c r="X32" s="34"/>
+      <c r="Y32" s="34"/>
+      <c r="Z32" s="34"/>
       <c r="AA32" s="30"/>
       <c r="AB32" s="33"/>
       <c r="AC32" s="30"/>
@@ -4059,34 +4159,34 @@
       <c r="AG32" s="30"/>
       <c r="AH32" s="30"/>
       <c r="AI32" s="30"/>
-      <c r="AJ32" s="36"/>
-      <c r="AK32" s="46"/>
-      <c r="AL32" s="81"/>
+      <c r="AJ32" s="35"/>
+      <c r="AK32" s="43"/>
+      <c r="AL32" s="73"/>
     </row>
     <row r="33" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="D33" s="62"/>
-      <c r="E33" s="62"/>
-      <c r="F33" s="62"/>
-      <c r="G33" s="62"/>
-      <c r="H33" s="62"/>
-      <c r="I33" s="65"/>
-      <c r="J33" s="133"/>
-      <c r="K33" s="64"/>
-      <c r="L33" s="64"/>
-      <c r="M33" s="64"/>
-      <c r="N33" s="64"/>
-      <c r="O33" s="64"/>
-      <c r="P33" s="64"/>
-      <c r="Q33" s="37"/>
+      <c r="D33" s="55"/>
+      <c r="E33" s="55"/>
+      <c r="F33" s="55"/>
+      <c r="G33" s="55"/>
+      <c r="H33" s="55"/>
+      <c r="I33" s="58"/>
+      <c r="J33" s="90"/>
+      <c r="K33" s="57"/>
+      <c r="L33" s="57"/>
+      <c r="M33" s="57"/>
+      <c r="N33" s="57"/>
+      <c r="O33" s="57"/>
+      <c r="P33" s="57"/>
+      <c r="Q33" s="36"/>
       <c r="R33" s="33"/>
-      <c r="S33" s="35"/>
-      <c r="T33" s="35"/>
-      <c r="U33" s="35"/>
-      <c r="V33" s="35"/>
-      <c r="W33" s="35"/>
-      <c r="X33" s="35"/>
-      <c r="Y33" s="35"/>
-      <c r="Z33" s="35"/>
+      <c r="S33" s="34"/>
+      <c r="T33" s="34"/>
+      <c r="U33" s="34"/>
+      <c r="V33" s="34"/>
+      <c r="W33" s="34"/>
+      <c r="X33" s="34"/>
+      <c r="Y33" s="34"/>
+      <c r="Z33" s="34"/>
       <c r="AA33" s="30"/>
       <c r="AB33" s="33"/>
       <c r="AC33" s="30"/>
@@ -4096,34 +4196,34 @@
       <c r="AG33" s="30"/>
       <c r="AH33" s="30"/>
       <c r="AI33" s="30"/>
-      <c r="AJ33" s="36"/>
-      <c r="AK33" s="46"/>
-      <c r="AL33" s="81"/>
+      <c r="AJ33" s="35"/>
+      <c r="AK33" s="43"/>
+      <c r="AL33" s="73"/>
     </row>
     <row r="34" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="D34" s="65"/>
-      <c r="E34" s="65"/>
-      <c r="F34" s="65"/>
-      <c r="G34" s="65"/>
-      <c r="H34" s="65"/>
-      <c r="I34" s="65"/>
-      <c r="J34" s="65"/>
-      <c r="K34" s="64"/>
-      <c r="L34" s="64"/>
-      <c r="M34" s="64"/>
-      <c r="N34" s="64"/>
-      <c r="O34" s="64"/>
-      <c r="P34" s="64"/>
-      <c r="Q34" s="37"/>
+      <c r="D34" s="58"/>
+      <c r="E34" s="58"/>
+      <c r="F34" s="58"/>
+      <c r="G34" s="58"/>
+      <c r="H34" s="58"/>
+      <c r="I34" s="58"/>
+      <c r="J34" s="58"/>
+      <c r="K34" s="57"/>
+      <c r="L34" s="57"/>
+      <c r="M34" s="57"/>
+      <c r="N34" s="57"/>
+      <c r="O34" s="57"/>
+      <c r="P34" s="57"/>
+      <c r="Q34" s="36"/>
       <c r="R34" s="33"/>
-      <c r="S34" s="35"/>
-      <c r="T34" s="35"/>
-      <c r="U34" s="35"/>
-      <c r="V34" s="35"/>
-      <c r="W34" s="35"/>
-      <c r="X34" s="35"/>
-      <c r="Y34" s="35"/>
-      <c r="Z34" s="35"/>
+      <c r="S34" s="34"/>
+      <c r="T34" s="34"/>
+      <c r="U34" s="34"/>
+      <c r="V34" s="34"/>
+      <c r="W34" s="34"/>
+      <c r="X34" s="34"/>
+      <c r="Y34" s="34"/>
+      <c r="Z34" s="34"/>
       <c r="AA34" s="30"/>
       <c r="AB34" s="33"/>
       <c r="AC34" s="30"/>
@@ -4133,364 +4233,343 @@
       <c r="AG34" s="30"/>
       <c r="AH34" s="30"/>
       <c r="AI34" s="30"/>
-      <c r="AJ34" s="36"/>
-      <c r="AK34" s="46"/>
-      <c r="AL34" s="81"/>
+      <c r="AJ34" s="35"/>
+      <c r="AK34" s="43"/>
+      <c r="AL34" s="73"/>
     </row>
     <row r="35" spans="1:38" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="D35" s="66"/>
-      <c r="E35" s="67"/>
-      <c r="F35" s="65"/>
-      <c r="G35" s="65"/>
-      <c r="H35" s="65"/>
-      <c r="I35" s="65"/>
-      <c r="J35" s="65"/>
-      <c r="K35" s="64"/>
-      <c r="L35" s="64"/>
-      <c r="M35" s="64"/>
-      <c r="N35" s="64"/>
-      <c r="O35" s="64"/>
-      <c r="P35" s="64"/>
-      <c r="Q35" s="39"/>
-      <c r="R35" s="40"/>
-      <c r="S35" s="41"/>
-      <c r="T35" s="41"/>
-      <c r="U35" s="41"/>
-      <c r="V35" s="41"/>
-      <c r="W35" s="41"/>
-      <c r="X35" s="41"/>
-      <c r="Y35" s="41"/>
-      <c r="Z35" s="41"/>
-      <c r="AA35" s="42"/>
-      <c r="AB35" s="40"/>
-      <c r="AC35" s="42"/>
-      <c r="AD35" s="42"/>
-      <c r="AE35" s="42"/>
-      <c r="AF35" s="42"/>
-      <c r="AG35" s="42"/>
-      <c r="AH35" s="42"/>
-      <c r="AI35" s="42"/>
-      <c r="AJ35" s="51"/>
-      <c r="AK35" s="47"/>
-      <c r="AL35" s="81"/>
+      <c r="D35" s="59"/>
+      <c r="E35" s="60"/>
+      <c r="F35" s="58"/>
+      <c r="G35" s="58"/>
+      <c r="H35" s="58"/>
+      <c r="I35" s="58"/>
+      <c r="J35" s="58"/>
+      <c r="K35" s="57"/>
+      <c r="L35" s="57"/>
+      <c r="M35" s="57"/>
+      <c r="N35" s="57"/>
+      <c r="O35" s="57"/>
+      <c r="P35" s="57"/>
+      <c r="Q35" s="38"/>
+      <c r="R35" s="39"/>
+      <c r="S35" s="40"/>
+      <c r="T35" s="40"/>
+      <c r="U35" s="40"/>
+      <c r="V35" s="40"/>
+      <c r="W35" s="40"/>
+      <c r="X35" s="40"/>
+      <c r="Y35" s="40"/>
+      <c r="Z35" s="40"/>
+      <c r="AA35" s="41"/>
+      <c r="AB35" s="39"/>
+      <c r="AC35" s="41"/>
+      <c r="AD35" s="41"/>
+      <c r="AE35" s="41"/>
+      <c r="AF35" s="41"/>
+      <c r="AG35" s="41"/>
+      <c r="AH35" s="41"/>
+      <c r="AI35" s="41"/>
+      <c r="AJ35" s="45"/>
+      <c r="AK35" s="44"/>
+      <c r="AL35" s="73"/>
     </row>
     <row r="36" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="D36" s="68"/>
-      <c r="E36" s="69"/>
-      <c r="F36" s="64"/>
-      <c r="G36" s="64"/>
-      <c r="H36" s="64"/>
-      <c r="I36" s="64"/>
-      <c r="J36" s="120"/>
-      <c r="K36" s="64"/>
-      <c r="L36" s="64"/>
-      <c r="M36" s="64"/>
-      <c r="N36" s="64"/>
-      <c r="O36" s="64"/>
-      <c r="P36" s="64"/>
-      <c r="Q36" s="43"/>
-      <c r="R36" s="43"/>
-      <c r="S36" s="43"/>
-      <c r="T36" s="43"/>
-      <c r="U36" s="43"/>
-      <c r="V36" s="43"/>
-      <c r="W36" s="43"/>
-      <c r="X36" s="43"/>
-      <c r="Y36" s="43"/>
-      <c r="Z36" s="43"/>
-      <c r="AA36" s="43"/>
-      <c r="AB36" s="43"/>
-      <c r="AC36" s="43"/>
-      <c r="AD36" s="43"/>
-      <c r="AE36" s="43"/>
-      <c r="AF36" s="43"/>
-      <c r="AG36" s="43"/>
-      <c r="AH36" s="43"/>
-      <c r="AI36" s="43"/>
-      <c r="AJ36" s="52"/>
-      <c r="AK36" s="43"/>
-      <c r="AL36" s="43"/>
+      <c r="D36" s="61"/>
+      <c r="E36" s="62"/>
+      <c r="F36" s="57"/>
+      <c r="G36" s="57"/>
+      <c r="H36" s="57"/>
+      <c r="I36" s="57"/>
+      <c r="J36" s="84"/>
+      <c r="K36" s="57"/>
+      <c r="L36" s="57"/>
+      <c r="M36" s="57"/>
+      <c r="N36" s="57"/>
+      <c r="O36" s="57"/>
+      <c r="P36" s="57"/>
+      <c r="Q36" s="42"/>
+      <c r="R36" s="42"/>
+      <c r="S36" s="42"/>
+      <c r="T36" s="42"/>
+      <c r="U36" s="42"/>
+      <c r="V36" s="42"/>
+      <c r="W36" s="42"/>
+      <c r="X36" s="42"/>
+      <c r="Y36" s="42"/>
+      <c r="Z36" s="42"/>
+      <c r="AA36" s="42"/>
+      <c r="AB36" s="42"/>
+      <c r="AC36" s="42"/>
+      <c r="AD36" s="42"/>
+      <c r="AE36" s="42"/>
+      <c r="AF36" s="42"/>
+      <c r="AG36" s="42"/>
+      <c r="AH36" s="42"/>
+      <c r="AI36" s="42"/>
+      <c r="AJ36" s="46"/>
+      <c r="AK36" s="42"/>
+      <c r="AL36" s="42"/>
     </row>
     <row r="37" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="D37" s="68"/>
-      <c r="E37" s="69"/>
-      <c r="F37" s="64"/>
-      <c r="G37" s="64"/>
-      <c r="H37" s="64"/>
-      <c r="I37" s="64"/>
-      <c r="J37" s="120"/>
-      <c r="K37" s="64"/>
-      <c r="L37" s="64"/>
-      <c r="M37" s="64"/>
-      <c r="N37" s="64"/>
-      <c r="O37" s="64"/>
-      <c r="P37" s="64"/>
-      <c r="Q37" s="43"/>
-      <c r="R37" s="43"/>
-      <c r="S37" s="43"/>
-      <c r="T37" s="43"/>
-      <c r="U37" s="43"/>
-      <c r="V37" s="43"/>
-      <c r="W37" s="43"/>
-      <c r="X37" s="43"/>
-      <c r="Y37" s="43"/>
-      <c r="Z37" s="43"/>
-      <c r="AA37" s="43"/>
-      <c r="AB37" s="43"/>
-      <c r="AC37" s="43"/>
-      <c r="AD37" s="43"/>
-      <c r="AE37" s="43"/>
-      <c r="AF37" s="43"/>
-      <c r="AG37" s="43"/>
-      <c r="AH37" s="43"/>
-      <c r="AI37" s="43"/>
-      <c r="AJ37" s="52"/>
-      <c r="AK37" s="43"/>
-      <c r="AL37" s="43"/>
+      <c r="D37" s="61"/>
+      <c r="E37" s="62"/>
+      <c r="F37" s="57"/>
+      <c r="G37" s="57"/>
+      <c r="H37" s="57"/>
+      <c r="I37" s="57"/>
+      <c r="J37" s="84"/>
+      <c r="K37" s="57"/>
+      <c r="L37" s="57"/>
+      <c r="M37" s="57"/>
+      <c r="N37" s="57"/>
+      <c r="O37" s="57"/>
+      <c r="P37" s="57"/>
+      <c r="Q37" s="42"/>
+      <c r="R37" s="42"/>
+      <c r="S37" s="42"/>
+      <c r="T37" s="42"/>
+      <c r="U37" s="42"/>
+      <c r="V37" s="42"/>
+      <c r="W37" s="42"/>
+      <c r="X37" s="42"/>
+      <c r="Y37" s="42"/>
+      <c r="Z37" s="42"/>
+      <c r="AA37" s="42"/>
+      <c r="AB37" s="42"/>
+      <c r="AC37" s="42"/>
+      <c r="AD37" s="42"/>
+      <c r="AE37" s="42"/>
+      <c r="AF37" s="42"/>
+      <c r="AG37" s="42"/>
+      <c r="AH37" s="42"/>
+      <c r="AI37" s="42"/>
+      <c r="AJ37" s="46"/>
+      <c r="AK37" s="42"/>
+      <c r="AL37" s="42"/>
     </row>
     <row r="38" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="D38" s="63"/>
-      <c r="E38" s="63"/>
-      <c r="F38" s="63"/>
-      <c r="G38" s="63"/>
-      <c r="H38" s="63"/>
-      <c r="I38" s="63"/>
-      <c r="J38" s="63"/>
-      <c r="K38" s="70"/>
-      <c r="L38" s="64"/>
-      <c r="M38" s="71"/>
-      <c r="N38" s="64"/>
-      <c r="O38" s="64"/>
-      <c r="P38" s="72"/>
-      <c r="Q38" s="43"/>
-      <c r="R38" s="43"/>
-      <c r="S38" s="43"/>
-      <c r="T38" s="43"/>
-      <c r="U38" s="43"/>
-      <c r="V38" s="43"/>
-      <c r="W38" s="43"/>
-      <c r="X38" s="43"/>
-      <c r="Y38" s="43"/>
-      <c r="Z38" s="43"/>
-      <c r="AA38" s="43"/>
-      <c r="AB38" s="43"/>
-      <c r="AC38" s="43"/>
-      <c r="AD38" s="43"/>
-      <c r="AE38" s="43"/>
-      <c r="AF38" s="43"/>
-      <c r="AG38" s="43"/>
-      <c r="AH38" s="43"/>
-      <c r="AI38" s="43"/>
-      <c r="AJ38" s="52"/>
-      <c r="AK38" s="43"/>
-      <c r="AL38" s="43"/>
+      <c r="D38" s="56"/>
+      <c r="E38" s="56"/>
+      <c r="F38" s="56"/>
+      <c r="G38" s="56"/>
+      <c r="H38" s="56"/>
+      <c r="I38" s="56"/>
+      <c r="J38" s="56"/>
+      <c r="K38" s="63"/>
+      <c r="L38" s="57"/>
+      <c r="M38" s="64"/>
+      <c r="N38" s="57"/>
+      <c r="O38" s="57"/>
+      <c r="P38" s="65"/>
+      <c r="Q38" s="42"/>
+      <c r="R38" s="42"/>
+      <c r="S38" s="42"/>
+      <c r="T38" s="42"/>
+      <c r="U38" s="42"/>
+      <c r="V38" s="42"/>
+      <c r="W38" s="42"/>
+      <c r="X38" s="42"/>
+      <c r="Y38" s="42"/>
+      <c r="Z38" s="42"/>
+      <c r="AA38" s="42"/>
+      <c r="AB38" s="42"/>
+      <c r="AC38" s="42"/>
+      <c r="AD38" s="42"/>
+      <c r="AE38" s="42"/>
+      <c r="AF38" s="42"/>
+      <c r="AG38" s="42"/>
+      <c r="AH38" s="42"/>
+      <c r="AI38" s="42"/>
+      <c r="AJ38" s="46"/>
+      <c r="AK38" s="42"/>
+      <c r="AL38" s="42"/>
     </row>
     <row r="39" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="60"/>
-      <c r="C39" s="63"/>
-      <c r="D39" s="63"/>
-      <c r="E39" s="63"/>
-      <c r="F39" s="63"/>
-      <c r="G39" s="63"/>
-      <c r="H39" s="63"/>
-      <c r="I39" s="63"/>
-      <c r="J39" s="63"/>
-      <c r="K39" s="70"/>
-      <c r="L39" s="64"/>
-      <c r="M39" s="71"/>
-      <c r="N39" s="64"/>
-      <c r="O39" s="64"/>
-      <c r="P39" s="72"/>
-      <c r="Q39" s="43"/>
-      <c r="R39" s="43"/>
-      <c r="S39" s="43"/>
-      <c r="T39" s="43"/>
-      <c r="U39" s="43"/>
-      <c r="V39" s="43"/>
-      <c r="W39" s="43"/>
-      <c r="X39" s="43"/>
-      <c r="Y39" s="43"/>
-      <c r="Z39" s="43"/>
-      <c r="AA39" s="43"/>
-      <c r="AB39" s="43"/>
-      <c r="AC39" s="43"/>
-      <c r="AD39" s="43"/>
-      <c r="AE39" s="43"/>
-      <c r="AF39" s="43"/>
-      <c r="AG39" s="43"/>
-      <c r="AH39" s="43"/>
-      <c r="AI39" s="43"/>
-      <c r="AJ39" s="52"/>
-      <c r="AK39" s="43"/>
-      <c r="AL39" s="43"/>
+      <c r="A39" s="53"/>
+      <c r="C39" s="56"/>
+      <c r="D39" s="56"/>
+      <c r="E39" s="56"/>
+      <c r="F39" s="56"/>
+      <c r="G39" s="56"/>
+      <c r="H39" s="56"/>
+      <c r="I39" s="56"/>
+      <c r="J39" s="56"/>
+      <c r="K39" s="63"/>
+      <c r="L39" s="57"/>
+      <c r="M39" s="64"/>
+      <c r="N39" s="57"/>
+      <c r="O39" s="57"/>
+      <c r="P39" s="65"/>
+      <c r="Q39" s="42"/>
+      <c r="R39" s="42"/>
+      <c r="S39" s="42"/>
+      <c r="T39" s="42"/>
+      <c r="U39" s="42"/>
+      <c r="V39" s="42"/>
+      <c r="W39" s="42"/>
+      <c r="X39" s="42"/>
+      <c r="Y39" s="42"/>
+      <c r="Z39" s="42"/>
+      <c r="AA39" s="42"/>
+      <c r="AB39" s="42"/>
+      <c r="AC39" s="42"/>
+      <c r="AD39" s="42"/>
+      <c r="AE39" s="42"/>
+      <c r="AF39" s="42"/>
+      <c r="AG39" s="42"/>
+      <c r="AH39" s="42"/>
+      <c r="AI39" s="42"/>
+      <c r="AJ39" s="46"/>
+      <c r="AK39" s="42"/>
+      <c r="AL39" s="42"/>
     </row>
     <row r="40" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="60"/>
-      <c r="C40" s="63"/>
-      <c r="D40" s="63"/>
-      <c r="E40" s="63"/>
-      <c r="F40" s="63"/>
-      <c r="G40" s="63"/>
-      <c r="H40" s="63"/>
-      <c r="I40" s="63"/>
-      <c r="J40" s="63"/>
-      <c r="K40" s="66"/>
-      <c r="L40" s="64"/>
-      <c r="M40" s="71"/>
-      <c r="N40" s="64"/>
-      <c r="O40" s="64"/>
-      <c r="P40" s="72"/>
-      <c r="Q40" s="43"/>
-      <c r="R40" s="43"/>
-      <c r="S40" s="43"/>
-      <c r="T40" s="43"/>
-      <c r="U40" s="43"/>
-      <c r="V40" s="43"/>
-      <c r="W40" s="43"/>
-      <c r="X40" s="43"/>
-      <c r="Y40" s="43"/>
-      <c r="Z40" s="43"/>
-      <c r="AA40" s="43"/>
-      <c r="AB40" s="43"/>
-      <c r="AC40" s="43"/>
-      <c r="AD40" s="43"/>
-      <c r="AE40" s="43"/>
-      <c r="AF40" s="43"/>
-      <c r="AG40" s="43"/>
-      <c r="AH40" s="43"/>
-      <c r="AI40" s="43"/>
-      <c r="AJ40" s="52"/>
-      <c r="AK40" s="43"/>
-      <c r="AL40" s="43"/>
+      <c r="A40" s="53"/>
+      <c r="C40" s="56"/>
+      <c r="D40" s="56"/>
+      <c r="E40" s="56"/>
+      <c r="F40" s="56"/>
+      <c r="G40" s="56"/>
+      <c r="H40" s="56"/>
+      <c r="I40" s="56"/>
+      <c r="J40" s="56"/>
+      <c r="K40" s="59"/>
+      <c r="L40" s="57"/>
+      <c r="M40" s="64"/>
+      <c r="N40" s="57"/>
+      <c r="O40" s="57"/>
+      <c r="P40" s="65"/>
+      <c r="Q40" s="42"/>
+      <c r="R40" s="42"/>
+      <c r="S40" s="42"/>
+      <c r="T40" s="42"/>
+      <c r="U40" s="42"/>
+      <c r="V40" s="42"/>
+      <c r="W40" s="42"/>
+      <c r="X40" s="42"/>
+      <c r="Y40" s="42"/>
+      <c r="Z40" s="42"/>
+      <c r="AA40" s="42"/>
+      <c r="AB40" s="42"/>
+      <c r="AC40" s="42"/>
+      <c r="AD40" s="42"/>
+      <c r="AE40" s="42"/>
+      <c r="AF40" s="42"/>
+      <c r="AG40" s="42"/>
+      <c r="AH40" s="42"/>
+      <c r="AI40" s="42"/>
+      <c r="AJ40" s="46"/>
+      <c r="AK40" s="42"/>
+      <c r="AL40" s="42"/>
     </row>
     <row r="41" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="60"/>
-      <c r="B41" s="62"/>
-      <c r="C41" s="63"/>
-      <c r="D41" s="63"/>
-      <c r="E41" s="63"/>
-      <c r="F41" s="63"/>
-      <c r="G41" s="63"/>
-      <c r="H41" s="63"/>
-      <c r="I41" s="63"/>
-      <c r="J41" s="63"/>
-      <c r="K41" s="70"/>
-      <c r="L41" s="64"/>
-      <c r="M41" s="71"/>
-      <c r="N41" s="64"/>
-      <c r="O41" s="64"/>
-      <c r="P41" s="72"/>
-      <c r="Q41" s="43"/>
-      <c r="R41" s="43"/>
-      <c r="S41" s="43"/>
-      <c r="T41" s="43"/>
-      <c r="U41" s="43"/>
-      <c r="V41" s="43"/>
-      <c r="W41" s="43"/>
-      <c r="X41" s="43"/>
-      <c r="Y41" s="43"/>
-      <c r="Z41" s="43"/>
-      <c r="AA41" s="43"/>
-      <c r="AB41" s="43"/>
-      <c r="AC41" s="43"/>
-      <c r="AD41" s="43"/>
-      <c r="AE41" s="43"/>
-      <c r="AF41" s="43"/>
-      <c r="AG41" s="43"/>
-      <c r="AH41" s="43"/>
-      <c r="AI41" s="43"/>
-      <c r="AJ41" s="52"/>
-      <c r="AK41" s="43"/>
-      <c r="AL41" s="43"/>
+      <c r="A41" s="53"/>
+      <c r="B41" s="55"/>
+      <c r="C41" s="56"/>
+      <c r="D41" s="56"/>
+      <c r="E41" s="56"/>
+      <c r="F41" s="56"/>
+      <c r="G41" s="56"/>
+      <c r="H41" s="56"/>
+      <c r="I41" s="56"/>
+      <c r="J41" s="56"/>
+      <c r="K41" s="63"/>
+      <c r="L41" s="57"/>
+      <c r="M41" s="64"/>
+      <c r="N41" s="57"/>
+      <c r="O41" s="57"/>
+      <c r="P41" s="65"/>
+      <c r="Q41" s="42"/>
+      <c r="R41" s="42"/>
+      <c r="S41" s="42"/>
+      <c r="T41" s="42"/>
+      <c r="U41" s="42"/>
+      <c r="V41" s="42"/>
+      <c r="W41" s="42"/>
+      <c r="X41" s="42"/>
+      <c r="Y41" s="42"/>
+      <c r="Z41" s="42"/>
+      <c r="AA41" s="42"/>
+      <c r="AB41" s="42"/>
+      <c r="AC41" s="42"/>
+      <c r="AD41" s="42"/>
+      <c r="AE41" s="42"/>
+      <c r="AF41" s="42"/>
+      <c r="AG41" s="42"/>
+      <c r="AH41" s="42"/>
+      <c r="AI41" s="42"/>
+      <c r="AJ41" s="46"/>
+      <c r="AK41" s="42"/>
+      <c r="AL41" s="42"/>
     </row>
     <row r="42" spans="1:38" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="61"/>
-      <c r="C42" s="63"/>
-      <c r="D42" s="63"/>
-      <c r="E42" s="63"/>
-      <c r="F42" s="63"/>
-      <c r="G42" s="63"/>
-      <c r="H42" s="63"/>
-      <c r="I42" s="63"/>
-      <c r="J42" s="63"/>
-      <c r="K42" s="67"/>
-      <c r="L42" s="64"/>
-      <c r="M42" s="71"/>
-      <c r="N42" s="64"/>
-      <c r="O42" s="64"/>
-      <c r="P42" s="72"/>
-      <c r="Q42" s="53"/>
-      <c r="R42" s="53"/>
-      <c r="S42" s="53"/>
-      <c r="T42" s="53"/>
-      <c r="U42" s="53"/>
-      <c r="V42" s="53"/>
-      <c r="W42" s="53"/>
-      <c r="X42" s="53"/>
-      <c r="Y42" s="53"/>
-      <c r="Z42" s="53"/>
-      <c r="AA42" s="53"/>
-      <c r="AB42" s="53"/>
-      <c r="AC42" s="53"/>
-      <c r="AD42" s="53"/>
-      <c r="AE42" s="53"/>
-      <c r="AF42" s="53"/>
-      <c r="AG42" s="53"/>
-      <c r="AH42" s="53"/>
-      <c r="AI42" s="53"/>
-      <c r="AJ42" s="54"/>
-      <c r="AK42" s="43"/>
-      <c r="AL42" s="43"/>
+      <c r="A42" s="54"/>
+      <c r="C42" s="56"/>
+      <c r="D42" s="56"/>
+      <c r="E42" s="56"/>
+      <c r="F42" s="56"/>
+      <c r="G42" s="56"/>
+      <c r="H42" s="56"/>
+      <c r="I42" s="56"/>
+      <c r="J42" s="56"/>
+      <c r="K42" s="60"/>
+      <c r="L42" s="57"/>
+      <c r="M42" s="64"/>
+      <c r="N42" s="57"/>
+      <c r="O42" s="57"/>
+      <c r="P42" s="65"/>
+      <c r="Q42" s="47"/>
+      <c r="R42" s="47"/>
+      <c r="S42" s="47"/>
+      <c r="T42" s="47"/>
+      <c r="U42" s="47"/>
+      <c r="V42" s="47"/>
+      <c r="W42" s="47"/>
+      <c r="X42" s="47"/>
+      <c r="Y42" s="47"/>
+      <c r="Z42" s="47"/>
+      <c r="AA42" s="47"/>
+      <c r="AB42" s="47"/>
+      <c r="AC42" s="47"/>
+      <c r="AD42" s="47"/>
+      <c r="AE42" s="47"/>
+      <c r="AF42" s="47"/>
+      <c r="AG42" s="47"/>
+      <c r="AH42" s="47"/>
+      <c r="AI42" s="47"/>
+      <c r="AJ42" s="48"/>
+      <c r="AK42" s="42"/>
+      <c r="AL42" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="71">
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="M16:O17"/>
-    <mergeCell ref="M6:O6"/>
+  <mergeCells count="78">
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="AN7:AN10"/>
+    <mergeCell ref="AN11:AN12"/>
+    <mergeCell ref="AQ14:AQ15"/>
+    <mergeCell ref="AQ17:AQ18"/>
+    <mergeCell ref="M14:O15"/>
+    <mergeCell ref="P14:P15"/>
+    <mergeCell ref="P7:P11"/>
+    <mergeCell ref="A3:E5"/>
+    <mergeCell ref="A1:P2"/>
+    <mergeCell ref="A7:A18"/>
     <mergeCell ref="M7:O11"/>
     <mergeCell ref="M12:O12"/>
     <mergeCell ref="M13:O13"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="J36:J37"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="B7:B15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="B18:B22"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="C18:C25"/>
-    <mergeCell ref="A7:A17"/>
-    <mergeCell ref="A18:A25"/>
-    <mergeCell ref="C11:J12"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="J32:J33"/>
-    <mergeCell ref="AA31:AB31"/>
-    <mergeCell ref="AA30:AB30"/>
-    <mergeCell ref="AA27:AB27"/>
-    <mergeCell ref="AA28:AB28"/>
-    <mergeCell ref="F3:J4"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="Q31:R31"/>
-    <mergeCell ref="Q27:R27"/>
-    <mergeCell ref="Q28:R28"/>
-    <mergeCell ref="Q29:R29"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="Z16:Z17"/>
-    <mergeCell ref="U16:U17"/>
-    <mergeCell ref="P16:P17"/>
-    <mergeCell ref="Q30:R30"/>
-    <mergeCell ref="AA29:AB29"/>
-    <mergeCell ref="V16:V17"/>
-    <mergeCell ref="AA16:AA17"/>
-    <mergeCell ref="Q16:Q17"/>
-    <mergeCell ref="R16:R17"/>
-    <mergeCell ref="AB16:AB17"/>
-    <mergeCell ref="AK4:AK6"/>
-    <mergeCell ref="AK16:AK17"/>
-    <mergeCell ref="AI16:AI17"/>
-    <mergeCell ref="AG16:AG17"/>
-    <mergeCell ref="AH16:AH17"/>
-    <mergeCell ref="AJ16:AJ17"/>
+    <mergeCell ref="M17:O18"/>
+    <mergeCell ref="M4:AP4"/>
+    <mergeCell ref="M5:AP5"/>
+    <mergeCell ref="K3:AP3"/>
+    <mergeCell ref="B7:B16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="AE1:AF1"/>
+    <mergeCell ref="AE2:AF2"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="K4:L4"/>
     <mergeCell ref="AE16:AE17"/>
     <mergeCell ref="AF16:AF17"/>
     <mergeCell ref="S16:S17"/>
@@ -4500,21 +4579,49 @@
     <mergeCell ref="Y16:Y17"/>
     <mergeCell ref="AD16:AD17"/>
     <mergeCell ref="AC16:AC17"/>
-    <mergeCell ref="A3:E5"/>
-    <mergeCell ref="K3:P3"/>
-    <mergeCell ref="A1:P2"/>
-    <mergeCell ref="AE1:AF1"/>
-    <mergeCell ref="AE2:AF2"/>
-    <mergeCell ref="AC5:AJ5"/>
-    <mergeCell ref="AC4:AJ4"/>
-    <mergeCell ref="F5:J5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="Q4:AB4"/>
-    <mergeCell ref="Q5:AB5"/>
-    <mergeCell ref="M5:P5"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:P4"/>
-    <mergeCell ref="P7:P11"/>
+    <mergeCell ref="AK16:AK17"/>
+    <mergeCell ref="AI16:AI17"/>
+    <mergeCell ref="AG16:AG17"/>
+    <mergeCell ref="AH16:AH17"/>
+    <mergeCell ref="AJ16:AJ17"/>
+    <mergeCell ref="AA29:AB29"/>
+    <mergeCell ref="V16:V17"/>
+    <mergeCell ref="AA16:AA17"/>
+    <mergeCell ref="Q16:Q17"/>
+    <mergeCell ref="R16:R17"/>
+    <mergeCell ref="AB16:AB17"/>
+    <mergeCell ref="AA31:AB31"/>
+    <mergeCell ref="AA30:AB30"/>
+    <mergeCell ref="AA27:AB27"/>
+    <mergeCell ref="AA28:AB28"/>
+    <mergeCell ref="F3:J4"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="Q31:R31"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="Q28:R28"/>
+    <mergeCell ref="Q29:R29"/>
+    <mergeCell ref="U19:U20"/>
+    <mergeCell ref="Z16:Z17"/>
+    <mergeCell ref="U16:U17"/>
+    <mergeCell ref="Q30:R30"/>
+    <mergeCell ref="M16:O16"/>
+    <mergeCell ref="M6:O6"/>
+    <mergeCell ref="J36:J37"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="C11:J12"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="J32:J33"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="C19:C26"/>
+    <mergeCell ref="A19:A26"/>
+    <mergeCell ref="B19:B23"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4548,89 +4655,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="154" t="s">
+      <c r="A1" s="142" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="155"/>
-      <c r="C1" s="155"/>
-      <c r="D1" s="155"/>
-      <c r="E1" s="155"/>
-      <c r="F1" s="155"/>
-      <c r="G1" s="155"/>
-      <c r="H1" s="155"/>
-      <c r="I1" s="155"/>
-      <c r="J1" s="155"/>
-      <c r="K1" s="155"/>
-      <c r="L1" s="155"/>
-      <c r="M1" s="92" t="s">
+      <c r="B1" s="143"/>
+      <c r="C1" s="143"/>
+      <c r="D1" s="143"/>
+      <c r="E1" s="143"/>
+      <c r="F1" s="143"/>
+      <c r="G1" s="143"/>
+      <c r="H1" s="143"/>
+      <c r="I1" s="143"/>
+      <c r="J1" s="143"/>
+      <c r="K1" s="143"/>
+      <c r="L1" s="143"/>
+      <c r="M1" s="104" t="s">
         <v>49</v>
       </c>
-      <c r="N1" s="92"/>
-      <c r="O1" s="92" t="s">
+      <c r="N1" s="104"/>
+      <c r="O1" s="104" t="s">
         <v>51</v>
       </c>
-      <c r="P1" s="152"/>
+      <c r="P1" s="140"/>
     </row>
     <row r="2" spans="1:16" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="156"/>
-      <c r="B2" s="157"/>
-      <c r="C2" s="157"/>
-      <c r="D2" s="157"/>
-      <c r="E2" s="157"/>
-      <c r="F2" s="157"/>
-      <c r="G2" s="157"/>
-      <c r="H2" s="157"/>
-      <c r="I2" s="157"/>
-      <c r="J2" s="157"/>
-      <c r="K2" s="157"/>
-      <c r="L2" s="157"/>
-      <c r="M2" s="93" t="s">
+      <c r="A2" s="144"/>
+      <c r="B2" s="145"/>
+      <c r="C2" s="145"/>
+      <c r="D2" s="145"/>
+      <c r="E2" s="145"/>
+      <c r="F2" s="145"/>
+      <c r="G2" s="145"/>
+      <c r="H2" s="145"/>
+      <c r="I2" s="145"/>
+      <c r="J2" s="145"/>
+      <c r="K2" s="145"/>
+      <c r="L2" s="145"/>
+      <c r="M2" s="105" t="s">
         <v>50</v>
       </c>
-      <c r="N2" s="93"/>
-      <c r="O2" s="93"/>
-      <c r="P2" s="153"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="105"/>
+      <c r="P2" s="141"/>
     </row>
     <row r="3" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.45"/>
     <row r="4" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A4" s="158" t="s">
+      <c r="A4" s="146" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="159"/>
-      <c r="C4" s="159"/>
-      <c r="D4" s="160"/>
-      <c r="E4" s="161" t="s">
+      <c r="B4" s="147"/>
+      <c r="C4" s="147"/>
+      <c r="D4" s="148"/>
+      <c r="E4" s="149" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="160"/>
-      <c r="G4" s="161" t="s">
+      <c r="F4" s="148"/>
+      <c r="G4" s="149" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="160"/>
-      <c r="I4" s="161" t="s">
+      <c r="H4" s="148"/>
+      <c r="I4" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="160"/>
-      <c r="K4" s="161" t="s">
+      <c r="J4" s="148"/>
+      <c r="K4" s="149" t="s">
         <v>26</v>
       </c>
-      <c r="L4" s="160"/>
+      <c r="L4" s="148"/>
       <c r="M4" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="161" t="s">
+      <c r="N4" s="149" t="s">
         <v>28</v>
       </c>
-      <c r="O4" s="160"/>
-      <c r="P4" s="143" t="s">
+      <c r="O4" s="148"/>
+      <c r="P4" s="131" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="145" t="s">
+      <c r="A5" s="133" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="146"/>
+      <c r="B5" s="134"/>
       <c r="C5" s="15" t="s">
         <v>0</v>
       </c>
@@ -4670,10 +4777,10 @@
       <c r="O5" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="P5" s="144"/>
+      <c r="P5" s="132"/>
     </row>
     <row r="6" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="147" t="s">
+      <c r="A6" s="135" t="s">
         <v>36</v>
       </c>
       <c r="B6" s="11" t="s">
@@ -4703,8 +4810,8 @@
       <c r="P6" s="6"/>
     </row>
     <row r="7" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="147"/>
-      <c r="B7" s="140" t="s">
+      <c r="A7" s="135"/>
+      <c r="B7" s="121" t="s">
         <v>53</v>
       </c>
       <c r="C7" s="5" t="s">
@@ -4713,47 +4820,47 @@
       <c r="D7" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="136"/>
-      <c r="F7" s="136"/>
-      <c r="G7" s="142" t="s">
+      <c r="E7" s="150"/>
+      <c r="F7" s="150"/>
+      <c r="G7" s="152" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="140" t="s">
+      <c r="H7" s="121" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="136"/>
-      <c r="J7" s="136"/>
-      <c r="K7" s="136"/>
-      <c r="L7" s="136"/>
-      <c r="M7" s="136"/>
-      <c r="N7" s="136"/>
-      <c r="O7" s="136"/>
-      <c r="P7" s="134"/>
+      <c r="I7" s="150"/>
+      <c r="J7" s="150"/>
+      <c r="K7" s="150"/>
+      <c r="L7" s="150"/>
+      <c r="M7" s="150"/>
+      <c r="N7" s="150"/>
+      <c r="O7" s="150"/>
+      <c r="P7" s="153"/>
     </row>
     <row r="8" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="148"/>
-      <c r="B8" s="141"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="123"/>
       <c r="C8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="137"/>
-      <c r="F8" s="137"/>
-      <c r="G8" s="142"/>
-      <c r="H8" s="141"/>
-      <c r="I8" s="137"/>
-      <c r="J8" s="137"/>
-      <c r="K8" s="137"/>
-      <c r="L8" s="137"/>
-      <c r="M8" s="137"/>
-      <c r="N8" s="137"/>
-      <c r="O8" s="137"/>
-      <c r="P8" s="135"/>
+      <c r="E8" s="151"/>
+      <c r="F8" s="151"/>
+      <c r="G8" s="152"/>
+      <c r="H8" s="123"/>
+      <c r="I8" s="151"/>
+      <c r="J8" s="151"/>
+      <c r="K8" s="151"/>
+      <c r="L8" s="151"/>
+      <c r="M8" s="151"/>
+      <c r="N8" s="151"/>
+      <c r="O8" s="151"/>
+      <c r="P8" s="154"/>
     </row>
     <row r="9" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="148"/>
+      <c r="A9" s="136"/>
       <c r="B9" s="16" t="s">
         <v>54</v>
       </c>
@@ -4781,8 +4888,8 @@
       <c r="P9" s="2"/>
     </row>
     <row r="10" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="148"/>
-      <c r="B10" s="140" t="s">
+      <c r="A10" s="136"/>
+      <c r="B10" s="121" t="s">
         <v>56</v>
       </c>
       <c r="C10" s="9" t="s">
@@ -4791,47 +4898,47 @@
       <c r="D10" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="136"/>
-      <c r="F10" s="136"/>
-      <c r="G10" s="138" t="s">
+      <c r="E10" s="150"/>
+      <c r="F10" s="150"/>
+      <c r="G10" s="155" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="140" t="s">
+      <c r="H10" s="121" t="s">
         <v>41</v>
       </c>
-      <c r="I10" s="136"/>
-      <c r="J10" s="136"/>
-      <c r="K10" s="136"/>
-      <c r="L10" s="136"/>
-      <c r="M10" s="136"/>
-      <c r="N10" s="136"/>
-      <c r="O10" s="136"/>
-      <c r="P10" s="134"/>
+      <c r="I10" s="150"/>
+      <c r="J10" s="150"/>
+      <c r="K10" s="150"/>
+      <c r="L10" s="150"/>
+      <c r="M10" s="150"/>
+      <c r="N10" s="150"/>
+      <c r="O10" s="150"/>
+      <c r="P10" s="153"/>
     </row>
     <row r="11" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="148"/>
-      <c r="B11" s="141"/>
+      <c r="A11" s="136"/>
+      <c r="B11" s="123"/>
       <c r="C11" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="137"/>
-      <c r="F11" s="137"/>
-      <c r="G11" s="139"/>
-      <c r="H11" s="141"/>
-      <c r="I11" s="137"/>
-      <c r="J11" s="137"/>
-      <c r="K11" s="137"/>
-      <c r="L11" s="137"/>
-      <c r="M11" s="137"/>
-      <c r="N11" s="137"/>
-      <c r="O11" s="137"/>
-      <c r="P11" s="135"/>
+      <c r="E11" s="151"/>
+      <c r="F11" s="151"/>
+      <c r="G11" s="156"/>
+      <c r="H11" s="123"/>
+      <c r="I11" s="151"/>
+      <c r="J11" s="151"/>
+      <c r="K11" s="151"/>
+      <c r="L11" s="151"/>
+      <c r="M11" s="151"/>
+      <c r="N11" s="151"/>
+      <c r="O11" s="151"/>
+      <c r="P11" s="154"/>
     </row>
     <row r="12" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="148"/>
+      <c r="A12" s="136"/>
       <c r="B12" s="12" t="s">
         <v>55</v>
       </c>
@@ -4859,7 +4966,7 @@
       <c r="P12" s="2"/>
     </row>
     <row r="13" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="149"/>
+      <c r="A13" s="137"/>
       <c r="B13" s="12" t="s">
         <v>57</v>
       </c>
@@ -4887,7 +4994,7 @@
       <c r="P13" s="2"/>
     </row>
     <row r="14" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="150" t="s">
+      <c r="A14" s="138" t="s">
         <v>37</v>
       </c>
       <c r="B14" s="12" t="s">
@@ -4917,7 +5024,7 @@
       <c r="P14" s="2"/>
     </row>
     <row r="15" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="148"/>
+      <c r="A15" s="136"/>
       <c r="B15" s="12" t="s">
         <v>58</v>
       </c>
@@ -4945,7 +5052,7 @@
       <c r="P15" s="2"/>
     </row>
     <row r="16" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="148"/>
+      <c r="A16" s="136"/>
       <c r="B16" s="12" t="s">
         <v>60</v>
       </c>
@@ -4973,7 +5080,7 @@
       <c r="P16" s="2"/>
     </row>
     <row r="17" spans="1:16" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="151"/>
+      <c r="A17" s="139"/>
       <c r="B17" s="13" t="s">
         <v>61</v>
       </c>
@@ -5002,6 +5109,31 @@
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="P7:P8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="P10:P11"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="J10:J11"/>
+    <mergeCell ref="K10:K11"/>
+    <mergeCell ref="L10:L11"/>
+    <mergeCell ref="M10:M11"/>
+    <mergeCell ref="N10:N11"/>
+    <mergeCell ref="O10:O11"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="J7:J8"/>
     <mergeCell ref="P4:P5"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:A13"/>
@@ -5018,31 +5150,6 @@
     <mergeCell ref="N4:O4"/>
     <mergeCell ref="M2:N2"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="O7:O8"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="P7:P8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="P10:P11"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="J10:J11"/>
-    <mergeCell ref="K10:K11"/>
-    <mergeCell ref="L10:L11"/>
-    <mergeCell ref="M10:M11"/>
-    <mergeCell ref="N10:N11"/>
-    <mergeCell ref="O10:O11"/>
-    <mergeCell ref="K7:K8"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
서브 시스템 수정(external api를map api와 ai api로 분할), 컴포넌트 다잉그램 수정(view component, server component -> auth component, chat component로 수정)
</commit_message>
<xml_diff>
--- a/Document/요구사항추적표(RTM).xlsx
+++ b/Document/요구사항추적표(RTM).xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\새 폴더\FlashTalk\Document\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rlaal\Documents\FalshTalk\Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E67AA8FF-B0B3-4015-9236-2A119367586E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A15BCD-0FB6-471A-A3C5-77F07AE0432C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2768" yWindow="52" windowWidth="17745" windowHeight="12728" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="원본" sheetId="4" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="317">
   <si>
     <t>번호</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -1236,6 +1236,10 @@
   </si>
   <si>
     <t>PACK-03</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SS-05</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -2041,83 +2045,116 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="36" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="36" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2180,39 +2217,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2525,374 +2529,374 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BC42"/>
-  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="11.5" customWidth="1"/>
-    <col min="2" max="2" width="13.1875" customWidth="1"/>
-    <col min="3" max="3" width="24.6875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.1875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.1875" customWidth="1"/>
-    <col min="10" max="10" width="20.1875" customWidth="1"/>
-    <col min="11" max="11" width="12.625" style="19" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="35.625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.8125" customWidth="1"/>
-    <col min="14" max="14" width="5.875" customWidth="1"/>
-    <col min="15" max="15" width="5.8125" customWidth="1"/>
-    <col min="16" max="16" width="24.125" customWidth="1"/>
-    <col min="17" max="17" width="12.125" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="24.125" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="34.125" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="21.625" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="24.625" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="42.625" hidden="1" customWidth="1"/>
-    <col min="23" max="25" width="21.625" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="15.125" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="12.125" hidden="1" customWidth="1"/>
-    <col min="28" max="28" width="24.125" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="10.625" hidden="1" customWidth="1"/>
-    <col min="30" max="30" width="31.125" hidden="1" customWidth="1"/>
-    <col min="31" max="32" width="18.625" hidden="1" customWidth="1"/>
-    <col min="33" max="33" width="12.625" hidden="1" customWidth="1"/>
-    <col min="34" max="34" width="18.125" hidden="1" customWidth="1"/>
-    <col min="35" max="35" width="21.125" hidden="1" customWidth="1"/>
-    <col min="36" max="36" width="24.625" hidden="1" customWidth="1"/>
-    <col min="37" max="37" width="8.625" hidden="1" customWidth="1"/>
-    <col min="38" max="38" width="11.1875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.19921875" customWidth="1"/>
+    <col min="3" max="3" width="24.69921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.19921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.59765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.09765625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.19921875" customWidth="1"/>
+    <col min="10" max="10" width="20.19921875" customWidth="1"/>
+    <col min="11" max="11" width="12.59765625" style="19" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="35.59765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.796875" customWidth="1"/>
+    <col min="14" max="14" width="5.8984375" customWidth="1"/>
+    <col min="15" max="15" width="5.796875" customWidth="1"/>
+    <col min="16" max="16" width="24.09765625" customWidth="1"/>
+    <col min="17" max="17" width="12.09765625" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="24.09765625" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="34.09765625" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="21.59765625" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="24.59765625" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="42.59765625" hidden="1" customWidth="1"/>
+    <col min="23" max="25" width="21.59765625" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="15.09765625" hidden="1" customWidth="1"/>
+    <col min="27" max="27" width="12.09765625" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="24.09765625" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="10.59765625" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="31.09765625" hidden="1" customWidth="1"/>
+    <col min="31" max="32" width="18.59765625" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="12.59765625" hidden="1" customWidth="1"/>
+    <col min="34" max="34" width="18.09765625" hidden="1" customWidth="1"/>
+    <col min="35" max="35" width="21.09765625" hidden="1" customWidth="1"/>
+    <col min="36" max="36" width="24.59765625" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="8.59765625" hidden="1" customWidth="1"/>
+    <col min="38" max="38" width="11.19921875" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="0" hidden="1" customWidth="1"/>
     <col min="40" max="40" width="15" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="14.875" customWidth="1"/>
+    <col min="41" max="41" width="14.8984375" customWidth="1"/>
     <col min="42" max="42" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="14.375" customWidth="1"/>
-    <col min="44" max="44" width="16.8125" customWidth="1"/>
-    <col min="45" max="45" width="20.875" customWidth="1"/>
+    <col min="43" max="43" width="14.3984375" customWidth="1"/>
+    <col min="44" max="44" width="16.796875" customWidth="1"/>
+    <col min="45" max="45" width="20.8984375" customWidth="1"/>
     <col min="46" max="46" width="19.5" bestFit="1" customWidth="1"/>
     <col min="47" max="48" width="19.5" customWidth="1"/>
-    <col min="49" max="49" width="27.3125" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="20.625" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="20.375" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="16.6875" customWidth="1"/>
-    <col min="53" max="53" width="29.625" customWidth="1"/>
+    <col min="49" max="49" width="27.296875" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="20.59765625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="20.3984375" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="16.69921875" customWidth="1"/>
+    <col min="53" max="53" width="29.59765625" customWidth="1"/>
     <col min="54" max="54" width="18.5" customWidth="1"/>
     <col min="55" max="55" width="21.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:55" ht="16.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="90" t="s">
+    <row r="1" spans="1:55" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="73" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="91"/>
-      <c r="C1" s="91"/>
-      <c r="D1" s="91"/>
-      <c r="E1" s="91"/>
-      <c r="F1" s="91"/>
-      <c r="G1" s="91"/>
-      <c r="H1" s="91"/>
-      <c r="I1" s="91"/>
-      <c r="J1" s="91"/>
-      <c r="K1" s="91"/>
-      <c r="L1" s="91"/>
-      <c r="M1" s="91"/>
-      <c r="N1" s="91"/>
-      <c r="O1" s="91"/>
-      <c r="P1" s="91"/>
-      <c r="Q1" s="91"/>
-      <c r="R1" s="91"/>
-      <c r="S1" s="91"/>
-      <c r="T1" s="91"/>
-      <c r="U1" s="91"/>
-      <c r="V1" s="91"/>
-      <c r="W1" s="91"/>
-      <c r="X1" s="91"/>
-      <c r="Y1" s="91"/>
-      <c r="Z1" s="91"/>
-      <c r="AA1" s="91"/>
-      <c r="AB1" s="91"/>
-      <c r="AC1" s="91"/>
-      <c r="AD1" s="91"/>
-      <c r="AE1" s="91"/>
-      <c r="AF1" s="91"/>
-      <c r="AG1" s="91"/>
-      <c r="AH1" s="91"/>
-      <c r="AI1" s="91"/>
-      <c r="AJ1" s="91"/>
-      <c r="AK1" s="91"/>
-      <c r="AL1" s="91"/>
-      <c r="AM1" s="91"/>
-      <c r="AN1" s="91"/>
-      <c r="AO1" s="91"/>
-      <c r="AP1" s="91"/>
-      <c r="AQ1" s="91"/>
-      <c r="AR1" s="91"/>
-      <c r="AS1" s="91"/>
-      <c r="AT1" s="91"/>
-      <c r="AU1" s="91"/>
-      <c r="AV1" s="91"/>
-      <c r="AW1" s="91"/>
-      <c r="AX1" s="91"/>
-      <c r="AY1" s="91"/>
-      <c r="AZ1" s="91"/>
-      <c r="BA1" s="91"/>
-      <c r="BB1" s="91"/>
-      <c r="BC1" s="91"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
+      <c r="I1" s="74"/>
+      <c r="J1" s="74"/>
+      <c r="K1" s="74"/>
+      <c r="L1" s="74"/>
+      <c r="M1" s="74"/>
+      <c r="N1" s="74"/>
+      <c r="O1" s="74"/>
+      <c r="P1" s="74"/>
+      <c r="Q1" s="74"/>
+      <c r="R1" s="74"/>
+      <c r="S1" s="74"/>
+      <c r="T1" s="74"/>
+      <c r="U1" s="74"/>
+      <c r="V1" s="74"/>
+      <c r="W1" s="74"/>
+      <c r="X1" s="74"/>
+      <c r="Y1" s="74"/>
+      <c r="Z1" s="74"/>
+      <c r="AA1" s="74"/>
+      <c r="AB1" s="74"/>
+      <c r="AC1" s="74"/>
+      <c r="AD1" s="74"/>
+      <c r="AE1" s="74"/>
+      <c r="AF1" s="74"/>
+      <c r="AG1" s="74"/>
+      <c r="AH1" s="74"/>
+      <c r="AI1" s="74"/>
+      <c r="AJ1" s="74"/>
+      <c r="AK1" s="74"/>
+      <c r="AL1" s="74"/>
+      <c r="AM1" s="74"/>
+      <c r="AN1" s="74"/>
+      <c r="AO1" s="74"/>
+      <c r="AP1" s="74"/>
+      <c r="AQ1" s="74"/>
+      <c r="AR1" s="74"/>
+      <c r="AS1" s="74"/>
+      <c r="AT1" s="74"/>
+      <c r="AU1" s="74"/>
+      <c r="AV1" s="74"/>
+      <c r="AW1" s="74"/>
+      <c r="AX1" s="74"/>
+      <c r="AY1" s="74"/>
+      <c r="AZ1" s="74"/>
+      <c r="BA1" s="74"/>
+      <c r="BB1" s="74"/>
+      <c r="BC1" s="74"/>
     </row>
-    <row r="2" spans="1:55" ht="17.25" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="90"/>
-      <c r="B2" s="91"/>
-      <c r="C2" s="91"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
-      <c r="H2" s="91"/>
-      <c r="I2" s="91"/>
-      <c r="J2" s="91"/>
-      <c r="K2" s="91"/>
-      <c r="L2" s="91"/>
-      <c r="M2" s="91"/>
-      <c r="N2" s="91"/>
-      <c r="O2" s="91"/>
-      <c r="P2" s="91"/>
-      <c r="Q2" s="91"/>
-      <c r="R2" s="91"/>
-      <c r="S2" s="91"/>
-      <c r="T2" s="91"/>
-      <c r="U2" s="91"/>
-      <c r="V2" s="91"/>
-      <c r="W2" s="91"/>
-      <c r="X2" s="91"/>
-      <c r="Y2" s="91"/>
-      <c r="Z2" s="91"/>
-      <c r="AA2" s="91"/>
-      <c r="AB2" s="91"/>
-      <c r="AC2" s="91"/>
-      <c r="AD2" s="91"/>
-      <c r="AE2" s="91"/>
-      <c r="AF2" s="91"/>
-      <c r="AG2" s="91"/>
-      <c r="AH2" s="91"/>
-      <c r="AI2" s="91"/>
-      <c r="AJ2" s="91"/>
-      <c r="AK2" s="91"/>
-      <c r="AL2" s="91"/>
-      <c r="AM2" s="91"/>
-      <c r="AN2" s="91"/>
-      <c r="AO2" s="91"/>
-      <c r="AP2" s="91"/>
-      <c r="AQ2" s="91"/>
-      <c r="AR2" s="91"/>
-      <c r="AS2" s="91"/>
-      <c r="AT2" s="91"/>
-      <c r="AU2" s="91"/>
-      <c r="AV2" s="91"/>
-      <c r="AW2" s="91"/>
-      <c r="AX2" s="91"/>
-      <c r="AY2" s="91"/>
-      <c r="AZ2" s="91"/>
-      <c r="BA2" s="91"/>
-      <c r="BB2" s="91"/>
-      <c r="BC2" s="91"/>
+    <row r="2" spans="1:55" ht="17.25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="73"/>
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
+      <c r="I2" s="74"/>
+      <c r="J2" s="74"/>
+      <c r="K2" s="74"/>
+      <c r="L2" s="74"/>
+      <c r="M2" s="74"/>
+      <c r="N2" s="74"/>
+      <c r="O2" s="74"/>
+      <c r="P2" s="74"/>
+      <c r="Q2" s="74"/>
+      <c r="R2" s="74"/>
+      <c r="S2" s="74"/>
+      <c r="T2" s="74"/>
+      <c r="U2" s="74"/>
+      <c r="V2" s="74"/>
+      <c r="W2" s="74"/>
+      <c r="X2" s="74"/>
+      <c r="Y2" s="74"/>
+      <c r="Z2" s="74"/>
+      <c r="AA2" s="74"/>
+      <c r="AB2" s="74"/>
+      <c r="AC2" s="74"/>
+      <c r="AD2" s="74"/>
+      <c r="AE2" s="74"/>
+      <c r="AF2" s="74"/>
+      <c r="AG2" s="74"/>
+      <c r="AH2" s="74"/>
+      <c r="AI2" s="74"/>
+      <c r="AJ2" s="74"/>
+      <c r="AK2" s="74"/>
+      <c r="AL2" s="74"/>
+      <c r="AM2" s="74"/>
+      <c r="AN2" s="74"/>
+      <c r="AO2" s="74"/>
+      <c r="AP2" s="74"/>
+      <c r="AQ2" s="74"/>
+      <c r="AR2" s="74"/>
+      <c r="AS2" s="74"/>
+      <c r="AT2" s="74"/>
+      <c r="AU2" s="74"/>
+      <c r="AV2" s="74"/>
+      <c r="AW2" s="74"/>
+      <c r="AX2" s="74"/>
+      <c r="AY2" s="74"/>
+      <c r="AZ2" s="74"/>
+      <c r="BA2" s="74"/>
+      <c r="BB2" s="74"/>
+      <c r="BC2" s="74"/>
     </row>
-    <row r="3" spans="1:55" x14ac:dyDescent="0.6">
-      <c r="A3" s="82" t="s">
+    <row r="3" spans="1:55" x14ac:dyDescent="0.4">
+      <c r="A3" s="79" t="s">
         <v>105</v>
       </c>
-      <c r="B3" s="82"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="82"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="82" t="s">
+      <c r="B3" s="79"/>
+      <c r="C3" s="79"/>
+      <c r="D3" s="79"/>
+      <c r="E3" s="79"/>
+      <c r="F3" s="79" t="s">
         <v>108</v>
       </c>
-      <c r="G3" s="82"/>
-      <c r="H3" s="82"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="82"/>
-      <c r="K3" s="89" t="s">
+      <c r="G3" s="79"/>
+      <c r="H3" s="79"/>
+      <c r="I3" s="79"/>
+      <c r="J3" s="79"/>
+      <c r="K3" s="72" t="s">
         <v>109</v>
       </c>
-      <c r="L3" s="89"/>
-      <c r="M3" s="89"/>
-      <c r="N3" s="89"/>
-      <c r="O3" s="89"/>
-      <c r="P3" s="89"/>
-      <c r="Q3" s="89"/>
-      <c r="R3" s="89"/>
-      <c r="S3" s="89"/>
-      <c r="T3" s="89"/>
-      <c r="U3" s="89"/>
-      <c r="V3" s="89"/>
-      <c r="W3" s="89"/>
-      <c r="X3" s="89"/>
-      <c r="Y3" s="89"/>
-      <c r="Z3" s="89"/>
-      <c r="AA3" s="89"/>
-      <c r="AB3" s="89"/>
-      <c r="AC3" s="89"/>
-      <c r="AD3" s="89"/>
-      <c r="AE3" s="89"/>
-      <c r="AF3" s="89"/>
-      <c r="AG3" s="89"/>
-      <c r="AH3" s="89"/>
-      <c r="AI3" s="89"/>
-      <c r="AJ3" s="89"/>
-      <c r="AK3" s="89"/>
-      <c r="AL3" s="89"/>
-      <c r="AM3" s="89"/>
-      <c r="AN3" s="89"/>
-      <c r="AO3" s="89"/>
-      <c r="AP3" s="89"/>
-      <c r="AQ3" s="89"/>
-      <c r="AR3" s="89"/>
-      <c r="AS3" s="89"/>
-      <c r="AT3" s="89"/>
-      <c r="AU3" s="89"/>
-      <c r="AV3" s="89"/>
-      <c r="AW3" s="89"/>
-      <c r="AX3" s="89"/>
-      <c r="AY3" s="89"/>
-      <c r="AZ3" s="89"/>
-      <c r="BA3" s="89"/>
-      <c r="BB3" s="89"/>
-      <c r="BC3" s="89"/>
+      <c r="L3" s="72"/>
+      <c r="M3" s="72"/>
+      <c r="N3" s="72"/>
+      <c r="O3" s="72"/>
+      <c r="P3" s="72"/>
+      <c r="Q3" s="72"/>
+      <c r="R3" s="72"/>
+      <c r="S3" s="72"/>
+      <c r="T3" s="72"/>
+      <c r="U3" s="72"/>
+      <c r="V3" s="72"/>
+      <c r="W3" s="72"/>
+      <c r="X3" s="72"/>
+      <c r="Y3" s="72"/>
+      <c r="Z3" s="72"/>
+      <c r="AA3" s="72"/>
+      <c r="AB3" s="72"/>
+      <c r="AC3" s="72"/>
+      <c r="AD3" s="72"/>
+      <c r="AE3" s="72"/>
+      <c r="AF3" s="72"/>
+      <c r="AG3" s="72"/>
+      <c r="AH3" s="72"/>
+      <c r="AI3" s="72"/>
+      <c r="AJ3" s="72"/>
+      <c r="AK3" s="72"/>
+      <c r="AL3" s="72"/>
+      <c r="AM3" s="72"/>
+      <c r="AN3" s="72"/>
+      <c r="AO3" s="72"/>
+      <c r="AP3" s="72"/>
+      <c r="AQ3" s="72"/>
+      <c r="AR3" s="72"/>
+      <c r="AS3" s="72"/>
+      <c r="AT3" s="72"/>
+      <c r="AU3" s="72"/>
+      <c r="AV3" s="72"/>
+      <c r="AW3" s="72"/>
+      <c r="AX3" s="72"/>
+      <c r="AY3" s="72"/>
+      <c r="AZ3" s="72"/>
+      <c r="BA3" s="72"/>
+      <c r="BB3" s="72"/>
+      <c r="BC3" s="72"/>
     </row>
-    <row r="4" spans="1:55" x14ac:dyDescent="0.6">
-      <c r="A4" s="82"/>
-      <c r="B4" s="82"/>
-      <c r="C4" s="82"/>
-      <c r="D4" s="82"/>
-      <c r="E4" s="82"/>
-      <c r="F4" s="82"/>
-      <c r="G4" s="82"/>
-      <c r="H4" s="82"/>
-      <c r="I4" s="82"/>
-      <c r="J4" s="82"/>
-      <c r="K4" s="82" t="s">
+    <row r="4" spans="1:55" x14ac:dyDescent="0.4">
+      <c r="A4" s="79"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="79"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="79"/>
+      <c r="F4" s="79"/>
+      <c r="G4" s="79"/>
+      <c r="H4" s="79"/>
+      <c r="I4" s="79"/>
+      <c r="J4" s="79"/>
+      <c r="K4" s="79" t="s">
         <v>80</v>
       </c>
-      <c r="L4" s="82"/>
-      <c r="M4" s="82" t="s">
+      <c r="L4" s="79"/>
+      <c r="M4" s="79" t="s">
         <v>79</v>
       </c>
-      <c r="N4" s="82"/>
-      <c r="O4" s="82"/>
-      <c r="P4" s="82"/>
-      <c r="Q4" s="82"/>
-      <c r="R4" s="82"/>
-      <c r="S4" s="82"/>
-      <c r="T4" s="82"/>
-      <c r="U4" s="82"/>
-      <c r="V4" s="82"/>
-      <c r="W4" s="82"/>
-      <c r="X4" s="82"/>
-      <c r="Y4" s="82"/>
-      <c r="Z4" s="82"/>
-      <c r="AA4" s="82"/>
-      <c r="AB4" s="82"/>
-      <c r="AC4" s="82"/>
-      <c r="AD4" s="82"/>
-      <c r="AE4" s="82"/>
-      <c r="AF4" s="82"/>
-      <c r="AG4" s="82"/>
-      <c r="AH4" s="82"/>
-      <c r="AI4" s="82"/>
-      <c r="AJ4" s="82"/>
-      <c r="AK4" s="82"/>
-      <c r="AL4" s="82"/>
-      <c r="AM4" s="82"/>
-      <c r="AN4" s="82"/>
-      <c r="AO4" s="82"/>
-      <c r="AP4" s="88" t="s">
+      <c r="N4" s="79"/>
+      <c r="O4" s="79"/>
+      <c r="P4" s="79"/>
+      <c r="Q4" s="79"/>
+      <c r="R4" s="79"/>
+      <c r="S4" s="79"/>
+      <c r="T4" s="79"/>
+      <c r="U4" s="79"/>
+      <c r="V4" s="79"/>
+      <c r="W4" s="79"/>
+      <c r="X4" s="79"/>
+      <c r="Y4" s="79"/>
+      <c r="Z4" s="79"/>
+      <c r="AA4" s="79"/>
+      <c r="AB4" s="79"/>
+      <c r="AC4" s="79"/>
+      <c r="AD4" s="79"/>
+      <c r="AE4" s="79"/>
+      <c r="AF4" s="79"/>
+      <c r="AG4" s="79"/>
+      <c r="AH4" s="79"/>
+      <c r="AI4" s="79"/>
+      <c r="AJ4" s="79"/>
+      <c r="AK4" s="79"/>
+      <c r="AL4" s="79"/>
+      <c r="AM4" s="79"/>
+      <c r="AN4" s="79"/>
+      <c r="AO4" s="79"/>
+      <c r="AP4" s="71" t="s">
         <v>221</v>
       </c>
-      <c r="AQ4" s="88"/>
-      <c r="AR4" s="88"/>
-      <c r="AS4" s="88"/>
-      <c r="AT4" s="88"/>
-      <c r="AU4" s="88"/>
-      <c r="AV4" s="88"/>
-      <c r="AW4" s="88"/>
-      <c r="AX4" s="88"/>
-      <c r="AY4" s="88"/>
-      <c r="AZ4" s="88"/>
-      <c r="BA4" s="88"/>
-      <c r="BB4" s="88"/>
-      <c r="BC4" s="88"/>
+      <c r="AQ4" s="71"/>
+      <c r="AR4" s="71"/>
+      <c r="AS4" s="71"/>
+      <c r="AT4" s="71"/>
+      <c r="AU4" s="71"/>
+      <c r="AV4" s="71"/>
+      <c r="AW4" s="71"/>
+      <c r="AX4" s="71"/>
+      <c r="AY4" s="71"/>
+      <c r="AZ4" s="71"/>
+      <c r="BA4" s="71"/>
+      <c r="BB4" s="71"/>
+      <c r="BC4" s="71"/>
     </row>
-    <row r="5" spans="1:55" ht="16.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A5" s="82"/>
-      <c r="B5" s="82"/>
-      <c r="C5" s="82"/>
-      <c r="D5" s="82"/>
-      <c r="E5" s="82"/>
-      <c r="F5" s="70" t="s">
+    <row r="5" spans="1:55" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="79"/>
+      <c r="B5" s="79"/>
+      <c r="C5" s="79"/>
+      <c r="D5" s="79"/>
+      <c r="E5" s="79"/>
+      <c r="F5" s="83" t="s">
         <v>104</v>
       </c>
-      <c r="G5" s="70"/>
-      <c r="H5" s="70"/>
-      <c r="I5" s="70"/>
-      <c r="J5" s="70"/>
-      <c r="K5" s="70" t="s">
+      <c r="G5" s="83"/>
+      <c r="H5" s="83"/>
+      <c r="I5" s="83"/>
+      <c r="J5" s="83"/>
+      <c r="K5" s="83" t="s">
         <v>103</v>
       </c>
-      <c r="L5" s="70"/>
-      <c r="M5" s="70" t="s">
+      <c r="L5" s="83"/>
+      <c r="M5" s="83" t="s">
         <v>107</v>
       </c>
-      <c r="N5" s="70"/>
-      <c r="O5" s="70"/>
-      <c r="P5" s="70"/>
-      <c r="Q5" s="70"/>
-      <c r="R5" s="70"/>
-      <c r="S5" s="70"/>
-      <c r="T5" s="70"/>
-      <c r="U5" s="70"/>
-      <c r="V5" s="70"/>
-      <c r="W5" s="70"/>
-      <c r="X5" s="70"/>
-      <c r="Y5" s="70"/>
-      <c r="Z5" s="70"/>
-      <c r="AA5" s="70"/>
-      <c r="AB5" s="70"/>
-      <c r="AC5" s="70"/>
-      <c r="AD5" s="70"/>
-      <c r="AE5" s="70"/>
-      <c r="AF5" s="70"/>
-      <c r="AG5" s="70"/>
-      <c r="AH5" s="70"/>
-      <c r="AI5" s="70"/>
-      <c r="AJ5" s="70"/>
-      <c r="AK5" s="70"/>
-      <c r="AL5" s="70"/>
-      <c r="AM5" s="70"/>
-      <c r="AN5" s="70"/>
-      <c r="AO5" s="70"/>
-      <c r="AP5" s="88" t="s">
+      <c r="N5" s="83"/>
+      <c r="O5" s="83"/>
+      <c r="P5" s="83"/>
+      <c r="Q5" s="83"/>
+      <c r="R5" s="83"/>
+      <c r="S5" s="83"/>
+      <c r="T5" s="83"/>
+      <c r="U5" s="83"/>
+      <c r="V5" s="83"/>
+      <c r="W5" s="83"/>
+      <c r="X5" s="83"/>
+      <c r="Y5" s="83"/>
+      <c r="Z5" s="83"/>
+      <c r="AA5" s="83"/>
+      <c r="AB5" s="83"/>
+      <c r="AC5" s="83"/>
+      <c r="AD5" s="83"/>
+      <c r="AE5" s="83"/>
+      <c r="AF5" s="83"/>
+      <c r="AG5" s="83"/>
+      <c r="AH5" s="83"/>
+      <c r="AI5" s="83"/>
+      <c r="AJ5" s="83"/>
+      <c r="AK5" s="83"/>
+      <c r="AL5" s="83"/>
+      <c r="AM5" s="83"/>
+      <c r="AN5" s="83"/>
+      <c r="AO5" s="83"/>
+      <c r="AP5" s="71" t="s">
         <v>222</v>
       </c>
-      <c r="AQ5" s="88"/>
-      <c r="AR5" s="88"/>
-      <c r="AS5" s="88"/>
-      <c r="AT5" s="88"/>
-      <c r="AU5" s="88"/>
-      <c r="AV5" s="88"/>
-      <c r="AW5" s="88"/>
-      <c r="AX5" s="88"/>
-      <c r="AY5" s="88"/>
-      <c r="AZ5" s="88"/>
-      <c r="BA5" s="88"/>
-      <c r="BB5" s="88"/>
-      <c r="BC5" s="88"/>
+      <c r="AQ5" s="71"/>
+      <c r="AR5" s="71"/>
+      <c r="AS5" s="71"/>
+      <c r="AT5" s="71"/>
+      <c r="AU5" s="71"/>
+      <c r="AV5" s="71"/>
+      <c r="AW5" s="71"/>
+      <c r="AX5" s="71"/>
+      <c r="AY5" s="71"/>
+      <c r="AZ5" s="71"/>
+      <c r="BA5" s="71"/>
+      <c r="BB5" s="71"/>
+      <c r="BC5" s="71"/>
     </row>
-    <row r="6" spans="1:55" ht="33.75" x14ac:dyDescent="0.6">
-      <c r="A6" s="70" t="s">
+    <row r="6" spans="1:55" ht="34.799999999999997" x14ac:dyDescent="0.4">
+      <c r="A6" s="83" t="s">
         <v>76</v>
       </c>
-      <c r="B6" s="70"/>
-      <c r="C6" s="70"/>
+      <c r="B6" s="83"/>
+      <c r="C6" s="83"/>
       <c r="D6" s="22" t="s">
         <v>0</v>
       </c>
@@ -2920,11 +2924,11 @@
       <c r="L6" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="M6" s="70" t="s">
+      <c r="M6" s="83" t="s">
         <v>83</v>
       </c>
-      <c r="N6" s="70"/>
-      <c r="O6" s="70"/>
+      <c r="N6" s="83"/>
+      <c r="O6" s="83"/>
       <c r="P6" s="23" t="s">
         <v>87</v>
       </c>
@@ -3044,11 +3048,11 @@
         <v>302</v>
       </c>
     </row>
-    <row r="7" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="72" t="s">
+    <row r="7" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="80" t="s">
         <v>99</v>
       </c>
-      <c r="B7" s="72" t="s">
+      <c r="B7" s="80" t="s">
         <v>101</v>
       </c>
       <c r="C7" s="20" t="s">
@@ -3081,12 +3085,12 @@
       <c r="L7" s="56" t="s">
         <v>117</v>
       </c>
-      <c r="M7" s="86" t="s">
+      <c r="M7" s="78" t="s">
         <v>200</v>
       </c>
-      <c r="N7" s="86"/>
-      <c r="O7" s="86"/>
-      <c r="P7" s="67" t="s">
+      <c r="N7" s="78"/>
+      <c r="O7" s="78"/>
+      <c r="P7" s="76" t="s">
         <v>206</v>
       </c>
       <c r="Q7" s="26"/>
@@ -3114,16 +3118,16 @@
         <v>231</v>
       </c>
       <c r="AM7" s="42"/>
-      <c r="AN7" s="84" t="s">
+      <c r="AN7" s="70" t="s">
         <v>214</v>
       </c>
-      <c r="AO7" s="87" t="s">
+      <c r="AO7" s="82" t="s">
         <v>230</v>
       </c>
       <c r="AP7" s="62" t="s">
         <v>248</v>
       </c>
-      <c r="AQ7" s="84" t="s">
+      <c r="AQ7" s="70" t="s">
         <v>224</v>
       </c>
       <c r="AR7" s="62" t="s">
@@ -3149,20 +3153,20 @@
       <c r="AZ7" s="62" t="s">
         <v>276</v>
       </c>
-      <c r="BA7" s="84" t="s">
+      <c r="BA7" s="70" t="s">
         <v>304</v>
       </c>
       <c r="BB7" s="62" t="s">
         <v>312</v>
       </c>
-      <c r="BC7" s="84" t="s">
+      <c r="BC7" s="70" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="8" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="75"/>
-      <c r="B8" s="75"/>
-      <c r="C8" s="72" t="s">
+    <row r="8" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="81"/>
+      <c r="B8" s="81"/>
+      <c r="C8" s="80" t="s">
         <v>127</v>
       </c>
       <c r="D8" s="24" t="s">
@@ -3192,10 +3196,10 @@
       <c r="L8" s="56" t="s">
         <v>196</v>
       </c>
-      <c r="M8" s="86"/>
-      <c r="N8" s="86"/>
-      <c r="O8" s="86"/>
-      <c r="P8" s="67"/>
+      <c r="M8" s="78"/>
+      <c r="N8" s="78"/>
+      <c r="O8" s="78"/>
+      <c r="P8" s="76"/>
       <c r="Q8" s="26"/>
       <c r="R8" s="27"/>
       <c r="S8" s="27"/>
@@ -3221,47 +3225,47 @@
         <v>232</v>
       </c>
       <c r="AM8" s="42"/>
-      <c r="AN8" s="84"/>
-      <c r="AO8" s="87"/>
-      <c r="AP8" s="84" t="s">
+      <c r="AN8" s="70"/>
+      <c r="AO8" s="82"/>
+      <c r="AP8" s="70" t="s">
         <v>245</v>
       </c>
-      <c r="AQ8" s="84"/>
-      <c r="AR8" s="84" t="s">
+      <c r="AQ8" s="70"/>
+      <c r="AR8" s="70" t="s">
         <v>254</v>
       </c>
-      <c r="AS8" s="84" t="s">
+      <c r="AS8" s="70" t="s">
         <v>259</v>
       </c>
-      <c r="AT8" s="84" t="s">
+      <c r="AT8" s="70" t="s">
         <v>285</v>
       </c>
       <c r="AU8" s="62"/>
-      <c r="AV8" s="84" t="s">
+      <c r="AV8" s="70" t="s">
         <v>293</v>
       </c>
-      <c r="AW8" s="84" t="s">
+      <c r="AW8" s="70" t="s">
         <v>298</v>
       </c>
-      <c r="AX8" s="84" t="s">
+      <c r="AX8" s="70" t="s">
         <v>287</v>
       </c>
-      <c r="AY8" s="84" t="s">
+      <c r="AY8" s="70" t="s">
         <v>300</v>
       </c>
       <c r="AZ8" s="62" t="s">
         <v>277</v>
       </c>
-      <c r="BA8" s="84"/>
-      <c r="BB8" s="124" t="s">
+      <c r="BA8" s="70"/>
+      <c r="BB8" s="67" t="s">
         <v>313</v>
       </c>
-      <c r="BC8" s="84"/>
+      <c r="BC8" s="70"/>
     </row>
-    <row r="9" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="75"/>
-      <c r="B9" s="75"/>
-      <c r="C9" s="72"/>
+    <row r="9" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="81"/>
+      <c r="B9" s="81"/>
+      <c r="C9" s="80"/>
       <c r="D9" s="24" t="s">
         <v>21</v>
       </c>
@@ -3283,16 +3287,16 @@
       <c r="J9" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="K9" s="67" t="s">
+      <c r="K9" s="76" t="s">
         <v>188</v>
       </c>
-      <c r="L9" s="83" t="s">
+      <c r="L9" s="77" t="s">
         <v>197</v>
       </c>
-      <c r="M9" s="86"/>
-      <c r="N9" s="86"/>
-      <c r="O9" s="86"/>
-      <c r="P9" s="67"/>
+      <c r="M9" s="78"/>
+      <c r="N9" s="78"/>
+      <c r="O9" s="78"/>
+      <c r="P9" s="76"/>
       <c r="Q9" s="26"/>
       <c r="R9" s="27"/>
       <c r="S9" s="27"/>
@@ -3314,32 +3318,32 @@
       <c r="AI9" s="20"/>
       <c r="AJ9" s="20"/>
       <c r="AK9" s="24"/>
-      <c r="AL9" s="67" t="s">
+      <c r="AL9" s="76" t="s">
         <v>233</v>
       </c>
       <c r="AM9" s="42"/>
-      <c r="AN9" s="84"/>
-      <c r="AO9" s="87"/>
-      <c r="AP9" s="84"/>
-      <c r="AQ9" s="84"/>
-      <c r="AR9" s="84"/>
-      <c r="AS9" s="84"/>
-      <c r="AT9" s="84"/>
+      <c r="AN9" s="70"/>
+      <c r="AO9" s="82"/>
+      <c r="AP9" s="70"/>
+      <c r="AQ9" s="70"/>
+      <c r="AR9" s="70"/>
+      <c r="AS9" s="70"/>
+      <c r="AT9" s="70"/>
       <c r="AU9" s="62"/>
-      <c r="AV9" s="84"/>
-      <c r="AW9" s="84"/>
-      <c r="AX9" s="84"/>
-      <c r="AY9" s="92"/>
-      <c r="AZ9" s="84" t="s">
+      <c r="AV9" s="70"/>
+      <c r="AW9" s="70"/>
+      <c r="AX9" s="70"/>
+      <c r="AY9" s="75"/>
+      <c r="AZ9" s="70" t="s">
         <v>278</v>
       </c>
-      <c r="BA9" s="84"/>
-      <c r="BB9" s="123"/>
-      <c r="BC9" s="84"/>
+      <c r="BA9" s="70"/>
+      <c r="BB9" s="68"/>
+      <c r="BC9" s="70"/>
     </row>
-    <row r="10" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="75"/>
-      <c r="B10" s="75"/>
+    <row r="10" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="81"/>
+      <c r="B10" s="81"/>
       <c r="C10" s="20" t="s">
         <v>128</v>
       </c>
@@ -3364,12 +3368,12 @@
       <c r="J10" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="K10" s="67"/>
-      <c r="L10" s="83"/>
-      <c r="M10" s="86"/>
-      <c r="N10" s="86"/>
-      <c r="O10" s="86"/>
-      <c r="P10" s="67"/>
+      <c r="K10" s="76"/>
+      <c r="L10" s="77"/>
+      <c r="M10" s="78"/>
+      <c r="N10" s="78"/>
+      <c r="O10" s="78"/>
+      <c r="P10" s="76"/>
       <c r="Q10" s="26"/>
       <c r="R10" s="27"/>
       <c r="S10" s="27"/>
@@ -3391,46 +3395,46 @@
       <c r="AI10" s="20"/>
       <c r="AJ10" s="20"/>
       <c r="AK10" s="24"/>
-      <c r="AL10" s="67"/>
+      <c r="AL10" s="76"/>
       <c r="AM10" s="42"/>
-      <c r="AN10" s="84"/>
-      <c r="AO10" s="87"/>
-      <c r="AP10" s="84"/>
-      <c r="AQ10" s="84"/>
-      <c r="AR10" s="84"/>
-      <c r="AS10" s="84"/>
-      <c r="AT10" s="84"/>
+      <c r="AN10" s="70"/>
+      <c r="AO10" s="82"/>
+      <c r="AP10" s="70"/>
+      <c r="AQ10" s="70"/>
+      <c r="AR10" s="70"/>
+      <c r="AS10" s="70"/>
+      <c r="AT10" s="70"/>
       <c r="AU10" s="62"/>
-      <c r="AV10" s="84"/>
-      <c r="AW10" s="84"/>
-      <c r="AX10" s="84"/>
-      <c r="AY10" s="92"/>
-      <c r="AZ10" s="84"/>
-      <c r="BA10" s="84"/>
-      <c r="BB10" s="123"/>
-      <c r="BC10" s="84"/>
+      <c r="AV10" s="70"/>
+      <c r="AW10" s="70"/>
+      <c r="AX10" s="70"/>
+      <c r="AY10" s="75"/>
+      <c r="AZ10" s="70"/>
+      <c r="BA10" s="70"/>
+      <c r="BB10" s="68"/>
+      <c r="BC10" s="70"/>
     </row>
-    <row r="11" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="75"/>
-      <c r="B11" s="75"/>
-      <c r="C11" s="71"/>
-      <c r="D11" s="71"/>
-      <c r="E11" s="71"/>
-      <c r="F11" s="71"/>
-      <c r="G11" s="71"/>
-      <c r="H11" s="71"/>
-      <c r="I11" s="71"/>
-      <c r="J11" s="71"/>
+    <row r="11" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="81"/>
+      <c r="B11" s="81"/>
+      <c r="C11" s="94"/>
+      <c r="D11" s="94"/>
+      <c r="E11" s="94"/>
+      <c r="F11" s="94"/>
+      <c r="G11" s="94"/>
+      <c r="H11" s="94"/>
+      <c r="I11" s="94"/>
+      <c r="J11" s="94"/>
       <c r="K11" s="24" t="s">
         <v>189</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>198</v>
       </c>
-      <c r="M11" s="86"/>
-      <c r="N11" s="86"/>
-      <c r="O11" s="86"/>
-      <c r="P11" s="67"/>
+      <c r="M11" s="78"/>
+      <c r="N11" s="78"/>
+      <c r="O11" s="78"/>
+      <c r="P11" s="76"/>
       <c r="Q11" s="26"/>
       <c r="R11" s="27"/>
       <c r="S11" s="27"/>
@@ -3452,49 +3456,49 @@
       <c r="AI11" s="20"/>
       <c r="AJ11" s="20"/>
       <c r="AK11" s="24"/>
-      <c r="AL11" s="67"/>
+      <c r="AL11" s="76"/>
       <c r="AM11" s="42"/>
-      <c r="AN11" s="84" t="s">
+      <c r="AN11" s="70" t="s">
         <v>215</v>
       </c>
-      <c r="AO11" s="87"/>
-      <c r="AP11" s="84"/>
-      <c r="AQ11" s="84"/>
-      <c r="AR11" s="84"/>
-      <c r="AS11" s="84"/>
-      <c r="AT11" s="84"/>
+      <c r="AO11" s="82"/>
+      <c r="AP11" s="70"/>
+      <c r="AQ11" s="70"/>
+      <c r="AR11" s="70"/>
+      <c r="AS11" s="70"/>
+      <c r="AT11" s="70"/>
       <c r="AU11" s="62"/>
-      <c r="AV11" s="84"/>
-      <c r="AW11" s="84"/>
-      <c r="AX11" s="84"/>
-      <c r="AY11" s="92"/>
-      <c r="AZ11" s="84"/>
-      <c r="BA11" s="84"/>
-      <c r="BB11" s="123"/>
-      <c r="BC11" s="84"/>
+      <c r="AV11" s="70"/>
+      <c r="AW11" s="70"/>
+      <c r="AX11" s="70"/>
+      <c r="AY11" s="75"/>
+      <c r="AZ11" s="70"/>
+      <c r="BA11" s="70"/>
+      <c r="BB11" s="68"/>
+      <c r="BC11" s="70"/>
     </row>
-    <row r="12" spans="1:55" ht="21" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A12" s="75"/>
-      <c r="B12" s="75"/>
-      <c r="C12" s="71"/>
-      <c r="D12" s="71"/>
-      <c r="E12" s="71"/>
-      <c r="F12" s="71"/>
-      <c r="G12" s="71"/>
-      <c r="H12" s="71"/>
-      <c r="I12" s="71"/>
-      <c r="J12" s="71"/>
+    <row r="12" spans="1:55" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="81"/>
+      <c r="B12" s="81"/>
+      <c r="C12" s="94"/>
+      <c r="D12" s="94"/>
+      <c r="E12" s="94"/>
+      <c r="F12" s="94"/>
+      <c r="G12" s="94"/>
+      <c r="H12" s="94"/>
+      <c r="I12" s="94"/>
+      <c r="J12" s="94"/>
       <c r="K12" s="24" t="s">
         <v>190</v>
       </c>
       <c r="L12" s="56" t="s">
         <v>199</v>
       </c>
-      <c r="M12" s="86" t="s">
+      <c r="M12" s="78" t="s">
         <v>205</v>
       </c>
-      <c r="N12" s="86"/>
-      <c r="O12" s="86"/>
+      <c r="N12" s="78"/>
+      <c r="O12" s="78"/>
       <c r="P12" s="24" t="s">
         <v>207</v>
       </c>
@@ -3519,34 +3523,34 @@
       <c r="AI12" s="20"/>
       <c r="AJ12" s="20"/>
       <c r="AK12" s="24"/>
-      <c r="AL12" s="67"/>
+      <c r="AL12" s="76"/>
       <c r="AM12" s="42"/>
-      <c r="AN12" s="84"/>
+      <c r="AN12" s="70"/>
       <c r="AO12" s="24" t="s">
         <v>234</v>
       </c>
-      <c r="AP12" s="84"/>
+      <c r="AP12" s="70"/>
       <c r="AQ12" s="62" t="s">
         <v>225</v>
       </c>
-      <c r="AR12" s="84"/>
-      <c r="AS12" s="84"/>
-      <c r="AT12" s="84"/>
+      <c r="AR12" s="70"/>
+      <c r="AS12" s="70"/>
+      <c r="AT12" s="70"/>
       <c r="AU12" s="62"/>
-      <c r="AV12" s="84"/>
-      <c r="AW12" s="84"/>
-      <c r="AX12" s="84"/>
+      <c r="AV12" s="70"/>
+      <c r="AW12" s="70"/>
+      <c r="AX12" s="70"/>
       <c r="AY12" s="62" t="s">
         <v>270</v>
       </c>
-      <c r="AZ12" s="84"/>
-      <c r="BA12" s="84"/>
-      <c r="BB12" s="117"/>
-      <c r="BC12" s="84"/>
+      <c r="AZ12" s="70"/>
+      <c r="BA12" s="70"/>
+      <c r="BB12" s="69"/>
+      <c r="BC12" s="70"/>
     </row>
-    <row r="13" spans="1:55" ht="27" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A13" s="75"/>
-      <c r="B13" s="75"/>
+    <row r="13" spans="1:55" ht="27" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="81"/>
+      <c r="B13" s="81"/>
       <c r="C13" s="20" t="s">
         <v>129</v>
       </c>
@@ -3577,11 +3581,11 @@
       <c r="L13" s="56" t="s">
         <v>121</v>
       </c>
-      <c r="M13" s="67" t="s">
+      <c r="M13" s="76" t="s">
         <v>202</v>
       </c>
-      <c r="N13" s="67"/>
-      <c r="O13" s="67"/>
+      <c r="N13" s="76"/>
+      <c r="O13" s="76"/>
       <c r="P13" s="24" t="s">
         <v>211</v>
       </c>
@@ -3651,45 +3655,45 @@
         <v>308</v>
       </c>
     </row>
-    <row r="14" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A14" s="75"/>
-      <c r="B14" s="75"/>
-      <c r="C14" s="72" t="s">
+    <row r="14" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="81"/>
+      <c r="B14" s="81"/>
+      <c r="C14" s="80" t="s">
         <v>130</v>
       </c>
-      <c r="D14" s="67" t="s">
+      <c r="D14" s="76" t="s">
         <v>144</v>
       </c>
-      <c r="E14" s="72" t="s">
+      <c r="E14" s="80" t="s">
         <v>130</v>
       </c>
-      <c r="F14" s="67" t="s">
+      <c r="F14" s="76" t="s">
         <v>114</v>
       </c>
-      <c r="G14" s="83" t="s">
+      <c r="G14" s="77" t="s">
         <v>122</v>
       </c>
-      <c r="H14" s="83" t="s">
+      <c r="H14" s="77" t="s">
         <v>182</v>
       </c>
-      <c r="I14" s="67" t="s">
+      <c r="I14" s="76" t="s">
         <v>166</v>
       </c>
-      <c r="J14" s="67" t="s">
+      <c r="J14" s="76" t="s">
         <v>174</v>
       </c>
-      <c r="K14" s="67" t="s">
+      <c r="K14" s="76" t="s">
         <v>192</v>
       </c>
-      <c r="L14" s="83" t="s">
+      <c r="L14" s="77" t="s">
         <v>122</v>
       </c>
-      <c r="M14" s="86" t="s">
+      <c r="M14" s="78" t="s">
         <v>204</v>
       </c>
-      <c r="N14" s="86"/>
-      <c r="O14" s="86"/>
-      <c r="P14" s="67" t="s">
+      <c r="N14" s="78"/>
+      <c r="O14" s="78"/>
+      <c r="P14" s="76" t="s">
         <v>208</v>
       </c>
       <c r="Q14" s="26"/>
@@ -3713,7 +3717,7 @@
       <c r="AI14" s="24"/>
       <c r="AJ14" s="24"/>
       <c r="AK14" s="24"/>
-      <c r="AL14" s="67" t="s">
+      <c r="AL14" s="76" t="s">
         <v>238</v>
       </c>
       <c r="AM14" s="42"/>
@@ -3723,60 +3727,60 @@
       <c r="AO14" s="24" t="s">
         <v>237</v>
       </c>
-      <c r="AP14" s="67" t="s">
+      <c r="AP14" s="76" t="s">
         <v>247</v>
       </c>
-      <c r="AQ14" s="84" t="s">
+      <c r="AQ14" s="70" t="s">
         <v>226</v>
       </c>
-      <c r="AR14" s="84"/>
-      <c r="AS14" s="84" t="s">
+      <c r="AR14" s="70"/>
+      <c r="AS14" s="70" t="s">
         <v>260</v>
       </c>
-      <c r="AT14" s="84" t="s">
+      <c r="AT14" s="70" t="s">
         <v>265</v>
       </c>
       <c r="AU14" s="62"/>
-      <c r="AV14" s="84" t="s">
+      <c r="AV14" s="70" t="s">
         <v>294</v>
       </c>
       <c r="AW14" s="62"/>
-      <c r="AX14" s="84" t="s">
+      <c r="AX14" s="70" t="s">
         <v>267</v>
       </c>
-      <c r="AY14" s="67" t="s">
+      <c r="AY14" s="76" t="s">
         <v>271</v>
       </c>
-      <c r="AZ14" s="84" t="s">
+      <c r="AZ14" s="70" t="s">
         <v>279</v>
       </c>
-      <c r="BA14" s="84" t="s">
+      <c r="BA14" s="70" t="s">
         <v>306</v>
       </c>
-      <c r="BB14" s="124" t="s">
+      <c r="BB14" s="67" t="s">
         <v>315</v>
       </c>
-      <c r="BC14" s="84" t="s">
+      <c r="BC14" s="70" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="15" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A15" s="75"/>
-      <c r="B15" s="75"/>
-      <c r="C15" s="72"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="72"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="83"/>
-      <c r="H15" s="83"/>
-      <c r="I15" s="67"/>
-      <c r="J15" s="67"/>
-      <c r="K15" s="67"/>
-      <c r="L15" s="83"/>
-      <c r="M15" s="86"/>
-      <c r="N15" s="86"/>
-      <c r="O15" s="86"/>
-      <c r="P15" s="67"/>
+    <row r="15" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="81"/>
+      <c r="B15" s="81"/>
+      <c r="C15" s="80"/>
+      <c r="D15" s="76"/>
+      <c r="E15" s="80"/>
+      <c r="F15" s="76"/>
+      <c r="G15" s="77"/>
+      <c r="H15" s="77"/>
+      <c r="I15" s="76"/>
+      <c r="J15" s="76"/>
+      <c r="K15" s="76"/>
+      <c r="L15" s="77"/>
+      <c r="M15" s="78"/>
+      <c r="N15" s="78"/>
+      <c r="O15" s="78"/>
+      <c r="P15" s="76"/>
       <c r="Q15" s="26"/>
       <c r="R15" s="27"/>
       <c r="S15" s="27"/>
@@ -3798,7 +3802,7 @@
       <c r="AI15" s="24"/>
       <c r="AJ15" s="24"/>
       <c r="AK15" s="24"/>
-      <c r="AL15" s="67"/>
+      <c r="AL15" s="76"/>
       <c r="AM15" s="42"/>
       <c r="AN15" s="62" t="s">
         <v>217</v>
@@ -3806,24 +3810,24 @@
       <c r="AO15" s="24" t="s">
         <v>239</v>
       </c>
-      <c r="AP15" s="67"/>
-      <c r="AQ15" s="84"/>
-      <c r="AR15" s="84"/>
-      <c r="AS15" s="84"/>
-      <c r="AT15" s="84"/>
+      <c r="AP15" s="76"/>
+      <c r="AQ15" s="70"/>
+      <c r="AR15" s="70"/>
+      <c r="AS15" s="70"/>
+      <c r="AT15" s="70"/>
       <c r="AU15" s="62"/>
-      <c r="AV15" s="84"/>
+      <c r="AV15" s="70"/>
       <c r="AW15" s="62"/>
-      <c r="AX15" s="84"/>
-      <c r="AY15" s="67"/>
-      <c r="AZ15" s="84"/>
-      <c r="BA15" s="84"/>
-      <c r="BB15" s="117"/>
-      <c r="BC15" s="84"/>
+      <c r="AX15" s="70"/>
+      <c r="AY15" s="76"/>
+      <c r="AZ15" s="70"/>
+      <c r="BA15" s="70"/>
+      <c r="BB15" s="69"/>
+      <c r="BC15" s="70"/>
     </row>
-    <row r="16" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A16" s="75"/>
-      <c r="B16" s="75"/>
+    <row r="16" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="81"/>
+      <c r="B16" s="81"/>
       <c r="C16" s="20" t="s">
         <v>131</v>
       </c>
@@ -3854,35 +3858,35 @@
       <c r="L16" s="56" t="s">
         <v>123</v>
       </c>
-      <c r="M16" s="67" t="s">
+      <c r="M16" s="76" t="s">
         <v>203</v>
       </c>
-      <c r="N16" s="67"/>
-      <c r="O16" s="67"/>
+      <c r="N16" s="76"/>
+      <c r="O16" s="76"/>
       <c r="P16" s="24" t="s">
         <v>209</v>
       </c>
-      <c r="Q16" s="67"/>
-      <c r="R16" s="69"/>
-      <c r="S16" s="69"/>
-      <c r="T16" s="69"/>
-      <c r="U16" s="69"/>
-      <c r="V16" s="85"/>
-      <c r="W16" s="69"/>
-      <c r="X16" s="69"/>
-      <c r="Y16" s="69"/>
-      <c r="Z16" s="69"/>
-      <c r="AA16" s="67"/>
-      <c r="AB16" s="69"/>
-      <c r="AC16" s="67"/>
-      <c r="AD16" s="72"/>
-      <c r="AE16" s="67"/>
-      <c r="AF16" s="67"/>
-      <c r="AG16" s="67"/>
-      <c r="AH16" s="67"/>
-      <c r="AI16" s="67"/>
-      <c r="AJ16" s="67"/>
-      <c r="AK16" s="67"/>
+      <c r="Q16" s="76"/>
+      <c r="R16" s="84"/>
+      <c r="S16" s="84"/>
+      <c r="T16" s="84"/>
+      <c r="U16" s="84"/>
+      <c r="V16" s="95"/>
+      <c r="W16" s="84"/>
+      <c r="X16" s="84"/>
+      <c r="Y16" s="84"/>
+      <c r="Z16" s="84"/>
+      <c r="AA16" s="76"/>
+      <c r="AB16" s="84"/>
+      <c r="AC16" s="76"/>
+      <c r="AD16" s="80"/>
+      <c r="AE16" s="76"/>
+      <c r="AF16" s="76"/>
+      <c r="AG16" s="76"/>
+      <c r="AH16" s="76"/>
+      <c r="AI16" s="76"/>
+      <c r="AJ16" s="76"/>
+      <c r="AK16" s="76"/>
       <c r="AL16" s="24" t="s">
         <v>240</v>
       </c>
@@ -3894,7 +3898,7 @@
         <v>241</v>
       </c>
       <c r="AP16" s="24" t="s">
-        <v>246</v>
+        <v>316</v>
       </c>
       <c r="AQ16" s="62" t="s">
         <v>229</v>
@@ -3928,9 +3932,9 @@
         <v>309</v>
       </c>
     </row>
-    <row r="17" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A17" s="75"/>
-      <c r="B17" s="72" t="s">
+    <row r="17" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="81"/>
+      <c r="B17" s="80" t="s">
         <v>132</v>
       </c>
       <c r="C17" s="54" t="s">
@@ -3963,35 +3967,35 @@
       <c r="L17" s="56" t="s">
         <v>124</v>
       </c>
-      <c r="M17" s="67" t="s">
+      <c r="M17" s="76" t="s">
         <v>201</v>
       </c>
-      <c r="N17" s="67"/>
-      <c r="O17" s="67"/>
+      <c r="N17" s="76"/>
+      <c r="O17" s="76"/>
       <c r="P17" s="24" t="s">
         <v>210</v>
       </c>
-      <c r="Q17" s="67"/>
-      <c r="R17" s="69"/>
-      <c r="S17" s="69"/>
-      <c r="T17" s="69"/>
-      <c r="U17" s="69"/>
-      <c r="V17" s="69"/>
-      <c r="W17" s="69"/>
-      <c r="X17" s="69"/>
-      <c r="Y17" s="69"/>
-      <c r="Z17" s="69"/>
-      <c r="AA17" s="69"/>
-      <c r="AB17" s="69"/>
-      <c r="AC17" s="67"/>
-      <c r="AD17" s="67"/>
-      <c r="AE17" s="67"/>
-      <c r="AF17" s="67"/>
-      <c r="AG17" s="67"/>
-      <c r="AH17" s="67"/>
-      <c r="AI17" s="67"/>
-      <c r="AJ17" s="67"/>
-      <c r="AK17" s="67"/>
+      <c r="Q17" s="76"/>
+      <c r="R17" s="84"/>
+      <c r="S17" s="84"/>
+      <c r="T17" s="84"/>
+      <c r="U17" s="84"/>
+      <c r="V17" s="84"/>
+      <c r="W17" s="84"/>
+      <c r="X17" s="84"/>
+      <c r="Y17" s="84"/>
+      <c r="Z17" s="84"/>
+      <c r="AA17" s="84"/>
+      <c r="AB17" s="84"/>
+      <c r="AC17" s="76"/>
+      <c r="AD17" s="76"/>
+      <c r="AE17" s="76"/>
+      <c r="AF17" s="76"/>
+      <c r="AG17" s="76"/>
+      <c r="AH17" s="76"/>
+      <c r="AI17" s="76"/>
+      <c r="AJ17" s="76"/>
+      <c r="AK17" s="76"/>
       <c r="AL17" s="24" t="s">
         <v>242</v>
       </c>
@@ -4000,16 +4004,16 @@
       <c r="AO17" s="24" t="s">
         <v>243</v>
       </c>
-      <c r="AP17" s="84" t="s">
+      <c r="AP17" s="70" t="s">
         <v>249</v>
       </c>
-      <c r="AQ17" s="84" t="s">
+      <c r="AQ17" s="70" t="s">
         <v>228</v>
       </c>
-      <c r="AR17" s="84" t="s">
+      <c r="AR17" s="70" t="s">
         <v>255</v>
       </c>
-      <c r="AS17" s="84" t="s">
+      <c r="AS17" s="70" t="s">
         <v>263</v>
       </c>
       <c r="AT17" s="64"/>
@@ -4027,9 +4031,9 @@
       <c r="BB17" s="65"/>
       <c r="BC17" s="62"/>
     </row>
-    <row r="18" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A18" s="75"/>
-      <c r="B18" s="75"/>
+    <row r="18" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="81"/>
+      <c r="B18" s="81"/>
       <c r="C18" s="20" t="s">
         <v>134</v>
       </c>
@@ -4060,9 +4064,9 @@
       <c r="L18" s="56" t="s">
         <v>212</v>
       </c>
-      <c r="M18" s="67"/>
-      <c r="N18" s="67"/>
-      <c r="O18" s="67"/>
+      <c r="M18" s="76"/>
+      <c r="N18" s="76"/>
+      <c r="O18" s="76"/>
       <c r="P18" s="24" t="s">
         <v>213</v>
       </c>
@@ -4093,10 +4097,10 @@
       <c r="AM18" s="42"/>
       <c r="AN18" s="62"/>
       <c r="AO18" s="42"/>
-      <c r="AP18" s="84"/>
-      <c r="AQ18" s="84"/>
-      <c r="AR18" s="84"/>
-      <c r="AS18" s="84"/>
+      <c r="AP18" s="70"/>
+      <c r="AQ18" s="70"/>
+      <c r="AR18" s="70"/>
+      <c r="AS18" s="70"/>
       <c r="AT18" s="64"/>
       <c r="AU18" s="62"/>
       <c r="AV18" s="62"/>
@@ -4112,30 +4116,30 @@
       <c r="BB18" s="65"/>
       <c r="BC18" s="62"/>
     </row>
-    <row r="19" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A19" s="72" t="s">
+    <row r="19" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="80" t="s">
         <v>78</v>
       </c>
-      <c r="B19" s="72" t="s">
+      <c r="B19" s="80" t="s">
         <v>101</v>
       </c>
-      <c r="C19" s="74"/>
+      <c r="C19" s="92"/>
       <c r="D19" s="55" t="s">
         <v>148</v>
       </c>
       <c r="E19" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="F19" s="81"/>
-      <c r="G19" s="81"/>
-      <c r="H19" s="81"/>
-      <c r="I19" s="81"/>
-      <c r="J19" s="81"/>
+      <c r="F19" s="90"/>
+      <c r="G19" s="90"/>
+      <c r="H19" s="90"/>
+      <c r="I19" s="90"/>
+      <c r="J19" s="90"/>
       <c r="K19" s="42"/>
       <c r="L19" s="42"/>
-      <c r="M19" s="81"/>
-      <c r="N19" s="81"/>
-      <c r="O19" s="81"/>
+      <c r="M19" s="90"/>
+      <c r="N19" s="90"/>
+      <c r="O19" s="90"/>
       <c r="P19" s="42"/>
       <c r="Q19" s="42"/>
       <c r="R19" s="42"/>
@@ -4177,26 +4181,26 @@
       <c r="BB19" s="65"/>
       <c r="BC19" s="62"/>
     </row>
-    <row r="20" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A20" s="75"/>
-      <c r="B20" s="75"/>
-      <c r="C20" s="74"/>
+    <row r="20" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="81"/>
+      <c r="B20" s="81"/>
+      <c r="C20" s="92"/>
       <c r="D20" s="55" t="s">
         <v>149</v>
       </c>
       <c r="E20" s="20" t="s">
         <v>136</v>
       </c>
-      <c r="F20" s="81"/>
-      <c r="G20" s="81"/>
-      <c r="H20" s="81"/>
-      <c r="I20" s="81"/>
-      <c r="J20" s="81"/>
+      <c r="F20" s="90"/>
+      <c r="G20" s="90"/>
+      <c r="H20" s="90"/>
+      <c r="I20" s="90"/>
+      <c r="J20" s="90"/>
       <c r="K20" s="42"/>
       <c r="L20" s="42"/>
-      <c r="M20" s="81"/>
-      <c r="N20" s="81"/>
-      <c r="O20" s="81"/>
+      <c r="M20" s="90"/>
+      <c r="N20" s="90"/>
+      <c r="O20" s="90"/>
       <c r="P20" s="42"/>
       <c r="Q20" s="42"/>
       <c r="R20" s="42"/>
@@ -4238,26 +4242,26 @@
       <c r="BB20" s="65"/>
       <c r="BC20" s="62"/>
     </row>
-    <row r="21" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A21" s="75"/>
-      <c r="B21" s="75"/>
-      <c r="C21" s="74"/>
+    <row r="21" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="81"/>
+      <c r="B21" s="81"/>
+      <c r="C21" s="92"/>
       <c r="D21" s="24" t="s">
         <v>150</v>
       </c>
       <c r="E21" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="F21" s="81"/>
-      <c r="G21" s="81"/>
-      <c r="H21" s="81"/>
-      <c r="I21" s="81"/>
-      <c r="J21" s="81"/>
+      <c r="F21" s="90"/>
+      <c r="G21" s="90"/>
+      <c r="H21" s="90"/>
+      <c r="I21" s="90"/>
+      <c r="J21" s="90"/>
       <c r="K21" s="42"/>
       <c r="L21" s="42"/>
-      <c r="M21" s="81"/>
-      <c r="N21" s="81"/>
-      <c r="O21" s="81"/>
+      <c r="M21" s="90"/>
+      <c r="N21" s="90"/>
+      <c r="O21" s="90"/>
       <c r="P21" s="42"/>
       <c r="Q21" s="42"/>
       <c r="R21" s="42"/>
@@ -4299,26 +4303,26 @@
       <c r="BB21" s="65"/>
       <c r="BC21" s="62"/>
     </row>
-    <row r="22" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A22" s="75"/>
-      <c r="B22" s="75"/>
-      <c r="C22" s="74"/>
+    <row r="22" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="81"/>
+      <c r="B22" s="81"/>
+      <c r="C22" s="92"/>
       <c r="D22" s="24" t="s">
         <v>151</v>
       </c>
       <c r="E22" s="20" t="s">
         <v>138</v>
       </c>
-      <c r="F22" s="81"/>
-      <c r="G22" s="81"/>
-      <c r="H22" s="81"/>
-      <c r="I22" s="81"/>
-      <c r="J22" s="81"/>
+      <c r="F22" s="90"/>
+      <c r="G22" s="90"/>
+      <c r="H22" s="90"/>
+      <c r="I22" s="90"/>
+      <c r="J22" s="90"/>
       <c r="K22" s="42"/>
       <c r="L22" s="42"/>
-      <c r="M22" s="81"/>
-      <c r="N22" s="81"/>
-      <c r="O22" s="81"/>
+      <c r="M22" s="90"/>
+      <c r="N22" s="90"/>
+      <c r="O22" s="90"/>
       <c r="P22" s="42"/>
       <c r="Q22" s="42"/>
       <c r="R22" s="42"/>
@@ -4362,26 +4366,26 @@
       <c r="BB22" s="65"/>
       <c r="BC22" s="62"/>
     </row>
-    <row r="23" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A23" s="75"/>
-      <c r="B23" s="75"/>
-      <c r="C23" s="74"/>
+    <row r="23" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="81"/>
+      <c r="B23" s="81"/>
+      <c r="C23" s="92"/>
       <c r="D23" s="20" t="s">
         <v>152</v>
       </c>
       <c r="E23" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="F23" s="81"/>
-      <c r="G23" s="81"/>
-      <c r="H23" s="81"/>
-      <c r="I23" s="81"/>
-      <c r="J23" s="81"/>
+      <c r="F23" s="90"/>
+      <c r="G23" s="90"/>
+      <c r="H23" s="90"/>
+      <c r="I23" s="90"/>
+      <c r="J23" s="90"/>
       <c r="K23" s="42"/>
       <c r="L23" s="42"/>
-      <c r="M23" s="81"/>
-      <c r="N23" s="81"/>
-      <c r="O23" s="81"/>
+      <c r="M23" s="90"/>
+      <c r="N23" s="90"/>
+      <c r="O23" s="90"/>
       <c r="P23" s="42"/>
       <c r="Q23" s="42"/>
       <c r="R23" s="42"/>
@@ -4423,28 +4427,28 @@
       <c r="BB23" s="65"/>
       <c r="BC23" s="62"/>
     </row>
-    <row r="24" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A24" s="75"/>
-      <c r="B24" s="72" t="s">
+    <row r="24" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="81"/>
+      <c r="B24" s="80" t="s">
         <v>132</v>
       </c>
-      <c r="C24" s="74"/>
+      <c r="C24" s="92"/>
       <c r="D24" s="20" t="s">
         <v>153</v>
       </c>
       <c r="E24" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="F24" s="81"/>
-      <c r="G24" s="81"/>
-      <c r="H24" s="81"/>
-      <c r="I24" s="81"/>
-      <c r="J24" s="81"/>
+      <c r="F24" s="90"/>
+      <c r="G24" s="90"/>
+      <c r="H24" s="90"/>
+      <c r="I24" s="90"/>
+      <c r="J24" s="90"/>
       <c r="K24" s="42"/>
       <c r="L24" s="42"/>
-      <c r="M24" s="81"/>
-      <c r="N24" s="81"/>
-      <c r="O24" s="81"/>
+      <c r="M24" s="90"/>
+      <c r="N24" s="90"/>
+      <c r="O24" s="90"/>
       <c r="P24" s="42"/>
       <c r="Q24" s="42"/>
       <c r="R24" s="42"/>
@@ -4486,26 +4490,26 @@
       <c r="BB24" s="65"/>
       <c r="BC24" s="62"/>
     </row>
-    <row r="25" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A25" s="75"/>
-      <c r="B25" s="75"/>
-      <c r="C25" s="74"/>
+    <row r="25" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="81"/>
+      <c r="B25" s="81"/>
+      <c r="C25" s="92"/>
       <c r="D25" s="20" t="s">
         <v>154</v>
       </c>
       <c r="E25" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="F25" s="81"/>
-      <c r="G25" s="81"/>
-      <c r="H25" s="81"/>
-      <c r="I25" s="81"/>
-      <c r="J25" s="81"/>
+      <c r="F25" s="90"/>
+      <c r="G25" s="90"/>
+      <c r="H25" s="90"/>
+      <c r="I25" s="90"/>
+      <c r="J25" s="90"/>
       <c r="K25" s="42"/>
       <c r="L25" s="42"/>
-      <c r="M25" s="81"/>
-      <c r="N25" s="81"/>
-      <c r="O25" s="81"/>
+      <c r="M25" s="90"/>
+      <c r="N25" s="90"/>
+      <c r="O25" s="90"/>
       <c r="P25" s="42"/>
       <c r="Q25" s="42"/>
       <c r="R25" s="42"/>
@@ -4555,26 +4559,26 @@
       <c r="BB25" s="65"/>
       <c r="BC25" s="62"/>
     </row>
-    <row r="26" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A26" s="75"/>
-      <c r="B26" s="75"/>
-      <c r="C26" s="74"/>
+    <row r="26" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="81"/>
+      <c r="B26" s="81"/>
+      <c r="C26" s="92"/>
       <c r="D26" s="20" t="s">
         <v>155</v>
       </c>
       <c r="E26" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="F26" s="81"/>
-      <c r="G26" s="81"/>
-      <c r="H26" s="81"/>
-      <c r="I26" s="81"/>
-      <c r="J26" s="81"/>
+      <c r="F26" s="90"/>
+      <c r="G26" s="90"/>
+      <c r="H26" s="90"/>
+      <c r="I26" s="90"/>
+      <c r="J26" s="90"/>
       <c r="K26" s="42"/>
       <c r="L26" s="42"/>
-      <c r="M26" s="81"/>
-      <c r="N26" s="81"/>
-      <c r="O26" s="81"/>
+      <c r="M26" s="90"/>
+      <c r="N26" s="90"/>
+      <c r="O26" s="90"/>
       <c r="P26" s="42"/>
       <c r="Q26" s="42"/>
       <c r="R26" s="42"/>
@@ -4618,7 +4622,7 @@
       <c r="BB26" s="65"/>
       <c r="BC26" s="62"/>
     </row>
-    <row r="27" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="27" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="44"/>
       <c r="B27" s="43"/>
       <c r="C27" s="43"/>
@@ -4635,8 +4639,8 @@
       <c r="N27" s="46"/>
       <c r="O27" s="46"/>
       <c r="P27" s="45"/>
-      <c r="Q27" s="79"/>
-      <c r="R27" s="80"/>
+      <c r="Q27" s="88"/>
+      <c r="R27" s="89"/>
       <c r="S27" s="59"/>
       <c r="T27" s="59"/>
       <c r="U27" s="59"/>
@@ -4645,8 +4649,8 @@
       <c r="X27" s="59"/>
       <c r="Y27" s="59"/>
       <c r="Z27" s="59"/>
-      <c r="AA27" s="68"/>
-      <c r="AB27" s="68"/>
+      <c r="AA27" s="93"/>
+      <c r="AB27" s="93"/>
       <c r="AC27" s="58"/>
       <c r="AD27" s="58"/>
       <c r="AE27" s="58"/>
@@ -4658,7 +4662,7 @@
       <c r="AK27" s="61"/>
       <c r="AL27" s="57"/>
     </row>
-    <row r="28" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="28" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="44"/>
       <c r="B28" s="43"/>
       <c r="C28" s="43"/>
@@ -4675,8 +4679,8 @@
       <c r="N28" s="46"/>
       <c r="O28" s="46"/>
       <c r="P28" s="45"/>
-      <c r="Q28" s="77"/>
-      <c r="R28" s="78"/>
+      <c r="Q28" s="86"/>
+      <c r="R28" s="87"/>
       <c r="S28" s="28"/>
       <c r="T28" s="28"/>
       <c r="U28" s="28"/>
@@ -4685,8 +4689,8 @@
       <c r="X28" s="28"/>
       <c r="Y28" s="28"/>
       <c r="Z28" s="28"/>
-      <c r="AA28" s="67"/>
-      <c r="AB28" s="67"/>
+      <c r="AA28" s="76"/>
+      <c r="AB28" s="76"/>
       <c r="AC28" s="24"/>
       <c r="AD28" s="24"/>
       <c r="AE28" s="24"/>
@@ -4698,7 +4702,7 @@
       <c r="AK28" s="36"/>
       <c r="AL28" s="57"/>
     </row>
-    <row r="29" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="29" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="44"/>
       <c r="B29" s="43"/>
       <c r="C29" s="43"/>
@@ -4715,8 +4719,8 @@
       <c r="N29" s="46"/>
       <c r="O29" s="46"/>
       <c r="P29" s="45"/>
-      <c r="Q29" s="77"/>
-      <c r="R29" s="78"/>
+      <c r="Q29" s="86"/>
+      <c r="R29" s="87"/>
       <c r="S29" s="28"/>
       <c r="T29" s="28"/>
       <c r="U29" s="28"/>
@@ -4725,8 +4729,8 @@
       <c r="X29" s="28"/>
       <c r="Y29" s="28"/>
       <c r="Z29" s="28"/>
-      <c r="AA29" s="67"/>
-      <c r="AB29" s="67"/>
+      <c r="AA29" s="76"/>
+      <c r="AB29" s="76"/>
       <c r="AC29" s="24"/>
       <c r="AD29" s="24"/>
       <c r="AE29" s="24"/>
@@ -4738,7 +4742,7 @@
       <c r="AK29" s="36"/>
       <c r="AL29" s="57"/>
     </row>
-    <row r="30" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="30" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="44"/>
       <c r="B30" s="43"/>
       <c r="C30" s="43"/>
@@ -4755,8 +4759,8 @@
       <c r="N30" s="46"/>
       <c r="O30" s="46"/>
       <c r="P30" s="45"/>
-      <c r="Q30" s="77"/>
-      <c r="R30" s="78"/>
+      <c r="Q30" s="86"/>
+      <c r="R30" s="87"/>
       <c r="S30" s="28"/>
       <c r="T30" s="28"/>
       <c r="U30" s="28"/>
@@ -4765,8 +4769,8 @@
       <c r="X30" s="28"/>
       <c r="Y30" s="28"/>
       <c r="Z30" s="28"/>
-      <c r="AA30" s="67"/>
-      <c r="AB30" s="67"/>
+      <c r="AA30" s="76"/>
+      <c r="AB30" s="76"/>
       <c r="AC30" s="24"/>
       <c r="AD30" s="24"/>
       <c r="AE30" s="24"/>
@@ -4778,7 +4782,7 @@
       <c r="AK30" s="36"/>
       <c r="AL30" s="57"/>
     </row>
-    <row r="31" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="31" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D31" s="46"/>
       <c r="E31" s="46"/>
       <c r="F31" s="46"/>
@@ -4792,8 +4796,8 @@
       <c r="N31" s="46"/>
       <c r="O31" s="46"/>
       <c r="P31" s="45"/>
-      <c r="Q31" s="77"/>
-      <c r="R31" s="78"/>
+      <c r="Q31" s="86"/>
+      <c r="R31" s="87"/>
       <c r="S31" s="28"/>
       <c r="T31" s="28"/>
       <c r="U31" s="28"/>
@@ -4802,8 +4806,8 @@
       <c r="X31" s="28"/>
       <c r="Y31" s="28"/>
       <c r="Z31" s="28"/>
-      <c r="AA31" s="67"/>
-      <c r="AB31" s="67"/>
+      <c r="AA31" s="76"/>
+      <c r="AB31" s="76"/>
       <c r="AC31" s="24"/>
       <c r="AD31" s="24"/>
       <c r="AE31" s="24"/>
@@ -4815,14 +4819,14 @@
       <c r="AK31" s="36"/>
       <c r="AL31" s="57"/>
     </row>
-    <row r="32" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="32" spans="1:55" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D32" s="43"/>
       <c r="E32" s="43"/>
       <c r="F32" s="43"/>
       <c r="G32" s="43"/>
       <c r="H32" s="43"/>
       <c r="I32" s="46"/>
-      <c r="J32" s="73"/>
+      <c r="J32" s="91"/>
       <c r="K32" s="45"/>
       <c r="L32" s="45"/>
       <c r="M32" s="45"/>
@@ -4852,14 +4856,14 @@
       <c r="AK32" s="36"/>
       <c r="AL32" s="57"/>
     </row>
-    <row r="33" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="33" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D33" s="43"/>
       <c r="E33" s="43"/>
       <c r="F33" s="43"/>
       <c r="G33" s="43"/>
       <c r="H33" s="43"/>
       <c r="I33" s="46"/>
-      <c r="J33" s="73"/>
+      <c r="J33" s="91"/>
       <c r="K33" s="45"/>
       <c r="L33" s="45"/>
       <c r="M33" s="45"/>
@@ -4889,7 +4893,7 @@
       <c r="AK33" s="36"/>
       <c r="AL33" s="57"/>
     </row>
-    <row r="34" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="34" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D34" s="46"/>
       <c r="E34" s="46"/>
       <c r="F34" s="46"/>
@@ -4926,7 +4930,7 @@
       <c r="AK34" s="36"/>
       <c r="AL34" s="57"/>
     </row>
-    <row r="35" spans="1:38" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
+    <row r="35" spans="1:38" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="D35" s="47"/>
       <c r="E35" s="48"/>
       <c r="F35" s="46"/>
@@ -4963,14 +4967,14 @@
       <c r="AK35" s="37"/>
       <c r="AL35" s="57"/>
     </row>
-    <row r="36" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="36" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D36" s="49"/>
       <c r="E36" s="50"/>
       <c r="F36" s="45"/>
       <c r="G36" s="45"/>
       <c r="H36" s="45"/>
       <c r="I36" s="45"/>
-      <c r="J36" s="76"/>
+      <c r="J36" s="85"/>
       <c r="K36" s="45"/>
       <c r="L36" s="45"/>
       <c r="M36" s="45"/>
@@ -5000,14 +5004,14 @@
       <c r="AK36" s="35"/>
       <c r="AL36" s="35"/>
     </row>
-    <row r="37" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="37" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D37" s="49"/>
       <c r="E37" s="50"/>
       <c r="F37" s="45"/>
       <c r="G37" s="45"/>
       <c r="H37" s="45"/>
       <c r="I37" s="45"/>
-      <c r="J37" s="76"/>
+      <c r="J37" s="85"/>
       <c r="K37" s="45"/>
       <c r="L37" s="45"/>
       <c r="M37" s="45"/>
@@ -5037,7 +5041,7 @@
       <c r="AK37" s="35"/>
       <c r="AL37" s="35"/>
     </row>
-    <row r="38" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="38" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D38" s="44"/>
       <c r="E38" s="44"/>
       <c r="F38" s="44"/>
@@ -5074,7 +5078,7 @@
       <c r="AK38" s="35"/>
       <c r="AL38" s="35"/>
     </row>
-    <row r="39" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="39" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="44"/>
       <c r="C39" s="44"/>
       <c r="D39" s="44"/>
@@ -5113,7 +5117,7 @@
       <c r="AK39" s="35"/>
       <c r="AL39" s="35"/>
     </row>
-    <row r="40" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="40" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="44"/>
       <c r="C40" s="44"/>
       <c r="D40" s="44"/>
@@ -5152,7 +5156,7 @@
       <c r="AK40" s="35"/>
       <c r="AL40" s="35"/>
     </row>
-    <row r="41" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="41" spans="1:38" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A41" s="44"/>
       <c r="B41" s="43"/>
       <c r="C41" s="44"/>
@@ -5192,7 +5196,7 @@
       <c r="AK41" s="35"/>
       <c r="AL41" s="35"/>
     </row>
-    <row r="42" spans="1:38" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
+    <row r="42" spans="1:38" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A42" s="44"/>
       <c r="C42" s="44"/>
       <c r="D42" s="44"/>
@@ -5233,15 +5237,84 @@
     </row>
   </sheetData>
   <mergeCells count="118">
-    <mergeCell ref="BB8:BB12"/>
-    <mergeCell ref="BB14:BB15"/>
-    <mergeCell ref="BA14:BA15"/>
-    <mergeCell ref="BA7:BA12"/>
-    <mergeCell ref="BC7:BC12"/>
-    <mergeCell ref="BC14:BC15"/>
-    <mergeCell ref="AP5:BC5"/>
-    <mergeCell ref="AP4:BC4"/>
-    <mergeCell ref="K3:BC3"/>
+    <mergeCell ref="A19:A26"/>
+    <mergeCell ref="B19:B23"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="AA31:AB31"/>
+    <mergeCell ref="AA30:AB30"/>
+    <mergeCell ref="AA27:AB27"/>
+    <mergeCell ref="AA28:AB28"/>
+    <mergeCell ref="Z16:Z17"/>
+    <mergeCell ref="U16:U17"/>
+    <mergeCell ref="AA29:AB29"/>
+    <mergeCell ref="V16:V17"/>
+    <mergeCell ref="AA16:AA17"/>
+    <mergeCell ref="AB16:AB17"/>
+    <mergeCell ref="M26:O26"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="M7:O11"/>
+    <mergeCell ref="M12:O12"/>
+    <mergeCell ref="M13:O13"/>
+    <mergeCell ref="M17:O18"/>
+    <mergeCell ref="J32:J33"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="C19:C26"/>
+    <mergeCell ref="C11:J12"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="F3:J4"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J36:J37"/>
+    <mergeCell ref="Q31:R31"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="Q28:R28"/>
+    <mergeCell ref="Q29:R29"/>
+    <mergeCell ref="Q30:R30"/>
+    <mergeCell ref="M16:O16"/>
+    <mergeCell ref="M6:O6"/>
+    <mergeCell ref="Q16:Q17"/>
+    <mergeCell ref="R16:R17"/>
+    <mergeCell ref="F19:J26"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="M20:O20"/>
+    <mergeCell ref="M21:O21"/>
+    <mergeCell ref="M22:O22"/>
+    <mergeCell ref="M23:O23"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="M25:O25"/>
+    <mergeCell ref="B7:B16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="AN7:AN10"/>
+    <mergeCell ref="AN11:AN12"/>
+    <mergeCell ref="AE16:AE17"/>
+    <mergeCell ref="AF16:AF17"/>
+    <mergeCell ref="S16:S17"/>
+    <mergeCell ref="T16:T17"/>
+    <mergeCell ref="W16:W17"/>
+    <mergeCell ref="X16:X17"/>
+    <mergeCell ref="Y16:Y17"/>
+    <mergeCell ref="AD16:AD17"/>
+    <mergeCell ref="AC16:AC17"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="AP17:AP18"/>
+    <mergeCell ref="AP14:AP15"/>
+    <mergeCell ref="AQ14:AQ15"/>
+    <mergeCell ref="AQ17:AQ18"/>
+    <mergeCell ref="AI16:AI17"/>
+    <mergeCell ref="AG16:AG17"/>
+    <mergeCell ref="AH16:AH17"/>
+    <mergeCell ref="AJ16:AJ17"/>
+    <mergeCell ref="AK16:AK17"/>
     <mergeCell ref="A1:BC2"/>
     <mergeCell ref="AY8:AY11"/>
     <mergeCell ref="AY14:AY15"/>
@@ -5266,91 +5339,22 @@
     <mergeCell ref="AS17:AS18"/>
     <mergeCell ref="AR14:AR15"/>
     <mergeCell ref="AQ7:AQ11"/>
+    <mergeCell ref="BB8:BB12"/>
+    <mergeCell ref="BB14:BB15"/>
+    <mergeCell ref="BA14:BA15"/>
+    <mergeCell ref="BA7:BA12"/>
+    <mergeCell ref="BC7:BC12"/>
+    <mergeCell ref="BC14:BC15"/>
+    <mergeCell ref="AP5:BC5"/>
+    <mergeCell ref="AP4:BC4"/>
+    <mergeCell ref="K3:BC3"/>
     <mergeCell ref="AO7:AO11"/>
     <mergeCell ref="AL9:AL12"/>
     <mergeCell ref="AV8:AV12"/>
     <mergeCell ref="AV14:AV15"/>
     <mergeCell ref="AW8:AW12"/>
-    <mergeCell ref="AP17:AP18"/>
-    <mergeCell ref="AP14:AP15"/>
-    <mergeCell ref="AQ14:AQ15"/>
-    <mergeCell ref="AQ17:AQ18"/>
-    <mergeCell ref="AI16:AI17"/>
-    <mergeCell ref="AG16:AG17"/>
-    <mergeCell ref="AH16:AH17"/>
-    <mergeCell ref="AJ16:AJ17"/>
-    <mergeCell ref="AK16:AK17"/>
     <mergeCell ref="M4:AO4"/>
     <mergeCell ref="M5:AO5"/>
-    <mergeCell ref="B7:B16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="F5:J5"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="AN7:AN10"/>
-    <mergeCell ref="AN11:AN12"/>
-    <mergeCell ref="AE16:AE17"/>
-    <mergeCell ref="AF16:AF17"/>
-    <mergeCell ref="S16:S17"/>
-    <mergeCell ref="T16:T17"/>
-    <mergeCell ref="W16:W17"/>
-    <mergeCell ref="X16:X17"/>
-    <mergeCell ref="Y16:Y17"/>
-    <mergeCell ref="AD16:AD17"/>
-    <mergeCell ref="AC16:AC17"/>
-    <mergeCell ref="F3:J4"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J36:J37"/>
-    <mergeCell ref="Q31:R31"/>
-    <mergeCell ref="Q27:R27"/>
-    <mergeCell ref="Q28:R28"/>
-    <mergeCell ref="Q29:R29"/>
-    <mergeCell ref="Q30:R30"/>
-    <mergeCell ref="M16:O16"/>
-    <mergeCell ref="M6:O6"/>
-    <mergeCell ref="Q16:Q17"/>
-    <mergeCell ref="R16:R17"/>
-    <mergeCell ref="F19:J26"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="M20:O20"/>
-    <mergeCell ref="M21:O21"/>
-    <mergeCell ref="M22:O22"/>
-    <mergeCell ref="M23:O23"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="M25:O25"/>
-    <mergeCell ref="M26:O26"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="M7:O11"/>
-    <mergeCell ref="M12:O12"/>
-    <mergeCell ref="M13:O13"/>
-    <mergeCell ref="M17:O18"/>
-    <mergeCell ref="J32:J33"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="C19:C26"/>
-    <mergeCell ref="A19:A26"/>
-    <mergeCell ref="B19:B23"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="AA31:AB31"/>
-    <mergeCell ref="AA30:AB30"/>
-    <mergeCell ref="AA27:AB27"/>
-    <mergeCell ref="AA28:AB28"/>
-    <mergeCell ref="Z16:Z17"/>
-    <mergeCell ref="U16:U17"/>
-    <mergeCell ref="AA29:AB29"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="C11:J12"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="V16:V17"/>
-    <mergeCell ref="AA16:AA17"/>
-    <mergeCell ref="AB16:AB17"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5364,109 +5368,109 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P17"/>
-  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.375" customWidth="1"/>
-    <col min="2" max="2" width="15.875" customWidth="1"/>
-    <col min="3" max="3" width="6.375" customWidth="1"/>
-    <col min="4" max="4" width="26.875" customWidth="1"/>
-    <col min="5" max="5" width="7.125" customWidth="1"/>
-    <col min="6" max="6" width="22.625" customWidth="1"/>
-    <col min="7" max="7" width="9.375" customWidth="1"/>
-    <col min="8" max="8" width="21.6875" customWidth="1"/>
+    <col min="1" max="1" width="11.3984375" customWidth="1"/>
+    <col min="2" max="2" width="15.8984375" customWidth="1"/>
+    <col min="3" max="3" width="6.3984375" customWidth="1"/>
+    <col min="4" max="4" width="26.8984375" customWidth="1"/>
+    <col min="5" max="5" width="7.09765625" customWidth="1"/>
+    <col min="6" max="6" width="22.59765625" customWidth="1"/>
+    <col min="7" max="7" width="9.3984375" customWidth="1"/>
+    <col min="8" max="8" width="21.69921875" customWidth="1"/>
     <col min="9" max="9" width="6" customWidth="1"/>
-    <col min="10" max="10" width="16.375" customWidth="1"/>
+    <col min="10" max="10" width="16.3984375" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="5.6875" customWidth="1"/>
-    <col min="13" max="13" width="13.875" customWidth="1"/>
-    <col min="14" max="14" width="11.1875" customWidth="1"/>
-    <col min="15" max="16" width="12.875" customWidth="1"/>
+    <col min="12" max="12" width="5.69921875" customWidth="1"/>
+    <col min="13" max="13" width="13.8984375" customWidth="1"/>
+    <col min="14" max="14" width="11.19921875" customWidth="1"/>
+    <col min="15" max="16" width="12.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="106" t="s">
+    <row r="1" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="117" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="107"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="107"/>
-      <c r="J1" s="107"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="107"/>
-      <c r="M1" s="102" t="s">
+      <c r="B1" s="118"/>
+      <c r="C1" s="118"/>
+      <c r="D1" s="118"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="118"/>
+      <c r="G1" s="118"/>
+      <c r="H1" s="118"/>
+      <c r="I1" s="118"/>
+      <c r="J1" s="118"/>
+      <c r="K1" s="118"/>
+      <c r="L1" s="118"/>
+      <c r="M1" s="113" t="s">
         <v>49</v>
       </c>
-      <c r="N1" s="102"/>
-      <c r="O1" s="102" t="s">
+      <c r="N1" s="113"/>
+      <c r="O1" s="113" t="s">
         <v>51</v>
       </c>
-      <c r="P1" s="103"/>
+      <c r="P1" s="114"/>
     </row>
-    <row r="2" spans="1:16" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A2" s="108"/>
-      <c r="B2" s="109"/>
-      <c r="C2" s="109"/>
-      <c r="D2" s="109"/>
-      <c r="E2" s="109"/>
-      <c r="F2" s="109"/>
-      <c r="G2" s="109"/>
-      <c r="H2" s="109"/>
-      <c r="I2" s="109"/>
-      <c r="J2" s="109"/>
-      <c r="K2" s="109"/>
-      <c r="L2" s="109"/>
-      <c r="M2" s="104" t="s">
+    <row r="2" spans="1:16" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="119"/>
+      <c r="B2" s="120"/>
+      <c r="C2" s="120"/>
+      <c r="D2" s="120"/>
+      <c r="E2" s="120"/>
+      <c r="F2" s="120"/>
+      <c r="G2" s="120"/>
+      <c r="H2" s="120"/>
+      <c r="I2" s="120"/>
+      <c r="J2" s="120"/>
+      <c r="K2" s="120"/>
+      <c r="L2" s="120"/>
+      <c r="M2" s="115" t="s">
         <v>50</v>
       </c>
-      <c r="N2" s="104"/>
-      <c r="O2" s="104"/>
-      <c r="P2" s="105"/>
+      <c r="N2" s="115"/>
+      <c r="O2" s="115"/>
+      <c r="P2" s="116"/>
     </row>
-    <row r="3" spans="1:16" ht="17.25" thickBot="1" x14ac:dyDescent="0.65"/>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.6">
-      <c r="A4" s="110" t="s">
+    <row r="3" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.45"/>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A4" s="121" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="111"/>
-      <c r="C4" s="111"/>
-      <c r="D4" s="112"/>
-      <c r="E4" s="113" t="s">
+      <c r="B4" s="122"/>
+      <c r="C4" s="122"/>
+      <c r="D4" s="123"/>
+      <c r="E4" s="124" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="112"/>
-      <c r="G4" s="113" t="s">
+      <c r="F4" s="123"/>
+      <c r="G4" s="124" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="112"/>
-      <c r="I4" s="113" t="s">
+      <c r="H4" s="123"/>
+      <c r="I4" s="124" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="112"/>
-      <c r="K4" s="113" t="s">
+      <c r="J4" s="123"/>
+      <c r="K4" s="124" t="s">
         <v>26</v>
       </c>
-      <c r="L4" s="112"/>
+      <c r="L4" s="123"/>
       <c r="M4" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="113" t="s">
+      <c r="N4" s="124" t="s">
         <v>28</v>
       </c>
-      <c r="O4" s="112"/>
-      <c r="P4" s="93" t="s">
+      <c r="O4" s="123"/>
+      <c r="P4" s="104" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A5" s="95" t="s">
+    <row r="5" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="106" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="96"/>
+      <c r="B5" s="107"/>
       <c r="C5" s="15" t="s">
         <v>0</v>
       </c>
@@ -5506,10 +5510,10 @@
       <c r="O5" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="P5" s="94"/>
+      <c r="P5" s="105"/>
     </row>
-    <row r="6" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="97" t="s">
+    <row r="6" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="108" t="s">
         <v>36</v>
       </c>
       <c r="B6" s="11" t="s">
@@ -5538,9 +5542,9 @@
       <c r="O6" s="5"/>
       <c r="P6" s="6"/>
     </row>
-    <row r="7" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="97"/>
-      <c r="B7" s="114" t="s">
+    <row r="7" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="108"/>
+      <c r="B7" s="101" t="s">
         <v>53</v>
       </c>
       <c r="C7" s="5" t="s">
@@ -5549,47 +5553,47 @@
       <c r="D7" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="116"/>
-      <c r="F7" s="116"/>
-      <c r="G7" s="118" t="s">
+      <c r="E7" s="98"/>
+      <c r="F7" s="98"/>
+      <c r="G7" s="103" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="114" t="s">
+      <c r="H7" s="101" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="116"/>
-      <c r="J7" s="116"/>
-      <c r="K7" s="116"/>
-      <c r="L7" s="116"/>
-      <c r="M7" s="116"/>
-      <c r="N7" s="116"/>
-      <c r="O7" s="116"/>
-      <c r="P7" s="119"/>
+      <c r="I7" s="98"/>
+      <c r="J7" s="98"/>
+      <c r="K7" s="98"/>
+      <c r="L7" s="98"/>
+      <c r="M7" s="98"/>
+      <c r="N7" s="98"/>
+      <c r="O7" s="98"/>
+      <c r="P7" s="96"/>
     </row>
-    <row r="8" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="98"/>
-      <c r="B8" s="115"/>
+    <row r="8" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="109"/>
+      <c r="B8" s="102"/>
       <c r="C8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="117"/>
-      <c r="F8" s="117"/>
-      <c r="G8" s="118"/>
-      <c r="H8" s="115"/>
-      <c r="I8" s="117"/>
-      <c r="J8" s="117"/>
-      <c r="K8" s="117"/>
-      <c r="L8" s="117"/>
-      <c r="M8" s="117"/>
-      <c r="N8" s="117"/>
-      <c r="O8" s="117"/>
-      <c r="P8" s="120"/>
+      <c r="E8" s="69"/>
+      <c r="F8" s="69"/>
+      <c r="G8" s="103"/>
+      <c r="H8" s="102"/>
+      <c r="I8" s="69"/>
+      <c r="J8" s="69"/>
+      <c r="K8" s="69"/>
+      <c r="L8" s="69"/>
+      <c r="M8" s="69"/>
+      <c r="N8" s="69"/>
+      <c r="O8" s="69"/>
+      <c r="P8" s="97"/>
     </row>
-    <row r="9" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="98"/>
+    <row r="9" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="109"/>
       <c r="B9" s="16" t="s">
         <v>54</v>
       </c>
@@ -5616,9 +5620,9 @@
       <c r="O9" s="1"/>
       <c r="P9" s="2"/>
     </row>
-    <row r="10" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="98"/>
-      <c r="B10" s="114" t="s">
+    <row r="10" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="109"/>
+      <c r="B10" s="101" t="s">
         <v>56</v>
       </c>
       <c r="C10" s="9" t="s">
@@ -5627,47 +5631,47 @@
       <c r="D10" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="116"/>
-      <c r="F10" s="116"/>
-      <c r="G10" s="121" t="s">
+      <c r="E10" s="98"/>
+      <c r="F10" s="98"/>
+      <c r="G10" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="114" t="s">
+      <c r="H10" s="101" t="s">
         <v>41</v>
       </c>
-      <c r="I10" s="116"/>
-      <c r="J10" s="116"/>
-      <c r="K10" s="116"/>
-      <c r="L10" s="116"/>
-      <c r="M10" s="116"/>
-      <c r="N10" s="116"/>
-      <c r="O10" s="116"/>
-      <c r="P10" s="119"/>
+      <c r="I10" s="98"/>
+      <c r="J10" s="98"/>
+      <c r="K10" s="98"/>
+      <c r="L10" s="98"/>
+      <c r="M10" s="98"/>
+      <c r="N10" s="98"/>
+      <c r="O10" s="98"/>
+      <c r="P10" s="96"/>
     </row>
-    <row r="11" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="98"/>
-      <c r="B11" s="115"/>
+    <row r="11" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="109"/>
+      <c r="B11" s="102"/>
       <c r="C11" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="117"/>
-      <c r="F11" s="117"/>
-      <c r="G11" s="122"/>
-      <c r="H11" s="115"/>
-      <c r="I11" s="117"/>
-      <c r="J11" s="117"/>
-      <c r="K11" s="117"/>
-      <c r="L11" s="117"/>
-      <c r="M11" s="117"/>
-      <c r="N11" s="117"/>
-      <c r="O11" s="117"/>
-      <c r="P11" s="120"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="100"/>
+      <c r="H11" s="102"/>
+      <c r="I11" s="69"/>
+      <c r="J11" s="69"/>
+      <c r="K11" s="69"/>
+      <c r="L11" s="69"/>
+      <c r="M11" s="69"/>
+      <c r="N11" s="69"/>
+      <c r="O11" s="69"/>
+      <c r="P11" s="97"/>
     </row>
-    <row r="12" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A12" s="98"/>
+    <row r="12" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="109"/>
       <c r="B12" s="12" t="s">
         <v>55</v>
       </c>
@@ -5694,8 +5698,8 @@
       <c r="O12" s="1"/>
       <c r="P12" s="2"/>
     </row>
-    <row r="13" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A13" s="99"/>
+    <row r="13" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="110"/>
       <c r="B13" s="12" t="s">
         <v>57</v>
       </c>
@@ -5722,8 +5726,8 @@
       <c r="O13" s="1"/>
       <c r="P13" s="2"/>
     </row>
-    <row r="14" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A14" s="100" t="s">
+    <row r="14" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="111" t="s">
         <v>37</v>
       </c>
       <c r="B14" s="12" t="s">
@@ -5752,8 +5756,8 @@
       <c r="O14" s="1"/>
       <c r="P14" s="2"/>
     </row>
-    <row r="15" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A15" s="98"/>
+    <row r="15" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="109"/>
       <c r="B15" s="12" t="s">
         <v>58</v>
       </c>
@@ -5780,8 +5784,8 @@
       <c r="O15" s="1"/>
       <c r="P15" s="2"/>
     </row>
-    <row r="16" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A16" s="98"/>
+    <row r="16" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="109"/>
       <c r="B16" s="12" t="s">
         <v>60</v>
       </c>
@@ -5808,8 +5812,8 @@
       <c r="O16" s="1"/>
       <c r="P16" s="2"/>
     </row>
-    <row r="17" spans="1:16" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A17" s="101"/>
+    <row r="17" spans="1:16" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="112"/>
       <c r="B17" s="13" t="s">
         <v>61</v>
       </c>
@@ -5838,6 +5842,31 @@
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="P4:P5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A6:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="J7:J8"/>
     <mergeCell ref="P7:P8"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="F7:F8"/>
@@ -5854,31 +5883,6 @@
     <mergeCell ref="N10:N11"/>
     <mergeCell ref="O10:O11"/>
     <mergeCell ref="K7:K8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="O7:O8"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="P4:P5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="O1:P1"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="A1:L2"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="B7:B8"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>